<commit_message>
feat: make 2027 the home page with checklist and new design
- Home page (/) is now the 2027 trip; the finished 2026 trip moves to a
  collapsed "已结束的旅行" section and keeps its pages at /itinerary etc.
- New pre-trip checklist (/nz2027/checklist): 28 items with stable ids that
  can be ticked off and sync between phones via a new nz2027_checklist table
  and /api/nz2027/checklist (added to the unapplied 2027 migration).
- Redesigned 2027 schedule and ledger: road-sign chips, day list on a road
  line, today/next-day hero, overnight route, stays and travel tips.
- All 2027 copy rewritten from the travellers' side.
- Per-day theme pictures picked up from public/nz2027/dNN.*, with prompts in
  docs/nz2027-day-image-prompts.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -541,7 +541,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>已有7笔住宿订单共13晚（含悉尼2/1补订），另有Milford和Hobbiton两项活动；四段机票均未购买，Auckland 2/14–16两晚待订。所有日期时间均为当地时间。</t>
+          <t>所有日期和时间都是当地时间。</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>导航07主线</t>
+          <t>导航07</t>
         </is>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
         <is>
           <t>住宿｜Twizel Holiday Park，第三晚。
 新月｜按月相推算，2027/2/6前后是新月，2/6、2/7晚上都几乎没有月光，是一年里很好的观星窗口；Mt Cook与湖区日互换也不影响观星。
-观星待订｜可选Silver River的Twizel产品，约75分钟；使用该产品指定集合点。若改选Tekapo Mount John，要另外增加夜间往返驾驶。主案保留Twizel观星。长周末场次紧，尽早预约。</t>
+观星待订｜可选Silver River的Twizel产品，约75分钟；使用该产品指定集合点。改去Tekapo Mount John的话，晚上要多开一趟来回，所以首选在Twizel看。长周末场次紧，尽早预约。</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
         <is>
           <t>住宿｜Private Ensuite in the Heart of Te Anau，3 Thomson Place；15:00后入住。
 驾驶安排｜纯驾驶约3.5–4.5小时，加Arrowtown午餐和停靠留5–6小时；抵达时间随休息调整。
-路线建议｜主线已改为Crown Range + Arrowtown（行程文件原为经Cromwell）。起雾、大风、下雨或不想开山路时改回Cromwell，导航见下方备选链接，从Frankton起两条路完全相同。</t>
+坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
         <is>
           <t>住宿｜Fernhill山景单间，第二晚。
 沙蝇｜Glenorchy码头和Lagoon湿地沙蝇多，下车前喷驱蚊液。
-天气备选｜小雨时缩短Lagoon段；大雨、路况或能见度不适合时留Queenstown城市活动。主行程止于Glenorchy，不延伸碎石支路。</t>
+天气备选｜小雨时缩短Lagoon段；大雨、路况或能见度不适合时留Queenstown城市活动。只到Glenorchy，不走碎石支路。</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       <c r="W17" t="inlineStr">
         <is>
           <t>住宿｜飞机；通常无需增加2/16酒店住宿。
-若最终买22:00航班｜可按17:00取包、17:30前离开市区、19:00前到机场规划；这是示例，出票后整体平移。</t>
+去机场｜以22:00起飞为例：17:00取包、17:30前离开市区、19:00前到机场；按实际航班往前推。</t>
         </is>
       </c>
     </row>
@@ -6074,7 +6074,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>入境、取车并熟悉车辆。南岛用车按Christchurch取、Queenstown还规划，车行和网点待落实。</t>
+          <t>入境、取车并熟悉车辆。南岛租车在基督城取、皇后镇还，租车公司和取车点还没订。</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -6388,7 +6388,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>原行程为08:00左右，因Waitangi长周末提前。</t>
+          <t>长周末停车场上午很早就满。</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>先满足最终航司的到场要求；规划可留起飞前约90分钟到国内航站楼，再向前加约45–60分钟还车/摆渡及路程。车行若要求更早，按其说明调整。今天不插入专门绕路的游览（Arrowtown已在2/10顺路去过）。</t>
+          <t>先满足最终航司的到场要求；大约起飞前90分钟到国内航站楼，再向前加约45–60分钟还车/摆渡及路程。车行若要求更早，按其说明调整。今天不插入专门绕路的游览（Arrowtown已在2/10顺路去过）。</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -10059,7 +10059,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>约2.5–3小时规划窗口</t>
+          <t>约2.5–3小时</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -10306,7 +10306,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>入退房时间按原凭证；122 Mackenzie Drive</t>
+          <t>入退房时间看订单确认；122 Mackenzie Drive</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -10521,568 +10521,947 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>todo_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>sort_order</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>kind</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>due_date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>due_label</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>detail</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>visa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>prep</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>最先办</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>澳大利亚、新西兰签证</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>如持中国护照，两国都需要单独申请旅游签证；办好后再出机票。具体材料和时长以两国官方为准。</t>
+          <t>办澳大利亚、新西兰签证</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>持中国护照两国都要单独办旅游签证，办好再出机票。材料和时长以两国官方为准。</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>licence</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>prep</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>出发前</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>驾照英文翻译件</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>新西兰开车需随身带中国驾照和认可的英文翻译件（或国际驾照认证件），两人都要准备；租车取车时会查，要求以租车公司为准。</t>
+          <t>两人的驾照英文翻译件</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>新西兰开车要带中国驾照和认可的英文翻译件（或国际驾照认证件），取车时会查。</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>flight-syd</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>30</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>尽早</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>四段机票</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2/1抵SYD；2/4当日SYD→CHC（优先上午起飞，新西兰快2小时）；2/14下午抵AKL；2/16晚AKL离境、2/17早晨抵国内。出票后补准确航班号及机场到场时间。</t>
+          <t>机票：国内 → 悉尼</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2/1 当天到悉尼。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>30</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>flight-chc</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>40</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>尽早</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Auckland两晚</t>
-        </is>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2/14入住、2/16退房；同一家连住，确认寄存及取包时段。最好选附近有支持晚间还车租车网点的位置，方便2/15。</t>
+          <t>机票：悉尼 → 基督城</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2/4，优先上午起飞——新西兰快 2 小时，落地后还要取车、买东西、21:00 前入住。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>40</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>定机票后</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>flight-akl</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>南岛租车</t>
+          <t>尽早</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Christchurch取、Queenstown还；按航班确定实际取还车时间、网点及异地还车条件。</t>
+          <t>机票：皇后镇 → 奥克兰</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2/14 下午到奥克兰。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>50</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>定机票后</t>
-        </is>
-      </c>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>flight-home</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>60</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Hobbiton当天交通</t>
+          <t>尽早</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>租车自驾和大巴 / 接驳二选一，待定。租车要支持晚间还车；大巴或接驳要确认13:30前送达Shire’s Rest、16:20后能接回，并接受自购票。</t>
+          <t>机票：奥克兰 → 国内</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2/16 晚上起飞，2/17 早上到。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>60</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>auckland-hotel</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>70</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>尽早</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Twizel观星</t>
-        </is>
-      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>优先2/7当地产品；2/6前后是新月，观星条件最好。核准确集合点、语言、天气改期条件。2/6–2/8是长周末，场次更紧。</t>
+          <t>订奥克兰两晚（2/14–16）</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>同一家连住，选 CBD / Britomart 附近，能在 2/16 退房后寄存行李。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>65</v>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>car-south</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>80</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>定了机票后</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>订南岛租车</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>基督城取车、皇后镇还车，按航班定取还时间，确认异地还车费用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>hobbiton-transport</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>90</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>定了机票后</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>定 2/15 去 Hobbiton 怎么走</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>租车自驾（要能晚上还车），或坐大巴 / 接驳（要 13:30 前送到 Shire’s Rest、16:20 后能接回）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stargazing</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>尽早</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>订 2/7 Twizel 观星</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2/6 前后是新月，星空最好；长周末场次紧。确认集合点、语言和天气改期规则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dinner-kika</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>110</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>提前预约</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>订 Kika（2/9 晚餐，Wānaka）</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>约 18:00，两人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dinner-redcliff</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>120</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>提前预约</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>订 The Redcliff（2/11 晚餐，Te Anau）</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Milford 回来约 18:30。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dinner-bluekanu</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>130</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>提前预约</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>订 Blue Kanu（2/12 晚餐，皇后镇）</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>缆车下来后约 19:00。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>lunch-amano</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>140</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>提前预约</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>订 Amano（2/16 午餐，奥克兰）</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>12:30–14:00。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>rippon</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>150</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>订 Rippon 品酒（2/9 下午）</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>订不到就跳过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>skyline</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>160</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>可选</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>买 Skyline 缆车票（2/12）</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>网上或现场都能买。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>milford-terms</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>170</v>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>prep</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
         <is>
           <t>出发前</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>查Milford订单退改规则</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>确认RealNZ在天气取消（Milford Road封路）时是全额退款还是改期，以及改期可选日期。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>70</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>booking</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>按计划时间</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>重点餐厅</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Kika 2/9、The Redcliff 2/11、Blue Kanu 2/12、Amano 2/16，按计划时间查询和预约；可选Rippon品酒 2/9下午；Skyline缆车2/12可提前网上买票。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>80</v>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>查 Milford 订单的天气退改规则</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>host-notes</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>180</v>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>prep</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>出发前</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>房东入住说明</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>三处Airbnb的停车位置、门锁/钥匙、晚到要求；Fernhill尤其确认停车和回程方式。</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>110</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>payment</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>入住前</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>拿到三处民宿的入住说明</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>sydney-0201</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>190</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>prep</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>有空时</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>把 2/1 悉尼那晚记进账本</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>补上金额、是否已付和取消规则。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>pay-fernhill</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>2027-01-05</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>1/5</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Queenstown Fernhill付款 NZ$721.63</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Apple Pay付款。付款日早于免费取消截止（1/13），付款日与取消截止分别管理。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>120</v>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Apple Pay 付款。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cancel-fernhill</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>210</v>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>deadline</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>2027-01-13</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>1/13 15:00</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Queenstown Fernhill免费取消截止</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>之后至2/5 15:00前取消可获部分退款，具体金额按订单。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>130</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>payment</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>皇后镇 Fernhill 免费取消截止</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>pay-hikuwai</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>220</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>2027-01-26</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>1/26</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Wānaka Hikuwai尾款 NZ$346.84</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Apple Pay扣款；订金NZ$86.71已付。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>140</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>payment</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>pay-teanau</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>230</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
         <is>
           <t>2027-01-28</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>1/28</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Te Anau尾款 NZ$386.40</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Apple Pay扣款；订金NZ$96.60已付。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>150</v>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Te Anau 尾款 NZ$386.40</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cancel-greatsouthern</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>240</v>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>deadline</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>2027-02-01</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>2/1 14:00</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>悉尼Great Southern免费取消截止</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>之后不可取消；未入住收全额。房费¥1,361.31离店扣款。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>160</v>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>悉尼 Great Southern 免费取消截止</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>之后不能取消，房费 ¥1,361.31 离店扣款。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cancel-metropolitan</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>250</v>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>deadline</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>2027-02-03</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>2/3 14:00</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>基督城Metropolitan免费取消截止</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>之后不可取消；未入住收全额。房费¥601.43离店扣款，另有NZ$200可退押金。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>170</v>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>基督城 Metropolitan 免费取消截止</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cancel-hikuwai</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>260</v>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>deadline</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>2027-02-03</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>2/3 16:00</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Wānaka Hikuwai免费取消截止</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>入住前部分退款，比例按订单。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>180</v>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Wānaka Hikuwai 免费取消截止</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>之后取消只退一部分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cancel-teanau</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>270</v>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>deadline</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>2027-02-05</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>2/5 15:00</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Te Anau Private Ensuite免费取消截止</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>入住前部分退款，比例按订单。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>190</v>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Te Anau 免费取消截止</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>之后取消只退一部分。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>supplies-0205</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>280</v>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>prep</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>2027-02-05</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>2/5</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2/6长周末补给</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2/6 Waitangi Day是限制营业日，部分超市和商店不开；2/5在途中把早餐、路餐和饮水买齐。</t>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>买齐长周末补给</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2/6 Waitangi Day 不少商店不开，路上把 2/6 的早餐、路餐和水买好。</t>
         </is>
       </c>
     </row>
@@ -11097,7 +11476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11143,12 +11522,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2/10 Wānaka → Te Anau：改走Crown Range，顺路Arrowtown</t>
+          <t>天气不好就别翻 Crown Range</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>已采用 · 不涉及订单</t>
+          <t>2/10</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -11158,12 +11537,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>行程文件主线经Cromwell + Kawarau Gorge到Frankton（约110公里）。改走Cardrona Valley Road翻Crown Range到Frankton约60公里，少约50公里、纯驾驶省约20–30分钟；Crown Range下山就是Arrow Junction，Arrowtown只需绕5分钟，可在这里吃午饭或喝咖啡。两条路线从Frankton起完全相同（Kingston → Five Rivers → Mossburn → Te Anau）。</t>
+          <t>Crown Range 是新西兰最高的铺装公路之一，皇后镇一侧连续急弯。起雾、大风或下雨时，改走 Cromwell 和 Kawarau 峡谷，多约 50 公里、20–30 分钟，从 Frankton 起路线一样。</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Crown Range是新西兰海拔最高的铺装主干道之一（约1,076米），Queenstown一侧有连续急弯；驾驶者不熟悉山路、起雾或大风时仍走Cromwell。Cromwell路线更平缓，2月沿途有水果摊。已采用为主线，Cromwell留作坏天气备选；导航时把Cardrona和Arrowtown设为途经点，否则手机可能自动选Cromwell。</t>
+          <t>导航时把 Cardrona、Arrowtown 设为途经点，不然手机可能直接带你走 Cromwell。</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -11178,27 +11557,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2/10与2/12重复Frankton–Kingston–Five Rivers路段</t>
+          <t>Hobbiton 那天是长日子</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>保持住宿不变</t>
+          <t>2/15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>d10,d12</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>这是Te Anau作为Milford大巴起点带来的固定代价：2/11已订RealNZ从Te Anau出发，从Queenstown当天往返Milford会变成12小时以上的大巴日。两天重复约2小时车程，换来Milford当天从容出发。</t>
+          <t>奥克兰到 Shire’s Rest 单程约 175 公里，来回 4.5–5 小时，加上 2.5 小时导览，全天 10 小时左右，前一天还刚飞过来。</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>执行上把湖边停留只放在一天：2/10在Kingston停10–20分钟，2/12经过Kingston不再停，直接到Queenstown早点吃午饭，下午多一点湖边时间。</t>
+          <t>租车的话两人轮流开，09:00 出发更从容；坐大巴或接驳就盯紧 13:30 报到和 16:20 结束。两种都建议 2/14 早点睡、午饭在 Shire’s Rest 解决、晚饭订 20:00 以后。</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -11209,88 +11588,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2/15 Hobbiton当天往返约5–6小时车程</t>
+          <t>2/6–2/8 是新西兰长周末</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>保持当天往返，交通方式待定</t>
+          <t>2/5–2/8</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d5,d6,d7,d8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Auckland到The Shire’s Rest单程约175公里，去回纯驾驶约4.5–5小时，加2.5小时导览和缓冲，全天约10–11小时，前一天还刚从Queenstown飞来。Auckland两晚尚未预订，理论上可改成2/15住Matamata/Cambridge，但会多一次搬行李，2/16早上还要开2小时回城，城市日被压缩，所以不建议。</t>
+          <t>2/6（周六）Waitangi Day、2/8（周一）补休。Mt Cook 停车场上午很早就满；2/6 不少商店不开；很多餐厅这两天加收 10–15% 假日附加费；观星和晚餐更难订。</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>如果租车：两人轮流开，去程和回程各换一次人；09:00出发比09:30更稳，周一早上出城方向不堵；租车选支持晚间自助还车、离酒店近的网点。如果坐大巴或接驳：不用开车更省力，但要确认班次衔接13:30报到和16:20结束。两种都建议2/14晚上早点休息、午饭在Shire’s Rest解决、晚餐订20:00以后或不订。</t>
+          <t>2/5 路上买齐补给，2/6 07:15–07:30 出发去 Mt Cook，观星和 2/8 晚餐尽早订。</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>40</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2/6–2/8 Waitangi长周末</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>保持顺序，提前出发和预订</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>d5,d6,d7,d8</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2027/2/6（周六）是Waitangi Day，2/8（周一）是补休日，2/5–2/8全程在Mackenzie和Wānaka的热门段。主要影响：White Horse Hill停车场周末上午很早停满；2/6是限制营业日，部分超市和商店不开门；不少餐厅在2/6和2/8收公众假期附加费（常见10–15%）；观星和Wānaka晚餐更难订。</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>建议：2/5在途中买齐2/6的补给；2/6提前到07:15–07:30出发去Mt Cook，天气不好就和2/7互换（两天都在长周末内）；观星和2/8晚餐尽早订；Kika放在2/9周二不受影响，保持。</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>50</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>已订住宿：不建议改订</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>不改订单</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>对照路线后，没有哪一笔已订住宿改了会明显更好：Te Anau是Milford的必要基地，Twizel连住三晚兼顾Mt Cook和观星，Wānaka和Fernhill的位置与当天安排吻合。可以优化的只有待订部分：Auckland两晚选CBD/Britomart、可寄存行李且附近有晚间还车网点的酒店。</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>如果之后仍想调整，免费取消截止（当地时间）依次为：Queenstown Fernhill 2027/1/13 15:00、悉尼Great Southern 2/1 14:00、基督城Metropolitan 2/3 14:00、Wānaka Hikuwai 2/3 16:00、Te Anau 2/5 15:00；Twizel未展开条款，不预设可免费取消。</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
content: add sunset-season evening walks to the 2027 itinerary
- 2/5 Lake Ruataniwha sunset stroll after dinner
- 2/8 Diamond Lake + Lake Wānaka Lookout after check-in
- 2/12 lunch in Frankton, Kelvin Peninsula Sculpture Trail, check-in 15:30–16:00, Skyline in the evening
- 2/13 Moke Lake loop in the evening, Fergburger moved to dinner
- Rental terms: no Glenorchy–Paradise Road; gravel driving note for Moke Lake Road

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3097,22 +3097,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fergburger-map</t>
+          <t>diamond-lake-map</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Diamond Lake 停车场</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Diamond+Lake+Track+Car+Park%2C+Wanaka-Mount+Aspiring+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3126,41 +3126,41 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fergburger-official</t>
+          <t>diamond-lake-official</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Fergburger官网</t>
+          <t>Lake Wānaka Lookout Track</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.fergburger.com/</t>
+          <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/otago/places/diamond-lake-and-hospital-flat/things-to-do/lake-wanaka-lookout-track</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>frankton-map</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>Frankton / Remarkables Park</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Remarkables+Park%2C+Frankton%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -3184,70 +3184,70 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>kelvin-trail-map</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Kelvin Heights 雕塑环线起点</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Peninsula+Road+and+Grove+Lane%2C+Kelvin+Heights%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>kelvin-trail-official</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>Kelvin Heights Peninsula Trail</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.queenstownnz.co.nz/listing/kelvin-heights-peninsula-trail/9101/</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Queenstown NZ</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>moke-lake-map</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Moke+Lake%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3271,99 +3271,99 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>moke-lake-official</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Moke Lake Loop Track</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/otago/places/queenstown-area/things-to-do/moke-lake-loop-track</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>fergburger-map</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>fergburger-official</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Glenorchy回住宿</t>
+          <t>Fergburger官网</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.fergburger.com/</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>机场方向参考路线</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3373,55 +3373,55 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>导航10</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>nav11-out-route</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>市区参考起点经Matamata到现场</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Britomart%2C+Auckland%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>导航11</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>nav11-matamata-route</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Matamata休息后到现场</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3431,26 +3431,26 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
-          <t>导航11</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>nav11-back-route</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>现场回Auckland市中心参考</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3460,12 +3460,215 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;destination=Britomart%2C+Auckland%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>nav08-route</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>完整路线到Fernhill</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>导航08</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>nav09-out-route</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>去程经Bennetts Bluff</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>nav09-back-route</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Glenorchy回住宿</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>机场方向参考路线</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>导航10</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>nav11-out-route</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>市区参考起点经Matamata到现场</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Britomart%2C+Auckland%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>导航11</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>nav11-matamata-route</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Matamata休息后到现场</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>导航11</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>nav11-back-route</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>现场回Auckland市中心参考</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;destination=Britomart%2C+Auckland%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
         <is>
           <t>导航11</t>
         </is>
@@ -4578,7 +4781,8 @@
         <is>
           <t>住宿｜Hikuwai Haven 1，1 Outlet Road；16:00后入住、2/10 10:00前退房。
 位置影响｜住宿到镇上按开车安排。纯驾驶约2.5–3小时，留出午餐和停靠。
-长周末｜今天是Waitangi Day补休日，Wānaka餐厅和超市人多，晚餐提前订或早点吃。</t>
+长周末｜今天是Waitangi Day补休日，Wānaka餐厅和超市人多，晚餐提前订，约 20:00。
+傍晚｜Diamond Lake 停车场在 Mt Aspiring Road，离住处约 20 分钟，全程铺装路；步道上没有厕所，停车场有。</t>
         </is>
       </c>
     </row>
@@ -4938,12 +5142,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>进入Queenstown，住进Fernhill</t>
+          <t>Kelvin半岛湖边步道，傍晚坐缆车</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>下午湖边散步，晚上用一顿饭开启皇后镇。</t>
+          <t>下午在Kelvin半岛沿湖走一圈，傍晚坐缆车看皇后镇。</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -4975,7 +5179,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>09:30左右出发；最迟10:00前退房</t>
+          <t>09:30左右出发；15:30–16:00入住</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -5044,12 +5248,12 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>沿湖开去Glenorchy</t>
+          <t>沿湖开去Glenorchy，傍晚Moke Lake</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>公路、红船屋、湿地步道和小镇午餐。</t>
+          <t>公路、红船屋、湿地步道，傍晚绕Moke Lake走一圈。</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -5108,7 +5312,8 @@
         <is>
           <t>住宿｜Fernhill山景单间，第二晚。
 沙蝇｜Glenorchy码头和Lagoon湿地沙蝇多，下车前喷驱蚊液。
-天气备选｜小雨时缩短Lagoon段；大雨、路况或能见度不适合时留Queenstown城市活动。只到Glenorchy，不走碎石支路。</t>
+天气备选｜小雨时缩短Lagoon段；大雨、路况或能见度不适合时留Queenstown城市活动。只到Glenorchy，不往Paradise方向开（租车合同禁止Glenorchy–Paradise Road）。
+碎石路｜Moke Lake Road后段约8km碎石路，窄、陡、有弯，有对向来车；车速压到30–40km/h。大雨后不去，改Queenstown Gardens湖边散步。碎石路造成的玻璃、轮胎、底盘损伤保险可能不赔，出发前看一眼保险条款。</t>
         </is>
       </c>
     </row>
@@ -5545,7 +5750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6541,66 +6746,66 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>20:00–21:00</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Fairlie / Twizel</t>
+          <t>Lake Ruataniwha</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>早餐：Riccarton；午餐：Fairlie Bakehouse；晚餐：Twizel镇上</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+          <t>晚饭后开 5–10 分钟到湖边散步，看 Ben Ohau 山脉后面的日落（约 21:00）。</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>湖边日落</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>累了就跳过，2/7 上午还会来。</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ruataniwha-map</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>d6</t>
+          <t>d5</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>07:15–07:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Twizel → White Horse Hill</t>
+          <t>Fairlie / Twizel</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Twizel出发，沿SH80进山，尽早到White Horse Hill停车场。</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>长周末停车场早满，提前出发</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>长周末停车场上午很早就满。</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>white-horse-hill-route</t>
-        </is>
-      </c>
+          <t>早餐：Riccarton；午餐：Fairlie Bakehouse；晚餐：Twizel镇上</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6609,36 +6814,36 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>09:15–14:00左右</t>
+          <t>07:15–07:30</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Hooker Valley Track</t>
+          <t>Twizel → White Horse Hill</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hooker Valley徒步，含拍照、路餐和休息预留4–5小时。</t>
+          <t>Twizel出发，沿SH80进山，尽早到White Horse Hill停车场。</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>全天主角</t>
+          <t>长周末停车场早满，提前出发</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>全程10km，官方约3小时往返。</t>
+          <t>长周末停车场上午很早就满。</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>doc-hooker-official</t>
+          <t>white-horse-hill-route</t>
         </is>
       </c>
     </row>
@@ -6649,32 +6854,36 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>09:15–14:00左右</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Mount Cook Village / Peter’s Lookout</t>
+          <t>Hooker Valley Track</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>村内咖啡休息；返程在Peter’s Lookout短停看Pukaki。</t>
+          <t>Hooker Valley徒步，含拍照、路餐和休息预留4–5小时。</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Pukaki回望</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>全天主角</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>全程10km，官方约3小时往返。</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>peters-lookout-route</t>
+          <t>doc-hooker-official</t>
         </is>
       </c>
     </row>
@@ -6685,26 +6894,34 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16:30–18:00左右</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Twizel</t>
+          <t>Mount Cook Village / Peter’s Lookout</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>回Twizel吃晚餐，晚上放松。</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr"/>
+          <t>村内咖啡休息；返程在Peter’s Lookout短停看Pukaki。</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Pukaki回望</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>peters-lookout-route</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6713,21 +6930,21 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>16:30–18:00左右</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>随身路餐 / Twizel</t>
+          <t>Twizel</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>早餐：出发前吃足；午餐：随身路餐；晚餐：Twizel</t>
+          <t>回Twizel吃晚餐，晚上放松。</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -6737,38 +6954,30 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>d7</t>
+          <t>d6</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Lake Ruataniwha</t>
+          <t>随身路餐 / Twizel</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>慢早餐；若前一天已完成Mt Cook，安排Lake Ruataniwha湖边轻走。</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>恢复日</t>
-        </is>
-      </c>
+          <t>早餐：出发前吃足；午餐：随身路餐；晚餐：Twizel</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>ruataniwha-map</t>
-        </is>
-      </c>
+      <c r="H35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6777,32 +6986,32 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>High Country Salmon</t>
+          <t>Lake Ruataniwha</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>High Country Salmon / Logans吃一顿鲑鱼午餐。</t>
+          <t>慢早餐；若前一天已完成Mt Cook，安排Lake Ruataniwha湖边轻走。</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>鲑鱼午餐</t>
+          <t>恢复日</t>
         </is>
       </c>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>logans-official</t>
+          <t>ruataniwha-map</t>
         </is>
       </c>
     </row>
@@ -6813,28 +7022,32 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>中午</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>住宿 / Pukaki南岸</t>
+          <t>High Country Salmon</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>回住宿休息、洗衣或整理行李；视天气短去Pukaki南岸。</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
+          <t>High Country Salmon / Logans吃一顿鲑鱼午餐。</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>鲑鱼午餐</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>pukaki-visitor-route</t>
+          <t>logans-official</t>
         </is>
       </c>
     </row>
@@ -6845,36 +7058,28 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>夜间</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Twizel观星</t>
+          <t>住宿 / Pukaki南岸</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>优先预约Twizel当地观星，具体集合点、语言和时间以确认单为准。</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>星空</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>观星待订。</t>
-        </is>
-      </c>
+          <t>回住宿休息、洗衣或整理行李；视天气短去Pukaki南岸。</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
-          <t>silver-river-official</t>
+          <t>pukaki-visitor-route</t>
         </is>
       </c>
     </row>
@@ -6885,49 +7090,61 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>夜间</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Twizel</t>
+          <t>Twizel观星</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>早餐：镇上或住宿；午餐：High Country Salmon；晚餐：观星前在Twizel吃</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+          <t>优先预约Twizel当地观星，具体集合点、语言和时间以确认单为准。</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>星空</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>观星待订。</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>silver-river-official</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>d8</t>
+          <t>d7</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Twizel → Omarama</t>
+          <t>Twizel</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Twizel出发，Omarama短休息。</t>
+          <t>早餐：镇上或住宿；午餐：High Country Salmon；晚餐：观星前在Twizel吃</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -6941,34 +7158,26 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>上午后段</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Lindis Pass Lookout</t>
+          <t>Twizel → Omarama</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Lindis Pass正规观景停车场停15–20分钟。</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>山口公路</t>
-        </is>
-      </c>
+          <t>Twizel出发，Omarama短休息。</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>lindis-pass-route,doc-lindis-official</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -6977,30 +7186,34 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>午后</t>
+          <t>上午后段</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Tarras → Luggate → Wānaka</t>
+          <t>Lindis Pass Lookout</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>经Tarras、Luggate到Wānaka，湖边午餐或咖啡。</t>
+          <t>Lindis Pass正规观景停车场停15–20分钟。</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>午后湖岸</t>
+          <t>山口公路</t>
         </is>
       </c>
       <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>lindis-pass-route,doc-lindis-official</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -7009,34 +7222,30 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16:00后</t>
+          <t>午后</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hikuwai Haven 1</t>
+          <t>Tarras → Luggate → Wānaka</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>入住Hikuwai Haven 1，再按体力安排湖边散步和晚餐。</t>
+          <t>经Tarras、Luggate到Wānaka，湖边午餐或咖啡。</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>入住两晚</t>
+          <t>午后湖岸</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>hikuwai-map</t>
-        </is>
-      </c>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -7045,138 +7254,130 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>16:00后</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>途中 / Wānaka</t>
+          <t>Hikuwai Haven 1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>早餐：Twizel；午餐：途中或Wānaka；晚餐：Wānaka镇上</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
+          <t>入住Hikuwai Haven 1，放下行李歇一会儿。</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>入住两晚</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>hikuwai-map</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>09:00–11:00</t>
+          <t>17:00–19:30</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Mount Iron</t>
+          <t>Diamond Lake / Lake Wānaka Lookout</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mount Iron步道，按1.5–2小时准备，有上下坡。</t>
+          <t>开约 20 分钟到 Diamond Lake 停车场：先到 Diamond Lake 湖边，再上 Lake Wānaka Lookout 俯瞰整个湖，往返约 2 小时，台阶多。只想轻松走就绕 Diamond Lake 一圈，约 45 分钟。</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>轻徒步</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>傍晚俯瞰 Wānaka 湖</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>日落约 21:00，天亮着时间很宽。</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>mount-iron-official,mount-iron-route</t>
+          <t>diamond-lake-map,diamond-lake-official</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>20:00左右</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Wānaka湖边 · That Wānaka Tree</t>
+          <t>Wānaka镇上</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>湖边午餐，前后去Roys Bay湖岸看That Wānaka Tree，之后咖啡和休息。</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>湖里那棵树</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>只在岸边看，不攀爬、不下水靠近。</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>wanaka-lakefront-route,wanaka-tree-map</t>
-        </is>
-      </c>
+          <t>回镇上吃晚饭。</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>湖边 / Cinema Paradiso</t>
+          <t>途中 / Wānaka</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>沿湖走走；喜欢电影时查看Cinema Paradiso实际片单。</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>可选电影</t>
-        </is>
-      </c>
+          <t>早餐：Twizel；午餐：途中或Wānaka；晚餐：Wānaka镇上</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>paradiso-official</t>
-        </is>
-      </c>
+      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -7185,36 +7386,32 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>下午（可选）</t>
+          <t>09:00–11:00</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Rippon品酒</t>
+          <t>Mount Iron</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>可选：Rippon湖景酒庄品酒，约45–60分钟，需提前预约场次；驾驶者不饮酒。</t>
+          <t>Mount Iron步道，按1.5–2小时准备，有上下坡。</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>补选项</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>订不到场次就跳过，不影响晚餐。</t>
-        </is>
-      </c>
+          <t>轻徒步</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>rippon-official,rippon-map</t>
+          <t>mount-iron-official,mount-iron-route</t>
         </is>
       </c>
     </row>
@@ -7225,36 +7422,36 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>18:00左右</t>
+          <t>中午</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Kika</t>
+          <t>Wānaka湖边 · That Wānaka Tree</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Kika分享式晚餐，待预约。之后回住宿休息。</t>
+          <t>湖边午餐，前后去Roys Bay湖岸看That Wānaka Tree，之后咖啡和休息。</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>认真吃一顿</t>
+          <t>湖里那棵树</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Kika待预约。</t>
+          <t>只在岸边看，不攀爬、不下水靠近。</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>kika-official,kika-route</t>
+          <t>wanaka-lakefront-route,wanaka-tree-map</t>
         </is>
       </c>
     </row>
@@ -7265,138 +7462,142 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>湖畔 / Kika</t>
+          <t>湖边 / Cinema Paradiso</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：湖畔简餐；晚餐：Kika</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
+          <t>沿湖走走；喜欢电影时查看Cinema Paradiso实际片单。</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>可选电影</t>
+        </is>
+      </c>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>paradiso-official</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>下午（可选）</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Wānaka → Cardrona → Crown Range</t>
+          <t>Rippon品酒</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>退房出发，沿Cardrona Valley Road经Cardrona小镇翻Crown Range；山顶观景点短停。</t>
+          <t>可选：Rippon湖景酒庄品酒，约45–60分钟，需提前预约场次；驾驶者不饮酒。</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>最长转场日</t>
+          <t>补选项</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>下山一侧连续急弯，低速档慢下。</t>
+          <t>订不到场次就跳过，不影响晚餐。</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>crown-range-route</t>
+          <t>rippon-official,rippon-map</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>上午后段至中午</t>
+          <t>18:00左右</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Arrowtown</t>
+          <t>Kika</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Arrowtown老街散步、午餐或咖啡，约60–90分钟；之后到Frankton加油。</t>
+          <t>Kika分享式晚餐，待预约。之后回住宿休息。</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>淘金小镇午餐</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr"/>
+          <t>认真吃一顿</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Kika待预约。</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>arrowtown-map</t>
+          <t>kika-official,kika-route</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>中午至下午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Kingston → Five Rivers → Mossburn</t>
+          <t>湖畔 / Kika</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>经Kingston、Five Rivers、Mossburn到Te Anau；Kingston湖边短停，分段休息。</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>分段休息</t>
-        </is>
-      </c>
+          <t>早餐：出发前；午餐：湖畔简餐；晚餐：Kika</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>nav07-leg2-route</t>
-        </is>
-      </c>
+      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -7405,32 +7606,36 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>15:00–16:30左右</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Wānaka → Cardrona → Crown Range</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>入住，去湖边走走，购买翌日路餐、检查活动集合点。</t>
+          <t>退房出发，沿Cardrona Valley Road经Cardrona小镇翻Crown Range；山顶观景点短停。</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>为Milford准备</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
+          <t>最长转场日</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>下山一侧连续急弯，低速档慢下。</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>te-anau-ensuite-map</t>
+          <t>crown-range-route</t>
         </is>
       </c>
     </row>
@@ -7441,130 +7646,134 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午后段至中午</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Frankton / Kingston / Te Anau</t>
+          <t>Arrowtown</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：Te Anau镇上，早点结束</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>Arrowtown老街散步、午餐或咖啡，约60–90分钟；之后到Frankton加油。</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>淘金小镇午餐</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>arrowtown-map</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>08:00左右</t>
+          <t>中午至下午</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Kingston → Five Rivers → Mossburn</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+          <t>经Kingston、Five Rivers、Mossburn到Te Anau；Kingston湖边短停，分段休息。</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>装备检查</t>
+          <t>分段休息</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>nav07-leg2-route</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>09:15左右到，09:30前完成报到</t>
+          <t>15:00–16:30左右</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+          <t>入住，去湖边走走，购买翌日路餐、检查活动集合点。</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>已订集合</t>
+          <t>为Milford准备</t>
         </is>
       </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr">
         <is>
-          <t>realnz-map,realnz-walk-route</t>
+          <t>te-anau-ensuite-map</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>09:50–17:00</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Milford Sound</t>
+          <t>Frankton / Kingston / Te Anau</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>峡湾</t>
-        </is>
-      </c>
+          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：Te Anau镇上，早点结束</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>realnz-booking</t>
-        </is>
-      </c>
+      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -7573,11 +7782,11 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>08:00左右</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7587,16 +7796,16 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff，之后回住宿。</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr"/>
+          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>装备检查</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>redcliff-official</t>
-        </is>
-      </c>
+      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -7605,130 +7814,130 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:15左右到，09:30前完成报到</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr"/>
+          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>已订集合</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>realnz-map,realnz-walk-route</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>09:50–17:00</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>Milford Sound</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr"/>
+          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>峡湾</t>
+        </is>
+      </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>realnz-booking</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>经Kingston到Queenstown，午餐吃Fergburger；店在市中心Shotover Street，饭点排队常很长，尽量错开12:00–13:30，或打包到湖边吃。</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>皇后镇招牌汉堡</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff，之后回住宿。</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr">
         <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
+          <t>redcliff-official</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>15:00后</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>入住15 Greenstone Place，放下行李休息。</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>入住Fernhill</t>
-        </is>
-      </c>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>fernhill-map</t>
-        </is>
-      </c>
+      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7737,36 +7946,28 @@
         </is>
       </c>
       <c r="B64" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16:30–18:30</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>俯瞰皇后镇</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>缆车票可网上或现场买；大风时可能停运。</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>nav08-route</t>
         </is>
       </c>
     </row>
@@ -7777,32 +7978,32 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>19:00–晚上</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Blue Kanu / 湖边</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>下山后湖边走走，晚餐Blue Kanu。不去缆车就改Queenstown Gardens湖边轻走。</t>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>晚餐</t>
+          <t>午餐</t>
         </is>
       </c>
       <c r="G65" t="inlineStr"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>blue-kanu-official</t>
+          <t>frankton-map</t>
         </is>
       </c>
     </row>
@@ -7813,170 +8014,178 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>13:30–15:00</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Fergburger / Blue Kanu</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Fergburger；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>起点在Peninsula Road和Grove Lane路口。</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>15:30–16:00</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>湖边公路</t>
+          <t>入住Fernhill</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>fernhill-map</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>傍晚 17:00–19:00</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>Skyline Gondola · Bob’s Peak</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>红船屋</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr"/>
+          <t>俯瞰皇后镇</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>日落约21:00；想在山上看日落，就先吃晚饭、19:30后再上山。缆车票网上或现场买，大风时可能停运。</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>19:30–晚上</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Blue Kanu / 湖边</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>下山后湖边走走，晚餐Blue Kanu。缆车停运就改Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>湿地步道</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
-        </is>
-      </c>
+          <t>晚餐</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>nav09-back-route</t>
-        </is>
-      </c>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7985,26 +8194,34 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Queenstown</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>湖边晚餐，整理行李、准备次日加油还车。</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>湖边公路</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>nav09-out-route</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8013,196 +8230,208 @@
         </is>
       </c>
       <c r="B72" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Glenorchy / Queenstown</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Queenstown</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>红船屋</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>bennetts-bluff-official</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>南岛收车</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr"/>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>等飞机</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>zqn-map</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>17:30–20:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
+          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>航班</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
+          <t>傍晚湖面倒影</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>20:30前开回铺装路。</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>moke-lake-map,moke-lake-official</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>20:30左右</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>回市中心吃Fergburger，饭点后排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>连住两晚</t>
+          <t>皇后镇招牌汉堡</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>傍晚</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Britomart / Viaduct Harbour</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Britomart、Quay Street、Viaduct Harbour散步；时间充裕再延伸Wynyard Quarter。</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>海港散步</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr"/>
     </row>
@@ -8213,158 +8442,166 @@
         </is>
       </c>
       <c r="B78" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Auckland市中心</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>南岛收车</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>08:30–09:30</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Auckland市区出发</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>交通待定</t>
+          <t>等飞机</t>
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>nav11-out-route,hobbiton-transfers-official</t>
+          <t>zqn-map</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>12:30–13:00</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>The Shire’s Rest</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr"/>
+          <t>飞奥克兰。</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>航班</t>
+        </is>
+      </c>
       <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>shire-rest-map</t>
-        </is>
-      </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>13:30前</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>The Shire’s Rest Ticketing Office</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>在The Shire’s Rest Ticketing Office报到。</t>
+          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>已订报到</t>
+          <t>连住两晚</t>
         </is>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>13:50–约16:20</t>
+          <t>傍晚</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>Britomart / Viaduct Harbour</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
+          <t>Britomart、Quay Street、Viaduct Harbour散步；时间充裕再延伸Wynyard Quarter。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>中文导览</t>
+          <t>海港散步</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
@@ -8373,38 +8610,30 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16:30–17:00左右返程</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Hobbiton → Auckland</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>晚间回城</t>
-        </is>
-      </c>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Auckland市中心</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8413,190 +8642,198 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>08:30–09:30</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Shire’s Rest / Auckland</t>
+          <t>Auckland市区出发</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
+          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>交通待定</t>
+        </is>
+      </c>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>nav11-out-route,hobbiton-transfers-official</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>12:30–13:00</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>The Shire’s Rest</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
+          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>shire-rest-map</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>13:30前</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>The Shire’s Rest Ticketing Office</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
+          <t>在The Shire’s Rest Ticketing Office报到。</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>美术馆</t>
+          <t>已订报到</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>art-gallery-map,art-gallery-official</t>
+          <t>hobbiton-booking</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>13:50–约16:20</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
+          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>完整午餐</t>
+          <t>中文导览</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr">
-        <is>
-          <t>amano-map,amano-official</t>
-        </is>
-      </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>16:30–17:00左右返程</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>Hobbiton → Auckland</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr"/>
+          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>晚间回城</t>
+        </is>
+      </c>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>nav11-back-route</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>Shire’s Rest / Auckland</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>夜航回国</t>
-        </is>
-      </c>
+          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8605,21 +8842,21 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -8629,102 +8866,266 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>转机</t>
+          <t>美术馆</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>art-gallery-map,art-gallery-official</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>09:10–11:10</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>CZ3803 → 杭州萧山T4</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>飞回杭州，取行李回家。</t>
+          <t>Britomart午餐，首选Amano，待预约。</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>到家</t>
+          <t>完整午餐</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>hgh-airport-map</t>
+          <t>amano-map,amano-official</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>落地后</t>
+          <t>Britomart</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>按航班实际到达时间</t>
-        </is>
-      </c>
+          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>50</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>晚上</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Auckland Airport</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>夜航回国</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>akl-intl-map,akl-departure-official</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>90</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>市区 / Amano</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>10</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>05:00–09:10</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>广州白云T2</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>转机</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>20</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>09:10–11:10</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>CZ3803 → 杭州萧山T4</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>90</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>落地后</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>按航班实际到达时间</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9017,12 +9418,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，加休息午餐留3–4小时；15:00后入住。</t>
+          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，12:00–13:00到Frankton；Kelvin半岛步道后15:30–16:00入住。</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>3 Thomson Place → SH94 / Mossburn → SH97 / Five Rivers → SH6 / Kingston → Frankton → SH6A / Queenstown → Fernhill → 15 Greenstone Place</t>
+          <t>3 Thomson Place → SH94 / Mossburn → SH97 / Five Rivers → SH6 / Kingston → Frankton → Kelvin Heights → SH6A / Queenstown → Fernhill → 15 Greenstone Place</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -9032,7 +9433,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nav08-route,boundary-street-map,fernhill-map,qldc-parking-official</t>
+          <t>nav08-route,kelvin-trail-map,fernhill-map,qldc-parking-official</t>
         </is>
       </c>
     </row>
@@ -9054,22 +9455,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>09:00左右出发；单程约50–70分钟，往返按约2小时，连步道午餐留5–6小时。</t>
+          <t>09:00左右出发；单程约50–70分钟，往返按约2小时，连步道午餐留5–6小时；傍晚再去Moke Lake，单程约30分钟。</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15 Greenstone Place → Queenstown–Glenorchy Road → Bennetts Bluff Viewpoint → Glenorchy Waterfront / Wharf → Lagoon步道 → 原路回Fernhill</t>
+          <t>15 Greenstone Place → Queenstown–Glenorchy Road → Bennetts Bluff Viewpoint → Glenorchy Waterfront / Wharf → Lagoon步道 → 原路回Fernhill → 傍晚 Moke Lake Road → Moke Lake → 市中心</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Bennetts Bluff是途中观景站；Glenorchy Waterfront/Wharf是小镇主停车区域。Paradise及未铺装支线不纳入本日主路线。</t>
+          <t>Bennetts Bluff是途中观景站；Glenorchy Waterfront/Wharf是小镇主停车区域。不往Paradise方向开（租车合同禁止）。Moke Lake Road后段是碎石路，慢开。</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nav09-out-route,glenorchy-lagoon-map,nav09-back-route,bennetts-bluff-official,glenorchy-lagoon-official</t>
+          <t>nav09-out-route,glenorchy-lagoon-map,nav09-back-route,moke-lake-map,bennetts-bluff-official,glenorchy-lagoon-official</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9874,17 +10275,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Kingston → Queenstown中心</t>
+          <t>Kingston → Frankton</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>约45–60分钟</t>
+          <t>约40–50分钟</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>市区午餐；停车可查Boundary Street等正规车场，按牌付费。</t>
+          <t>Frankton一带午餐，停商场或有标识的车位。</t>
         </is>
       </c>
     </row>
@@ -9899,42 +10300,42 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>中心 → 15 Greenstone Place</t>
+          <t>Frankton → Kelvin Heights</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>约10–15分钟</t>
+          <t>约10分钟</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>上Fernhill后按房东说明停车，15:00前不默认能入房。</t>
+          <t>停Peninsula Road / Grove Lane附近的公共车位，走雕塑环线约1小时。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>nav09</t>
+          <t>nav08</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Fernhill → Bennetts Bluff</t>
+          <t>Kelvin Heights → 15 Greenstone Place</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>约25–35分钟</t>
+          <t>约20–25分钟</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>使用新正规观景停车场，步行观景20–30分钟，不停旧盲弯路肩。</t>
+          <t>穿过市区上Fernhill，按房东说明停车；缆车站在Brecon Street，离住处很近。</t>
         </is>
       </c>
     </row>
@@ -9945,11 +10346,11 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bennetts Bluff → Glenorchy Wharf</t>
+          <t>Fernhill → Bennetts Bluff</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -9959,7 +10360,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>停湖滨正规车位；码头、红船屋拍照20–30分钟。</t>
+          <t>使用新正规观景停车场，步行观景20–30分钟，不停旧盲弯路肩。</t>
         </is>
       </c>
     </row>
@@ -9970,21 +10371,21 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>码头/湖滨停车 → Lagoon Walkway</t>
+          <t>Bennetts Bluff → Glenorchy Wharf</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>步行</t>
+          <t>约25–35分钟</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>按标识接入，留1–2小时；官方路线3.2km，雨后注意积水提示。</t>
+          <t>停湖滨正规车位；码头、红船屋拍照20–30分钟。</t>
         </is>
       </c>
     </row>
@@ -9995,71 +10396,71 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Glenorchy → Fernhill</t>
+          <t>码头/湖滨停车 → Lagoon Walkway</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>约50–70分钟</t>
+          <t>步行</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>午餐后原路返；途中最多选一处正规停车点，下午回城。</t>
+          <t>按标识接入，留1–2小时；官方路线3.2km，雨后注意积水提示。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>nav10</t>
+          <t>nav09</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>住宿 → Frankton加油</t>
+          <t>Glenorchy → Fernhill</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>约20–30分钟</t>
+          <t>约50–70分钟</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>按租车油量要求加油，保留凭证。</t>
+          <t>午餐后原路返；途中最多选一处正规停车点，下午回城休息。</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>nav10</t>
+          <t>nav09</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>加油 → 皇后镇机场还车</t>
+          <t>Fernhill → Moke Lake</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>约5–10分钟</t>
+          <t>约25–35分钟</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>10:00 还车；验车时拍照留底。</t>
+          <t>Glenorchy路走约10分钟后右转Moke Lake Road，先是陡弯铺装路，后段约8km碎石路；停湖边营地停车场。</t>
         </is>
       </c>
     </row>
@@ -10070,71 +10471,71 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>还车 → 航站楼</t>
+          <t>住宿 → Frankton加油</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>步行或摆渡</t>
+          <t>约20–30分钟</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>12:30 前办托运，JQ296 13:30 起飞。</t>
+          <t>按租车油量要求加油，保留凭证。</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>nav11</t>
+          <t>nav10</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>取车点 → Matamata</t>
+          <t>加油 → 皇后镇机场还车</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>约2–2.5小时，路况另留量</t>
+          <t>约5–10分钟</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>可在Matamata短休息；i-SITE只是途中停靠参考，并非这张票的报到点。</t>
+          <t>10:00 还车；验车时拍照留底。</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>nav11</t>
+          <t>nav10</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Matamata → The Shire’s Rest</t>
+          <t>还车 → 航站楼</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>约15–25分钟</t>
+          <t>步行或摆渡</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>最终目的地501 Buckland Road。乡村道路跟当日导航与标识，不套用旧攻略出口号。</t>
+          <t>12:30 前办托运，JQ296 13:30 起飞。</t>
         </is>
       </c>
     </row>
@@ -10145,21 +10546,21 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>现场停车、午餐、报到</t>
+          <t>取车点 → Matamata</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>约30–60分钟缓冲</t>
+          <t>约2–2.5小时，路况另留量</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>目标12:30–13:00到；停访客停车区，13:30前到Ticketing Office。</t>
+          <t>可在Matamata短休息；i-SITE只是途中停靠参考，并非这张票的报到点。</t>
         </is>
       </c>
     </row>
@@ -10170,21 +10571,21 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>13:50 → 约16:20</t>
+          <t>Matamata → The Shire’s Rest</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>已订导览约2.5小时</t>
+          <t>约15–25分钟</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>乘运营商巴士进出片场，私家车停在Shire’s Rest。</t>
+          <t>最终目的地501 Buckland Road。乡村道路跟当日导航与标识，不套用旧攻略出口号。</t>
         </is>
       </c>
     </row>
@@ -10195,19 +10596,69 @@
         </is>
       </c>
       <c r="B42" t="n">
+        <v>30</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>现场停车、午餐、报到</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>约30–60分钟缓冲</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>目标12:30–13:00到；停访客停车区，13:30前到Ticketing Office。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>nav11</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>40</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>13:50 → 约16:20</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>已订导览约2.5小时</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>乘运营商巴士进出片场，私家车停在Shire’s Rest。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>nav11</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
         <v>50</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>约16:30–17:00 → Auckland</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>约2.5–3小时</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>按19:00–20:00抵城安排；堵车、离场晚时顺延，不在当天衔接国际航班。</t>
         </is>

</xml_diff>

<commit_message>
content: D10 glowworm caves at 17:45, dinner 20:15, lakefront sunset after
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -5200,7 +5200,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>09:00左右出发；10:00前退房</t>
+          <t>09:00左右出发；17:15到RealNZ报到萤火虫团</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -5227,7 +5227,8 @@
         <is>
           <t>住宿｜Private Ensuite in the Heart of Te Anau，3 Thomson Place；15:00后入住。
 驾驶安排｜纯驾驶约3.5–4.5小时，加Arrowtown午餐和停靠留5–6小时；抵达时间随休息调整。
-坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。</t>
+坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。
+傍晚｜17:45 萤火虫洞团。Arrowtown 控制在 90 分钟内，15:00–16:30 到 Te Anau；改走 Cromwell 多 20–30 分钟也赶得上，最晚 16:30 前到住处。</t>
         </is>
       </c>
     </row>
@@ -5982,7 +5983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H115"/>
+  <dimension ref="A1:H116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8330,22 +8331,34 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:15–17:30</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Te Anau镇上</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>早点吃晚饭。</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
+          <t>开几分钟到85 Lakefront Drive报到，就是明天Milford的集合点。</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>报到</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>报到时间以确认单为准。</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>realnz-map</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8354,32 +8367,36 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>20:40–21:15</t>
+          <t>17:45–20:00</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau萤火虫洞</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>沿Lakefront Drive散步，湖岸朝西，看日落落在湖上；离住处几分钟。</t>
+          <t>RealNZ萤火虫洞团：坐船过湖，步行进洞，再坐小船看萤火虫，约2小时15分。</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>湖上日落</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>萤火虫</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>洞内8–12°C，带外套；洞里不能拍照。</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
+          <t>realnz-map,glowworm-official</t>
         </is>
       </c>
     </row>
@@ -8390,38 +8407,30 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>19:00–21:15（可选）</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Te Anau萤火虫洞</t>
+          <t>Te Anau镇上</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>可选：RealNZ萤火虫洞夜游，坐船过湖再进洞，约2小时15分；19:00那班回程的船差不多赶上日落。订了就不再单独去湖边。</t>
+          <t>回来直接吃晚饭；不少餐厅厨房21:00前后停止点餐，要提前订，选离湖边近的。</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>萤火虫</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>要预约，场次以RealNZ官网为准；第二天09:15要去Milford报到，累了就不订。</t>
-        </is>
-      </c>
-      <c r="H70" t="inlineStr">
-        <is>
-          <t>realnz-map,glowworm-official</t>
-        </is>
-      </c>
+          <t>晚饭</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8430,56 +8439,64 @@
         </is>
       </c>
       <c r="B71" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>21:00–21:15</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Frankton / Kingston / Te Anau</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：17:30在Te Anau镇上</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
+          <t>饭后沿Lakefront Drive走走，湖岸朝西，看21:09的日落，然后回住宿早点睡。</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>湖上日落</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>明早09:15去Milford报到。</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>realnz-walk-route</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>08:00左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Frankton / Kingston / Te Anau</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>装备检查</t>
-        </is>
-      </c>
+          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：20:15在Te Anau镇上（要订）</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
     </row>
@@ -8490,34 +8507,30 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>09:15左右到，09:30前完成报到</t>
+          <t>08:00左右</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>已订集合</t>
+          <t>装备检查</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr">
-        <is>
-          <t>realnz-map,realnz-walk-route</t>
-        </is>
-      </c>
+      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8526,32 +8539,32 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>09:50–17:00</t>
+          <t>09:15左右到，09:30前完成报到</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Milford Sound</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>峡湾</t>
+          <t>已订集合</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>realnz-booking</t>
+          <t>realnz-map,realnz-walk-route</t>
         </is>
       </c>
     </row>
@@ -8562,28 +8575,32 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>09:50–17:00</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Milford Sound</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff。</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr"/>
+          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>峡湾</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>redcliff-official</t>
+          <t>realnz-booking</t>
         </is>
       </c>
     </row>
@@ -8594,32 +8611,28 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>20:45–21:15</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>饭后散步</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
+          <t>redcliff-official</t>
         </is>
       </c>
     </row>
@@ -8630,58 +8643,62 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>20:45–21:15</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
+          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>饭后散步</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>realnz-walk-route</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr">
-        <is>
-          <t>nav08-route</t>
-        </is>
-      </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8690,32 +8707,28 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>12:00–13:00</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Frankton</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>午餐</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr"/>
       <c r="H79" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>nav08-route</t>
         </is>
       </c>
     </row>
@@ -8726,36 +8739,32 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>13:30–15:00</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Kelvin Peninsula Sculpture Trail</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>湖畔雕塑步道</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>起点在Peninsula Road和Grove Lane路口。</t>
-        </is>
-      </c>
+          <t>午餐</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>kelvin-trail-map,kelvin-trail-official</t>
+          <t>frankton-map</t>
         </is>
       </c>
     </row>
@@ -8766,32 +8775,36 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15:30–16:00</t>
+          <t>13:30–15:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>入住Fernhill</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr"/>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>起点在Peninsula Road和Grove Lane路口。</t>
+        </is>
+      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>fernhill-map</t>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
         </is>
       </c>
     </row>
@@ -8802,36 +8815,32 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>傍晚 17:00–19:00</t>
+          <t>15:30–16:00</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>俯瞰皇后镇</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
-        </is>
-      </c>
+          <t>入住Fernhill</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>fernhill-map</t>
         </is>
       </c>
     </row>
@@ -8842,32 +8851,36 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>19:00–20:30</t>
+          <t>傍晚 17:00–19:00</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Blue Kanu</t>
+          <t>Skyline Gondola · Bob’s Peak</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
+          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>晚餐</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr"/>
+          <t>俯瞰皇后镇</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
+        </is>
+      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>blue-kanu-official</t>
+          <t>skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
@@ -8878,32 +8891,32 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>20:40–21:10</t>
+          <t>19:00–20:30</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Earnslaw Park / 湖边</t>
+          <t>Blue Kanu</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>湖边日落</t>
+          <t>晚餐</t>
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
     </row>
@@ -8914,62 +8927,62 @@
         </is>
       </c>
       <c r="B85" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>20:40–21:10</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Frankton / Blue Kanu</t>
+          <t>Earnslaw Park / 湖边</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr"/>
+          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>湖边日落</t>
+        </is>
+      </c>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>earnslaw-park-map</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>湖边公路</t>
-        </is>
-      </c>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>nav09-out-route</t>
-        </is>
-      </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8978,32 +8991,32 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>红船屋</t>
+          <t>湖边公路</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
     </row>
@@ -9014,36 +9027,32 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>湿地步道</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
-        </is>
-      </c>
+          <t>红船屋</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>bennetts-bluff-official</t>
         </is>
       </c>
     </row>
@@ -9054,28 +9063,36 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
     </row>
@@ -9086,36 +9103,28 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>18:00–20:30</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>傍晚湖面倒影</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>moke-lake-map,moke-lake-official</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
     </row>
@@ -9126,32 +9135,36 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>21:00左右</t>
+          <t>18:00–20:30</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>皇后镇招牌汉堡</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr"/>
+          <t>傍晚湖面倒影</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
+        </is>
+      </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
+          <t>moke-lake-map,moke-lake-official</t>
         </is>
       </c>
     </row>
@@ -9162,62 +9175,62 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>21:00左右</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Glenorchy / Fergburger</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr"/>
+          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>皇后镇招牌汉堡</t>
+        </is>
+      </c>
       <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>南岛收车</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>nav10-route</t>
-        </is>
-      </c>
+      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9226,32 +9239,32 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>等飞机</t>
+          <t>南岛收车</t>
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>zqn-map</t>
+          <t>nav10-route</t>
         </is>
       </c>
     </row>
@@ -9262,30 +9275,34 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>航班</t>
+          <t>等飞机</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>zqn-map</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -9294,34 +9311,30 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>飞奥克兰。</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>连住两晚</t>
+          <t>航班</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>akl-intl-map</t>
-        </is>
-      </c>
+      <c r="H96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9330,32 +9343,32 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>18:00–19:30</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
+          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>情人节晚餐</t>
+          <t>连住两晚</t>
         </is>
       </c>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
     </row>
@@ -9366,36 +9379,32 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>19:45–20:45</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Wynyard Quarter / Silo Park</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
+          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>海港日落</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>想换个角度可以上Sky Tower观景台，要另买票，人也多。</t>
-        </is>
-      </c>
+          <t>情人节晚餐</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>viaduct-map</t>
         </is>
       </c>
     </row>
@@ -9406,62 +9415,66 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>19:45–20:45</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Wynyard Quarter / Silo Park</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
+          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>海港日落</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>想换个角度可以上Sky Tower观景台，要另买票，人也多。</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>wynyard-map</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>08:30–09:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Auckland市区出发</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>交通待定</t>
-        </is>
-      </c>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr">
-        <is>
-          <t>nav11-out-route,hobbiton-transfers-official</t>
-        </is>
-      </c>
+      <c r="H100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9470,28 +9483,32 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>12:30–13:00</t>
+          <t>08:30–09:30</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>The Shire’s Rest</t>
+          <t>Auckland市区出发</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr"/>
+          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>交通待定</t>
+        </is>
+      </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>shire-rest-map</t>
+          <t>nav11-out-route,hobbiton-transfers-official</t>
         </is>
       </c>
     </row>
@@ -9502,32 +9519,28 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>13:30前</t>
+          <t>12:30–13:00</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>The Shire’s Rest Ticketing Office</t>
+          <t>The Shire’s Rest</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>在The Shire’s Rest Ticketing Office报到。</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>已订报到</t>
-        </is>
-      </c>
+          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
+          <t>shire-rest-map</t>
         </is>
       </c>
     </row>
@@ -9538,30 +9551,34 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>13:50–约16:20</t>
+          <t>13:30前</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>The Shire’s Rest Ticketing Office</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
+          <t>在The Shire’s Rest Ticketing Office报到。</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>中文导览</t>
+          <t>已订报到</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>hobbiton-booking</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9570,34 +9587,30 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16:30–17:00左右返程</t>
+          <t>13:50–约16:20</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Hobbiton → Auckland</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
+          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>晚间回城</t>
+          <t>中文导览</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
+      <c r="H104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9606,36 +9619,32 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>19:45–20:40（可选，租车时）</t>
+          <t>16:30–17:00左右返程</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Mt Eden · Maungawhau</t>
+          <t>Hobbiton → Auckland</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>租车且19:30前回到奥克兰的话，顺路去Mt Eden：车停山脚，走15–20分钟上山顶，20:18看整座城的日落，下山再吃晚饭、还车。</t>
+          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>城市日落</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>山顶不能开车上去；坐大巴或接驳就跳过。</t>
-        </is>
-      </c>
+          <t>晚间回城</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
       <c r="H105" t="inlineStr">
         <is>
-          <t>mt-eden-map</t>
+          <t>nav11-back-route</t>
         </is>
       </c>
     </row>
@@ -9646,49 +9655,61 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>19:45–20:40（可选，租车时）</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Shire’s Rest / Auckland</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+          <t>租车且19:30前回到奥克兰的话，顺路去Mt Eden：车停山脚，走15–20分钟上山顶，20:18看整座城的日落，下山再吃晚饭、还车。</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>城市日落</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>山顶不能开车上去；坐大巴或接驳就跳过。</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>mt-eden-map</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>Shire’s Rest / Auckland</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
+          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
         </is>
       </c>
       <c r="F107" t="inlineStr"/>
@@ -9702,34 +9723,26 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>美术馆</t>
-        </is>
-      </c>
+          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>art-gallery-map,art-gallery-official</t>
-        </is>
-      </c>
+      <c r="H108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9738,32 +9751,32 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>完整午餐</t>
+          <t>美术馆</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>amano-map,amano-official</t>
+          <t>art-gallery-map,art-gallery-official</t>
         </is>
       </c>
     </row>
@@ -9774,26 +9787,34 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr"/>
+          <t>Britomart午餐，首选Amano，待预约。</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>完整午餐</t>
+        </is>
+      </c>
       <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>amano-map,amano-official</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9802,34 +9823,26 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>Britomart</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>夜航回国</t>
-        </is>
-      </c>
+          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
+      <c r="H111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9838,56 +9851,60 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>晚上</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>Auckland Airport</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr"/>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>夜航回国</t>
+        </is>
+      </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>akl-intl-map,akl-departure-official</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>市区 / Amano</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>转机</t>
-        </is>
-      </c>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr"/>
     </row>
@@ -9898,34 +9915,30 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>09:10–11:10</t>
+          <t>05:00–09:10</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>CZ3803 → 杭州萧山T4</t>
+          <t>广州白云T2</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>飞回杭州，取行李回家。</t>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>到家</t>
+          <t>转机</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>hgh-airport-map</t>
-        </is>
-      </c>
+      <c r="H114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9934,30 +9947,66 @@
         </is>
       </c>
       <c r="B115" t="n">
+        <v>20</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>09:10–11:10</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>CZ3803 → 杭州萧山T4</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
         <v>90</v>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>饮食</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D116" t="inlineStr">
         <is>
           <t>落地后</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E116" t="inlineStr">
         <is>
           <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F116" t="inlineStr">
         <is>
           <t>按航班实际到达时间</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12388,17 +12437,17 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>尽早</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>订 Te Anau 萤火虫洞夜游（2/10 19:00）</t>
+          <t>订 Te Anau 萤火虫洞 2/10 17:45 场</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>RealNZ 坐船过湖进洞，约 2 小时 15 分，每人约 NZ$154；洞内 8–12°C 要带外套，洞里不能拍照。场次以官网为准；第二天要去 Milford，累了就不订。</t>
+          <t>RealNZ 坐船过湖进洞，约 2 小时 15 分，约 20:00 回来，每人约 NZ$154；先在官网确认这天有 17:45 场。同时订 20:15 的晚饭（不少餐厅 21:00 前后停止点餐）。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: swap Te Anau glowworms and Hobbiton tour for a Waitomo + Hobbiton day tour
- 2/15: Klook Hobbiton + Waitomo join-in tour, 06:00–17:30 from Auckland; drive guide 11 removed
- 2/10: glowworm tour removed, back to early dinner and lakefront sunset
- Checklist: drop glowworm and Hobbiton transport, add pickup check (26 → 25)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>每天保留一个主要体验：悉尼Bondi海岸与城市漫步、湖区公路与星空、Mt Cook徒步、Wānaka的一顿晚餐、Milford峡湾、Glenorchy公路、Hobbiton中文导览。</t>
+          <t>每天保留一个主要体验：悉尼Bondi海岸与城市漫步、湖区公路与星空、Mt Cook徒步、Wānaka的一顿晚餐、Milford峡湾、Glenorchy公路、Waitomo萤火虫洞和Hobbiton。</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1009,12 +1009,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hobbiton Mandarin Language Tour 13:50（已订）</t>
+          <t>Hobbiton + Waitomo萤火虫洞一日团（Klook，已订）</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1024,14 +1024,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand</t>
+          <t>https://www.klook.cn/zh-CN/activity/23913-hobbiton-waitomo-caves-join-in-tour-auckland/</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>13:30前在Ticketing Office报到</t>
+          <t>06:00出发，约17:30回到Auckland</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Shire’s Rest报到点</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2082,41 +2082,41 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>hobbiton-faq-official</t>
+          <t>art-gallery-map</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Hobbiton官方FAQ</t>
+          <t>Auckland Art Gallery Toi o Tāmaki</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.hobbitontours.com/plan-visit/frequently-asked-questions/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Art+Gallery+Toi+o+Tamaki%2C+1+Kitchener+Street%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>hobbiton-transfers-official</t>
+          <t>art-gallery-official</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Hobbiton官方交通伙伴</t>
+          <t>Auckland Art Gallery参观信息</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.hobbitontours.com/plan-visit/transfers/</t>
+          <t>https://www.aucklandartgallery.com/visit/plan-your-visit</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2140,22 +2140,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>art-gallery-map</t>
+          <t>amano-map</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki</t>
+          <t>Amano</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Art+Gallery+Toi+o+Tamaki%2C+1+Kitchener+Street%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Amano%2C+68+Tyler+Street%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2169,22 +2169,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>art-gallery-official</t>
+          <t>amano-official</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery参观信息</t>
+          <t>Amano预约</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.aucklandartgallery.com/visit/plan-your-visit</t>
+          <t>https://savor.co.nz/amano</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2198,22 +2198,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>amano-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Amano</t>
+          <t>Auckland Airport国际航站楼</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Amano%2C+68+Tyler+Street%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Airport+International+Terminal%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2227,41 +2227,41 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>amano-official</t>
+          <t>akl-departure-official</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Amano预约</t>
+          <t>Auckland机场出发指南</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://savor.co.nz/amano</t>
+          <t>https://www.aucklandairport.co.nz/information/departure-information</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>机场官网</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>hgh-airport-map</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Auckland Airport国际航站楼</t>
+          <t>杭州萧山国际机场</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Airport+International+Terminal%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hangzhou+Xiaoshan+International+Airport</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2285,41 +2285,41 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>akl-departure-official</t>
+          <t>syd-t1-map</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Auckland机场出发指南</t>
+          <t>悉尼机场国际航站楼 T1</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.aucklandairport.co.nz/information/departure-information</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Sydney+Airport+International+Terminal+T1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>机场官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>hgh-airport-map</t>
+          <t>darling-harbour-map</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>杭州萧山国际机场</t>
+          <t>Darling Harbour</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hangzhou+Xiaoshan+International+Airport</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Darling+Harbour%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2343,99 +2343,99 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>syd-t1-map</t>
+          <t>rental-car-booking</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>悉尼机场国际航站楼 T1</t>
+          <t>南岛租车：起亚 Seltos 或同级（已订）</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Sydney+Airport+International+Terminal+T1</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Christchurch+Airport%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>2/5 10:00 基督城机场取，2/14 10:00 皇后镇机场还</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>darling-harbour-map</t>
+          <t>mackenzie-parking-official</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Darling Harbour</t>
+          <t>Mackenzie停车规则</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Darling+Harbour%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://www.mackenzie.govt.nz/services/roading-and-transport/parking</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Mackenzie District Council</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>rental-car-booking</t>
+          <t>nzta-journey-official</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>南岛租车：起亚 Seltos 或同级（已订）</t>
+          <t>NZTA路况</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>booking</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Christchurch+Airport%2C+New+Zealand</t>
+          <t>https://www.journeys.nzta.govt.nz/journey-planner</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2/5 10:00 基督城机场取，2/14 10:00 皇后镇机场还</t>
+          <t>NZTA</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>mackenzie-parking-official</t>
+          <t>nzta-five-rivers-official</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Mackenzie停车规则</t>
+          <t>NZTA Five Rivers路口资料</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2445,26 +2445,26 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.mackenzie.govt.nz/services/roading-and-transport/parking</t>
+          <t>https://www.nzta.govt.nz/driving-skills/safe-driving-habits/following-speed-limits/state-highway-speed-management/speed-limit-reviews-under-the-2024-rule/targeted-speed-limit-reviews-canterbury-west-coast-southland/sh6-five-riverssh97-isz-approved-speed-limit-change-100kmh-100-60kmh-variable</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Mackenzie District Council</t>
+          <t>NZTA</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>nzta-journey-official</t>
+          <t>govt-holidays-official</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NZTA路况</t>
+          <t>新西兰政府假期表</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2474,84 +2474,84 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.journeys.nzta.govt.nz/journey-planner</t>
+          <t>https://www.govt.nz/browse/work/public-holidays-and-work/public-holidays-and-anniversary-dates/</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NZTA</t>
+          <t>govt.nz</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>nzta-five-rivers-official</t>
+          <t>chc-airport-route</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NZTA Five Rivers路口资料</t>
+          <t>基督城机场至住宿参考路线</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.nzta.govt.nz/driving-skills/safe-driving-habits/following-speed-limits/state-highway-speed-management/speed-limit-reviews-under-the-2024-rule/targeted-speed-limit-reviews-canterbury-west-coast-southland/sh6-five-riverssh97-isz-approved-speed-limit-change-100kmh-100-60kmh-variable</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=175+Riccarton+Road%2C+Riccarton%2C+Christchurch%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>NZTA</t>
+          <t>导航01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>govt-holidays-official</t>
+          <t>nav02-a-route</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>新西兰政府假期表</t>
+          <t>前半程至Tekapo</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.govt.nz/browse/work/public-holidays-and-work/public-holidays-and-anniversary-dates/</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Ashburton%2C+New+Zealand%7CGeraldine%2C+Canterbury%2C+New+Zealand%7CFairlie+Bakehouse%2C+Fairlie%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>govt.nz</t>
+          <t>导航02</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>chc-airport-route</t>
+          <t>nav02-b-route</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>基督城机场至住宿参考路线</t>
+          <t>后半程至Twizel</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2561,26 +2561,26 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=175+Riccarton+Road%2C+Riccarton%2C+Christchurch%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Pukaki+Visitor+Centre%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>导航01</t>
+          <t>导航02</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>nav02-a-route</t>
+          <t>white-horse-hill-route</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>前半程至Tekapo</t>
+          <t>先到Hooker起点停车场</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2590,26 +2590,26 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Ashburton%2C+New+Zealand%7CGeraldine%2C+Canterbury%2C+New+Zealand%7CFairlie+Bakehouse%2C+Fairlie%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>导航02</t>
+          <t>导航03</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>nav02-b-route</t>
+          <t>peters-lookout-route</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>后半程至Twizel</t>
+          <t>返程经Peter’s Lookout</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2619,26 +2619,26 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Pukaki+Visitor+Centre%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Peter%27s+Lookout%2C+Lake+Pukaki%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>导航02</t>
+          <t>导航03</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>white-horse-hill-route</t>
+          <t>tasman-route</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>先到Hooker起点停车场</t>
+          <t>可选Tasman停车场</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Tasman+Valley+Car+Park%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -2662,12 +2662,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>peters-lookout-route</t>
+          <t>lake-loop-route</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>返程经Peter’s Lookout</t>
+          <t>湖区午餐小环线</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2677,26 +2677,26 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Peter%27s+Lookout%2C+Lake+Pukaki%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Ruataniwha+Reserve%2C+Twizel%2C+New+Zealand%7CHigh+Country+Salmon%2C+2602+Twizel-Omarama+Highway%2C+Twizel%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>导航03</t>
+          <t>导航04</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>tasman-route</t>
+          <t>pukaki-visitor-route</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>可选Tasman停车场</t>
+          <t>可选Pukaki南岸</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2706,26 +2706,26 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Tasman+Valley+Car+Park%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lake+Pukaki+Visitor+Centre%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>导航03</t>
+          <t>导航04</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>lake-loop-route</t>
+          <t>lindis-pass-route</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>湖区午餐小环线</t>
+          <t>完整山口路线</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2735,26 +2735,26 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Ruataniwha+Reserve%2C+Twizel%2C+New+Zealand%7CHigh+Country+Salmon%2C+2602+Twizel-Omarama+Highway%2C+Twizel%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand%7CLindis+Pass+Lookout%2C+New+Zealand%7CLuggate%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>导航04</t>
+          <t>导航05</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>pukaki-visitor-route</t>
+          <t>nav05-a-route</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>可选Pukaki南岸</t>
+          <t>前半程到Lindis Pass</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2764,26 +2764,26 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lake+Pukaki+Visitor+Centre%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lindis+Pass+Lookout%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>导航04</t>
+          <t>导航05</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>lindis-pass-route</t>
+          <t>nav05-b-route</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>完整山口路线</t>
+          <t>后半程到已订住宿</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand%7CLindis+Pass+Lookout%2C+New+Zealand%7CLuggate%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Lindis+Pass+Lookout%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Luggate%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -2807,12 +2807,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>nav05-a-route</t>
+          <t>mount-iron-route</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>前半程到Lindis Pass</t>
+          <t>去Mount Iron</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2822,26 +2822,26 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lindis+Pass+Lookout%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>导航05</t>
+          <t>导航06</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>nav05-b-route</t>
+          <t>wanaka-lakefront-route</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>后半程到已订住宿</t>
+          <t>去湖滨</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2851,26 +2851,26 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Lindis+Pass+Lookout%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Luggate%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;destination=Wanaka+Lakefront%2C+Ardmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>导航05</t>
+          <t>导航06</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>mount-iron-route</t>
+          <t>kika-route</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>去Mount Iron</t>
+          <t>去Kika晚餐</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Kika%2C+2+Dunmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -2894,12 +2894,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>wanaka-lakefront-route</t>
+          <t>waterfall-creek-route</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>去湖滨</t>
+          <t>平缓备选Waterfall Creek</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;destination=Wanaka+Lakefront%2C+Ardmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Waterfall+Creek+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -2923,12 +2923,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>kika-route</t>
+          <t>nav07-leg1-route</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>去Kika晚餐</t>
+          <t>备选：经Cromwell到Frankton</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2938,26 +2938,26 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Kika%2C+2+Dunmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cromwell+Heritage+Precinct%2C+Cromwell%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>导航06</t>
+          <t>导航07</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>waterfall-creek-route</t>
+          <t>nav07-leg2-route</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>平缓备选Waterfall Creek</t>
+          <t>第二段Frankton到Te Anau</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2967,26 +2967,26 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Waterfall+Creek+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Frankton%2C+Queenstown%2C+New+Zealand&amp;destination=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Kingston%2C+Otago%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CMossburn%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>导航06</t>
+          <t>导航07</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>nav07-leg1-route</t>
+          <t>crown-range-route</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>备选：经Cromwell到Frankton</t>
+          <t>第一段经Crown Range、Arrowtown到Frankton</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cromwell+Heritage+Precinct%2C+Cromwell%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cardrona+Hotel%2C+Cardrona%2C+New+Zealand%7CCrown+Range+Summit%2C+New+Zealand%7CArrowtown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -3010,12 +3010,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>nav07-leg2-route</t>
+          <t>arrowtown-map</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>第二段Frankton到Te Anau</t>
+          <t>Arrowtown</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3025,26 +3025,26 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Frankton%2C+Queenstown%2C+New+Zealand&amp;destination=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Kingston%2C+Otago%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CMossburn%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Arrowtown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>导航07</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>crown-range-route</t>
+          <t>diamond-lake-map</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>第一段经Crown Range、Arrowtown到Frankton</t>
+          <t>Diamond Lake 停车场</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3054,55 +3054,55 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cardrona+Hotel%2C+Cardrona%2C+New+Zealand%7CCrown+Range+Summit%2C+New+Zealand%7CArrowtown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Diamond+Lake+Track+Car+Park%2C+Wanaka-Mount+Aspiring+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>导航07</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>arrowtown-map</t>
+          <t>diamond-lake-official</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Arrowtown</t>
+          <t>Lake Wānaka Lookout Track</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Arrowtown%2C+New+Zealand</t>
+          <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/otago/places/diamond-lake-and-hospital-flat/things-to-do/lake-wanaka-lookout-track</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>diamond-lake-map</t>
+          <t>frankton-map</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Diamond Lake 停车场</t>
+          <t>Frankton / Remarkables Park</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Diamond+Lake+Track+Car+Park%2C+Wanaka-Mount+Aspiring+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Remarkables+Park%2C+Frankton%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3126,70 +3126,70 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>diamond-lake-official</t>
+          <t>kelvin-trail-map</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Lake Wānaka Lookout Track</t>
+          <t>Kelvin Heights 雕塑环线起点</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/otago/places/diamond-lake-and-hospital-flat/things-to-do/lake-wanaka-lookout-track</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Peninsula+Road+and+Grove+Lane%2C+Kelvin+Heights%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>kelvin-trail-official</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Frankton / Remarkables Park</t>
+          <t>Kelvin Heights Peninsula Trail</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Remarkables+Park%2C+Frankton%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.queenstownnz.co.nz/listing/kelvin-heights-peninsula-trail/9101/</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Queenstown NZ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>kelvin-trail-map</t>
+          <t>moke-lake-map</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Kelvin Heights 雕塑环线起点</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Peninsula+Road+and+Grove+Lane%2C+Kelvin+Heights%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Moke+Lake%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3213,12 +3213,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>kelvin-trail-official</t>
+          <t>moke-lake-official</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Kelvin Heights Peninsula Trail</t>
+          <t>Moke Lake Loop Track</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3228,26 +3228,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://www.queenstownnz.co.nz/listing/kelvin-heights-peninsula-trail/9101/</t>
+          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/otago/places/queenstown-area/things-to-do/moke-lake-loop-track</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Queenstown NZ</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>moke-lake-map</t>
+          <t>barangaroo-map</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Barangaroo Reserve</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Moke+Lake%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Barangaroo+Reserve%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3271,70 +3271,70 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>moke-lake-official</t>
+          <t>mrs-macquarie-map</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Moke Lake Loop Track</t>
+          <t>Mrs Macquarie's Chair</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/otago/places/queenstown-area/things-to-do/moke-lake-loop-track</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Mrs+Macquarie%27s+Chair%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>barangaroo-map</t>
+          <t>manly-ferry-official</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Barangaroo Reserve</t>
+          <t>悉尼渡轮（F1 Manly线）</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Barangaroo+Reserve%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://transportnsw.info/travel-info/ways-to-get-around/ferry</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Transport for NSW</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>mrs-macquarie-map</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Mrs Macquarie's Chair</t>
+          <t>Earnslaw Park</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Mrs+Macquarie%27s+Chair%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3358,70 +3358,70 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>manly-ferry-official</t>
+          <t>waitomo-map</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>悉尼渡轮（F1 Manly线）</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://transportnsw.info/travel-info/ways-to-get-around/ferry</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Transport for NSW</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>glowworm-official</t>
+          <t>viaduct-map</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Te Anau Glowworm Caves（RealNZ）</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://www.realnz.com/en/experiences/glowworm-caves/te-anau-glowworm-caves/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>RealNZ</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>wynyard-map</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Earnslaw Park</t>
+          <t>Silo Park / Wynyard Quarter</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -3445,12 +3445,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>mt-eden-map</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Maungawhau+Mount+Eden+Summit%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -3474,22 +3474,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>fergburger-map</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Silo Park / Wynyard Quarter</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -3503,51 +3503,51 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>mt-eden-map</t>
+          <t>fergburger-official</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Mt Eden · Maungawhau</t>
+          <t>Fergburger官网</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Maungawhau+Mount+Eden+Summit%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.fergburger.com/</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>fergburger-map</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -3561,22 +3561,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>fergburger-official</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Fergburger官网</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.fergburger.com/</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -3590,12 +3590,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -3619,41 +3619,41 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>完整路线到Fernhill</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3663,26 +3663,26 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>导航08</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>去程经Bennetts Bluff</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3692,26 +3692,26 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>导航09</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Glenorchy回住宿</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3721,26 +3721,26 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>导航09</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>nav10-route</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>机场方向参考路线</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3750,159 +3750,14 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>导航09</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>nav09-back-route</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Glenorchy回住宿</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>导航09</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>nav10-route</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>机场方向参考路线</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr">
-        <is>
           <t>导航10</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>nav11-out-route</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>市区参考起点经Matamata到现场</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Britomart%2C+Auckland%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>导航11</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>nav11-matamata-route</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Matamata休息后到现场</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>导航11</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>现场回Auckland市中心参考</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;destination=Britomart%2C+Auckland%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>导航11</t>
         </is>
       </c>
     </row>
@@ -4039,7 +3894,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>南岛还车飞Auckland，Hobbiton中文团，城市日后夜航回国。</t>
+          <t>南岛还车飞Auckland，萤火虫洞＋霍比屯一日团，城市日后夜航回国。</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5055,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>09:00左右出发；17:15到RealNZ报到萤火虫团</t>
+          <t>09:00左右出发；10:00前退房</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -5227,8 +5082,7 @@
         <is>
           <t>住宿｜Private Ensuite in the Heart of Te Anau，3 Thomson Place；15:00后入住。
 驾驶安排｜纯驾驶约3.5–4.5小时，加Arrowtown午餐和停靠留5–6小时；抵达时间随休息调整。
-坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。
-傍晚｜17:45 萤火虫洞团。Arrowtown 控制在 90 分钟内，15:00–16:30 到 Te Anau；改走 Cromwell 多 20–30 分钟也赶得上，最晚 16:30 前到住处。</t>
+坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。</t>
         </is>
       </c>
     </row>
@@ -5681,7 +5535,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Auckland ↔ Hobbiton</t>
+          <t>Auckland ↔ Waitomo ↔ Hobbiton</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -5697,12 +5551,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Hobbiton中文团，一天往返</t>
+          <t>Waitomo萤火虫洞 + Hobbiton一日团</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>保留已付13:50普通话导览，把往返时间留宽。</t>
+          <t>跟团一天：上午坐船看萤火虫，下午走进霍比屯。</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -5717,24 +5571,24 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Waikato约15–26°C，午后日晒强，偶有阵雨。</t>
+          <t>Waikato约15–26°C，午后日晒强，偶有阵雨；洞里常年凉。</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>防晒、帽子、好走的鞋；车上备一件薄外套。</t>
+          <t>防晒、帽子、好走的鞋；带一件外套进洞。</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>交通待定：一日租车自驾，或大巴 / 接驳</t>
+          <t>跟团大巴（Klook，已订）· 06:00出发，约17:30回到Auckland</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>13:30前到The Shire’s Rest报到</t>
+          <t>06:00出发；上车地点以确认单为准</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -5744,26 +5598,21 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>shire-rest-map</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
+          <t>waitomo-hobbiton-booking</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>住宿｜回同一家Auckland住宿，第二晚。
-交通待定｜还没决定租车还是公共交通。现票只含Shire’s Rest至片场巴士，不含Auckland往返。
-方案A 租车｜一日租车自驾，往返纯驾驶约4.5–5小时，须支持晚间还车；按下方导航11执行。
-方案B 大巴 / 接驳｜Auckland没有直达Shire’s Rest的公共交通：可坐长途大巴到Matamata再打车到501 Buckland Road，或订接受自购票的纯接送。选这个方案前确认班次能13:30前送到Shire’s Rest、16:20后能接回Auckland。
-回程｜Hobbiton约16:20结束，随后返程，约19:00–20:00回到Auckland。</t>
+跟团｜Klook Hobbiton + Waitomo 一日团：先去Waitomo萤火虫洞（洞里约1小时，最后坐小船看萤火虫，洞内讲解是英文），再去Hobbiton片场；车上有中文讲解。06:00出发，约17:30回到Auckland。
+以确认单为准｜上车地点（集合点还是酒店接送）、午餐是否包含，出发前一周在Klook确认。
+准备｜前一晚早睡；早餐带上车；洞里凉、不能拍照，带外套；车程单程约2–2.5小时，带水和零食。</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8331,34 +8180,22 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17:15–17:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau镇上</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>开几分钟到85 Lakefront Drive报到，就是明天Milford的集合点。</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>报到</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>报到时间以确认单为准。</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>realnz-map</t>
-        </is>
-      </c>
+          <t>早点吃晚饭。</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8367,36 +8204,36 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17:45–20:00</t>
+          <t>20:40–21:15</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Te Anau萤火虫洞</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>RealNZ萤火虫洞团：坐船过湖，步行进洞，再坐小船看萤火虫，约2小时15分。</t>
+          <t>沿Lakefront Drive散步，湖岸朝西，看21:09的日落落在湖上；离住处几分钟，看完回去早点睡。</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>萤火虫</t>
+          <t>湖上日落</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>洞内8–12°C，带外套；洞里不能拍照。</t>
+          <t>明早09:15去Milford报到。</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>realnz-map,glowworm-official</t>
+          <t>realnz-walk-route</t>
         </is>
       </c>
     </row>
@@ -8407,98 +8244,94 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Te Anau镇上</t>
+          <t>Frankton / Kingston / Te Anau</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>回来直接吃晚饭；不少餐厅厨房21:00前后停止点餐，要提前订，选离湖边近的。</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>晚饭</t>
-        </is>
-      </c>
+          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：17:30在Te Anau镇上</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>21:00–21:15</t>
+          <t>08:00左右</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>饭后沿Lakefront Drive走走，湖岸朝西，看21:09的日落，然后回住宿早点睡。</t>
+          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>湖上日落</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>明早09:15去Milford报到。</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>realnz-walk-route</t>
-        </is>
-      </c>
+          <t>装备检查</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:15左右到，09:30前完成报到</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Frankton / Kingston / Te Anau</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：20:15在Te Anau镇上（要订）</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>已订集合</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>realnz-map,realnz-walk-route</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8507,30 +8340,34 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>08:00左右</t>
+          <t>09:50–17:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Milford Sound</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>装备检查</t>
+          <t>峡湾</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>realnz-booking</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8539,32 +8376,28 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>09:15左右到，09:30前完成报到</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>已订集合</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>realnz-map,realnz-walk-route</t>
+          <t>redcliff-official</t>
         </is>
       </c>
     </row>
@@ -8575,32 +8408,32 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>09:50–17:00</t>
+          <t>20:45–21:15</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Milford Sound</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>峡湾</t>
+          <t>饭后散步</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>realnz-booking</t>
+          <t>realnz-walk-route</t>
         </is>
       </c>
     </row>
@@ -8611,94 +8444,94 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>redcliff-official</t>
-        </is>
-      </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>20:45–21:15</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>饭后散步</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
+          <t>nav08-route</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>frankton-map</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8707,28 +8540,36 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>13:30–15:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>起点在Peninsula Road和Grove Lane路口。</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
         </is>
       </c>
     </row>
@@ -8739,32 +8580,32 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>12:00–13:00</t>
+          <t>15:30–16:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Frankton</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>午餐</t>
+          <t>入住Fernhill</t>
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>fernhill-map</t>
         </is>
       </c>
     </row>
@@ -8775,36 +8616,36 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>13:30–15:00</t>
+          <t>傍晚 17:00–19:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Kelvin Peninsula Sculpture Trail</t>
+          <t>Skyline Gondola · Bob’s Peak</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>湖畔雕塑步道</t>
+          <t>俯瞰皇后镇</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>起点在Peninsula Road和Grove Lane路口。</t>
+          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>kelvin-trail-map,kelvin-trail-official</t>
+          <t>skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
@@ -8815,32 +8656,32 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15:30–16:00</t>
+          <t>19:00–20:30</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>Blue Kanu</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
+          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>入住Fernhill</t>
+          <t>晚餐</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fernhill-map</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
     </row>
@@ -8851,36 +8692,32 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>傍晚 17:00–19:00</t>
+          <t>20:40–21:10</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>Earnslaw Park / 湖边</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
+          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>俯瞰皇后镇</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
-        </is>
-      </c>
+          <t>湖边日落</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
     </row>
@@ -8891,98 +8728,98 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>19:00–20:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Blue Kanu</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>晚餐</t>
-        </is>
-      </c>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>blue-kanu-official</t>
-        </is>
-      </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>20:40–21:10</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Earnslaw Park / 湖边</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>湖边日落</t>
+          <t>湖边公路</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Frankton / Blue Kanu</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr"/>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>红船屋</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>bennetts-bluff-official</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8991,32 +8828,36 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>湖边公路</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr"/>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
     </row>
@@ -9027,32 +8868,28 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>红船屋</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
     </row>
@@ -9063,36 +8900,36 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>18:00–20:30</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>湿地步道</t>
+          <t>傍晚湖面倒影</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
+          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>moke-lake-map,moke-lake-official</t>
         </is>
       </c>
     </row>
@@ -9103,28 +8940,32 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>21:00左右</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr"/>
+          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>皇后镇招牌汉堡</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
         </is>
       </c>
     </row>
@@ -9135,102 +8976,98 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>18:00–20:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>傍晚湖面倒影</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>moke-lake-map,moke-lake-official</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>21:00左右</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>皇后镇招牌汉堡</t>
+          <t>南岛收车</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
+          <t>nav10-route</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Glenorchy / Fergburger</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr"/>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>等飞机</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>zqn-map</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9239,34 +9076,30 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+          <t>飞奥克兰。</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>南岛收车</t>
+          <t>航班</t>
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>nav10-route</t>
-        </is>
-      </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9275,32 +9108,32 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>等飞机</t>
+          <t>连住两晚</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>zqn-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
     </row>
@@ -9311,30 +9144,34 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
+          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>航班</t>
+          <t>情人节晚餐</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>viaduct-map</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9343,32 +9180,36 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>19:45–20:45</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>Wynyard Quarter / Silo Park</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>连住两晚</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
+          <t>海港日落</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>明早06:00出发，看完日落就回酒店早睡。</t>
+        </is>
+      </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>wynyard-map</t>
         </is>
       </c>
     </row>
@@ -9379,102 +9220,102 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>18:00–19:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>情人节晚餐</t>
-        </is>
-      </c>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>viaduct-map</t>
-        </is>
-      </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>19:45–20:45</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Wynyard Quarter / Silo Park</t>
+          <t>Auckland出发</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
+          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>海港日落</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>想换个角度可以上Sky Tower观景台，要另买票，人也多。</t>
-        </is>
-      </c>
+          <t>早起出发</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
+          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>萤火虫洞</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>洞里凉、不能拍照；讲解是英文。</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>waitomo-map</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9483,32 +9324,32 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>08:30–09:30</t>
+          <t>中午–下午</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Auckland市区出发</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
+          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>交通待定</t>
+          <t>霍比屯</t>
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>nav11-out-route,hobbiton-transfers-official</t>
+          <t>shire-rest-map</t>
         </is>
       </c>
     </row>
@@ -9519,30 +9360,26 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>12:30–13:00</t>
+          <t>约17:30</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>The Shire’s Rest</t>
+          <t>回到Auckland</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
+          <t>回到市区，回酒店歇一会儿。</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>shire-rest-map</t>
-        </is>
-      </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9551,34 +9388,26 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>13:30前</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>The Shire’s Rest Ticketing Office</t>
+          <t>Auckland市中心</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>在The Shire’s Rest Ticketing Office报到。</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>已订报到</t>
-        </is>
-      </c>
+          <t>酒店附近吃晚饭。</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>hobbiton-booking</t>
-        </is>
-      </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9587,30 +9416,38 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>13:50–约16:20</t>
+          <t>19:45–20:40（可选）</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
+          <t>打车约15分钟到山脚，走15–20分钟上山顶，20:18看整座城的日落，下山打车回酒店。</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>中文导览</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+          <t>城市日落</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>早起累了就跳过；山顶不能开车上去。</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>mt-eden-map</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9619,102 +9456,90 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16:30–17:00左右返程</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Hobbiton → Auckland</t>
+          <t>车上 / 途中 / Auckland</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>晚间回城</t>
-        </is>
-      </c>
+          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>19:45–20:40（可选，租车时）</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Mt Eden · Maungawhau</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>租车且19:30前回到奥克兰的话，顺路去Mt Eden：车停山脚，走15–20分钟上山顶，20:18看整座城的日落，下山再吃晚饭、还车。</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>城市日落</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>山顶不能开车上去；坐大巴或接驳就跳过。</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>mt-eden-map</t>
-        </is>
-      </c>
+          <t>退房并寄存行李。</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Shire’s Rest / Auckland</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr"/>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>美术馆</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>art-gallery-map,art-gallery-official</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9723,26 +9548,34 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
+          <t>Britomart午餐，首选Amano，待预约。</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>完整午餐</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>amano-map,amano-official</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9751,34 +9584,26 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>Britomart</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>美术馆</t>
-        </is>
-      </c>
+          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>art-gallery-map,art-gallery-official</t>
-        </is>
-      </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9787,32 +9612,32 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>晚上</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>Auckland Airport</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>完整午餐</t>
+          <t>夜航回国</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>amano-map,amano-official</t>
+          <t>akl-intl-map,akl-departure-official</t>
         </is>
       </c>
     </row>
@@ -9823,21 +9648,21 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>市区 / Amano</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -9847,66 +9672,70 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d17</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>05:00–09:10</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>广州白云T2</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>夜航回国</t>
+          <t>转机</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d17</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:10–11:10</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>CZ3803 → 杭州萧山T4</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9915,98 +9744,30 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>落地后</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>转机</t>
+          <t>按航班实际到达时间</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>d17</t>
-        </is>
-      </c>
-      <c r="B115" t="n">
-        <v>20</v>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>09:10–11:10</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>CZ3803 → 杭州萧山T4</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>飞回杭州，取行李回家。</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>到家</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>hgh-airport-map</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>d17</t>
-        </is>
-      </c>
-      <c r="B116" t="n">
-        <v>90</v>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>饮食</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>落地后</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>按航班实际到达时间</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10019,7 +9780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10389,43 +10150,6 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>nav10-route,zqn-map,qt-airport-rental-official</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>d15</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>导航11 · （若租车）Auckland ↔ Hobbiton</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>08:30–09:00提车，09:30左右离开市区；去回各预留约3小时交通窗口含短休息，13:30前报到。</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Auckland市区实际取车点 → SH1南行 → 按当日导航经SH2 / SH27到Matamata → 501 Buckland Road / The Shire’s Rest；返程回实际还车点</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>取还车点尚未确定，地图先以Britomart作CBD参考；实际使用时替换成车行地址。优先支持晚间自助还车的网点；若必须次晨还，另计过夜停车和租期，2/16先还车再城市活动。现有票不含Auckland接送；纯接送只有确认接受自购票、13:30前送达且16:20后接回才可替代本页自驾。</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nav11-out-route,nav11-matamata-route,nav11-back-route,shire-rest-map,hobbiton-faq-official,hobbiton-transfers-official</t>
         </is>
       </c>
     </row>
@@ -10440,7 +10164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11442,131 +11166,6 @@
       <c r="E40" t="inlineStr">
         <is>
           <t>12:30 前办托运，JQ296 13:30 起飞。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>10</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>取车点 → Matamata</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>约2–2.5小时，路况另留量</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>可在Matamata短休息；i-SITE只是途中停靠参考，并非这张票的报到点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>20</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Matamata → The Shire’s Rest</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>约15–25分钟</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>最终目的地501 Buckland Road。乡村道路跟当日导航与标识，不套用旧攻略出口号。</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>30</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>现场停车、午餐、报到</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>约30–60分钟缓冲</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>目标12:30–13:00到；停访客停车区，13:30前到Ticketing Office。</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>40</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>13:50 → 约16:20</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>已订导览约2.5小时</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>乘运营商巴士进出片场，私家车停在Shire’s Rest。</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>50</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>约16:30–17:00 → Auckland</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>约2.5–3小时</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>按19:00–20:00抵城安排；堵车、离场晚时顺延，不在当天衔接国际航班。</t>
         </is>
       </c>
     </row>
@@ -11977,7 +11576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12144,42 +11743,42 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>auckland-hotel</t>
+          <t>tour-0215-pickup</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>尽早</t>
+          <t>出发前一周</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>订奥克兰两晚（2/14–16）</t>
+          <t>确认 2/15 一日团的上车地点</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>同一家连住，选 CBD / Britomart 附近，能在 2/16 退房后寄存行李。</t>
+          <t>06:00 出发：在 Klook 确认单或客服问清是集合点还是酒店接送、午餐包不包含；订好奥克兰酒店后把地址发给他们。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hobbiton-transport</t>
+          <t>auckland-hotel</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -12189,17 +11788,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>定了机票后</t>
+          <t>尽早</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>定 2/15 去 Hobbiton 怎么走</t>
+          <t>订奥克兰两晚（2/14–16）</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>租车自驾（要能晚上还车），或坐大巴 / 接驳（要 13:30 前送到 Shire’s Rest、16:20 后能接回）。</t>
+          <t>同一家连住，选 CBD / Britomart 附近，能在 2/16 退房后寄存行李。</t>
         </is>
       </c>
     </row>
@@ -12423,11 +12022,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>glowworm</t>
+          <t>skyline</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -12437,59 +12036,59 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>尽早</t>
+          <t>可选</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>订 Te Anau 萤火虫洞 2/10 17:45 场</t>
+          <t>买 Skyline 缆车票（2/12）</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>RealNZ 坐船过湖进洞，约 2 小时 15 分，约 20:00 回来，每人约 NZ$154；先在官网确认这天有 17:45 场。同时订 20:15 的晚饭（不少餐厅 21:00 前后停止点餐）。</t>
+          <t>网上或现场都能买。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>skyline</t>
+          <t>milford-terms</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>出发前</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>买 Skyline 缆车票（2/12）</t>
+          <t>查 Milford 订单的天气退改规则</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>网上或现场都能买。</t>
+          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>milford-terms</t>
+          <t>host-notes</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -12499,129 +12098,133 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>出发前</t>
+          <t>入住前</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>查 Milford 订单的天气退改规则</t>
+          <t>拿到三处民宿的入住说明</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
+          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>host-notes</t>
+          <t>pay-fernhill</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>入住前</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>拿到三处民宿的入住说明</t>
+          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
+          <t>Apple Pay 付款。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>pay-hikuwai</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>pay</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-01-26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>pay-teanau</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -12630,68 +12233,68 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>1/28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Te Anau 尾款 NZ$386.40</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>cancel-metropolitan</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -12700,33 +12303,33 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/3 14:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>基督城 Metropolitan 免费取消截止</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
+          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cancel-metropolitan</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -12740,28 +12343,28 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2/3 14:00</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>基督城 Metropolitan 免费取消截止</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cancel-hikuwai</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -12770,17 +12373,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2027-02-03</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2/3 16:00</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -12792,15 +12395,15 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cancel-teanau</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -12810,50 +12413,15 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2/5 15:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Te Anau 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>280</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>
@@ -12951,7 +12519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hobbiton 那天是长日子</t>
+          <t>2/15 要早起</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12966,15 +12534,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>奥克兰到 Shire’s Rest 单程约 175 公里，来回 4.5–5 小时，加上 2.5 小时导览，全天 10 小时左右，前一天还刚飞过来。</t>
+          <t>一日团 06:00 出发、约 17:30 回来，单程车程约 2–2.5 小时，前一天还刚从皇后镇飞过来。</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>租车的话两人轮流开，09:00 出发更从容；坐大巴或接驳就盯紧 13:30 报到和 16:20 结束。两种都建议 2/14 早点睡、午饭在 Shire’s Rest 解决、晚饭订 20:00 以后。</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>2/14 看完日落就回酒店早睡；早餐带上车；回来后晚上不排硬行程，Mt Eden 看日落只在有精神时去。</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>waitomo-hobbiton-booking</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">

</xml_diff>

<commit_message>
content: swap Te Anau glowworms and Hobbiton tour for a Waitomo + Hobbiton day tour (#9)
- 2/15: Klook Hobbiton + Waitomo join-in tour, 06:00–17:30 from Auckland; drive guide 11 removed
- 2/10: glowworm tour removed, back to early dinner and lakefront sunset
- Checklist: drop glowworm and Hobbiton transport, add pickup check (26 → 25)

Co-authored-by: SeanSun <s413286943-cmyk@users.noreply.github.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>每天保留一个主要体验：悉尼Bondi海岸与城市漫步、湖区公路与星空、Mt Cook徒步、Wānaka的一顿晚餐、Milford峡湾、Glenorchy公路、Hobbiton中文导览。</t>
+          <t>每天保留一个主要体验：悉尼Bondi海岸与城市漫步、湖区公路与星空、Mt Cook徒步、Wānaka的一顿晚餐、Milford峡湾、Glenorchy公路、Waitomo萤火虫洞和Hobbiton。</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G115"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1009,12 +1009,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Hobbiton Mandarin Language Tour 13:50（已订）</t>
+          <t>Hobbiton + Waitomo萤火虫洞一日团（Klook，已订）</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1024,14 +1024,14 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand</t>
+          <t>https://www.klook.cn/zh-CN/activity/23913-hobbiton-waitomo-caves-join-in-tour-auckland/</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>13:30前在Ticketing Office报到</t>
+          <t>06:00出发，约17:30回到Auckland</t>
         </is>
       </c>
     </row>
@@ -2058,7 +2058,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>The Shire’s Rest报到点</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2082,41 +2082,41 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>hobbiton-faq-official</t>
+          <t>art-gallery-map</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Hobbiton官方FAQ</t>
+          <t>Auckland Art Gallery Toi o Tāmaki</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://www.hobbitontours.com/plan-visit/frequently-asked-questions/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Art+Gallery+Toi+o+Tamaki%2C+1+Kitchener+Street%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>hobbiton-transfers-official</t>
+          <t>art-gallery-official</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Hobbiton官方交通伙伴</t>
+          <t>Auckland Art Gallery参观信息</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://www.hobbitontours.com/plan-visit/transfers/</t>
+          <t>https://www.aucklandartgallery.com/visit/plan-your-visit</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2140,22 +2140,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>art-gallery-map</t>
+          <t>amano-map</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki</t>
+          <t>Amano</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Art+Gallery+Toi+o+Tamaki%2C+1+Kitchener+Street%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Amano%2C+68+Tyler+Street%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2169,22 +2169,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>art-gallery-official</t>
+          <t>amano-official</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery参观信息</t>
+          <t>Amano预约</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://www.aucklandartgallery.com/visit/plan-your-visit</t>
+          <t>https://savor.co.nz/amano</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2198,22 +2198,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>amano-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Amano</t>
+          <t>Auckland Airport国际航站楼</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Amano%2C+68+Tyler+Street%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Airport+International+Terminal%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2227,41 +2227,41 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>amano-official</t>
+          <t>akl-departure-official</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Amano预约</t>
+          <t>Auckland机场出发指南</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://savor.co.nz/amano</t>
+          <t>https://www.aucklandairport.co.nz/information/departure-information</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>机场官网</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>hgh-airport-map</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Auckland Airport国际航站楼</t>
+          <t>杭州萧山国际机场</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Auckland+Airport+International+Terminal%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Hangzhou+Xiaoshan+International+Airport</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2285,41 +2285,41 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>akl-departure-official</t>
+          <t>syd-t1-map</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Auckland机场出发指南</t>
+          <t>悉尼机场国际航站楼 T1</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://www.aucklandairport.co.nz/information/departure-information</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Sydney+Airport+International+Terminal+T1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>机场官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>hgh-airport-map</t>
+          <t>darling-harbour-map</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>杭州萧山国际机场</t>
+          <t>Darling Harbour</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Hangzhou+Xiaoshan+International+Airport</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Darling+Harbour%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2343,99 +2343,99 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>syd-t1-map</t>
+          <t>rental-car-booking</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>悉尼机场国际航站楼 T1</t>
+          <t>南岛租车：起亚 Seltos 或同级（已订）</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Sydney+Airport+International+Terminal+T1</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Christchurch+Airport%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>2/5 10:00 基督城机场取，2/14 10:00 皇后镇机场还</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>darling-harbour-map</t>
+          <t>mackenzie-parking-official</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Darling Harbour</t>
+          <t>Mackenzie停车规则</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Darling+Harbour%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://www.mackenzie.govt.nz/services/roading-and-transport/parking</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Mackenzie District Council</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>rental-car-booking</t>
+          <t>nzta-journey-official</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>南岛租车：起亚 Seltos 或同级（已订）</t>
+          <t>NZTA路况</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>booking</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Christchurch+Airport%2C+New+Zealand</t>
+          <t>https://www.journeys.nzta.govt.nz/journey-planner</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2/5 10:00 基督城机场取，2/14 10:00 皇后镇机场还</t>
+          <t>NZTA</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>mackenzie-parking-official</t>
+          <t>nzta-five-rivers-official</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Mackenzie停车规则</t>
+          <t>NZTA Five Rivers路口资料</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2445,26 +2445,26 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://www.mackenzie.govt.nz/services/roading-and-transport/parking</t>
+          <t>https://www.nzta.govt.nz/driving-skills/safe-driving-habits/following-speed-limits/state-highway-speed-management/speed-limit-reviews-under-the-2024-rule/targeted-speed-limit-reviews-canterbury-west-coast-southland/sh6-five-riverssh97-isz-approved-speed-limit-change-100kmh-100-60kmh-variable</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Mackenzie District Council</t>
+          <t>NZTA</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>nzta-journey-official</t>
+          <t>govt-holidays-official</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NZTA路况</t>
+          <t>新西兰政府假期表</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2474,84 +2474,84 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://www.journeys.nzta.govt.nz/journey-planner</t>
+          <t>https://www.govt.nz/browse/work/public-holidays-and-work/public-holidays-and-anniversary-dates/</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
-          <t>NZTA</t>
+          <t>govt.nz</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>nzta-five-rivers-official</t>
+          <t>chc-airport-route</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NZTA Five Rivers路口资料</t>
+          <t>基督城机场至住宿参考路线</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://www.nzta.govt.nz/driving-skills/safe-driving-habits/following-speed-limits/state-highway-speed-management/speed-limit-reviews-under-the-2024-rule/targeted-speed-limit-reviews-canterbury-west-coast-southland/sh6-five-riverssh97-isz-approved-speed-limit-change-100kmh-100-60kmh-variable</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=175+Riccarton+Road%2C+Riccarton%2C+Christchurch%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
-          <t>NZTA</t>
+          <t>导航01</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>govt-holidays-official</t>
+          <t>nav02-a-route</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>新西兰政府假期表</t>
+          <t>前半程至Tekapo</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://www.govt.nz/browse/work/public-holidays-and-work/public-holidays-and-anniversary-dates/</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Ashburton%2C+New+Zealand%7CGeraldine%2C+Canterbury%2C+New+Zealand%7CFairlie+Bakehouse%2C+Fairlie%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
-          <t>govt.nz</t>
+          <t>导航02</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>chc-airport-route</t>
+          <t>nav02-b-route</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>基督城机场至住宿参考路线</t>
+          <t>后半程至Twizel</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2561,26 +2561,26 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=175+Riccarton+Road%2C+Riccarton%2C+Christchurch%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Pukaki+Visitor+Centre%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
-          <t>导航01</t>
+          <t>导航02</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>nav02-a-route</t>
+          <t>white-horse-hill-route</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>前半程至Tekapo</t>
+          <t>先到Hooker起点停车场</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2590,26 +2590,26 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Christchurch+Airport%2C+New+Zealand&amp;destination=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Ashburton%2C+New+Zealand%7CGeraldine%2C+Canterbury%2C+New+Zealand%7CFairlie+Bakehouse%2C+Fairlie%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>导航02</t>
+          <t>导航03</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>nav02-b-route</t>
+          <t>peters-lookout-route</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>后半程至Twizel</t>
+          <t>返程经Peter’s Lookout</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2619,26 +2619,26 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Church+of+the+Good+Shepherd%2C+Pioneer+Drive%2C+Lake+Tekapo%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Pukaki+Visitor+Centre%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Peter%27s+Lookout%2C+Lake+Pukaki%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>导航02</t>
+          <t>导航03</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>white-horse-hill-route</t>
+          <t>tasman-route</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>先到Hooker起点停车场</t>
+          <t>可选Tasman停车场</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Tasman+Valley+Car+Park%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -2662,12 +2662,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>peters-lookout-route</t>
+          <t>lake-loop-route</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>返程经Peter’s Lookout</t>
+          <t>湖区午餐小环线</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2677,26 +2677,26 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Peter%27s+Lookout%2C+Lake+Pukaki%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Ruataniwha+Reserve%2C+Twizel%2C+New+Zealand%7CHigh+Country+Salmon%2C+2602+Twizel-Omarama+Highway%2C+Twizel%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>导航03</t>
+          <t>导航04</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>tasman-route</t>
+          <t>pukaki-visitor-route</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>可选Tasman停车场</t>
+          <t>可选Pukaki南岸</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2706,26 +2706,26 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=White+Horse+Hill+Car+Park%2C+Hooker+Valley+Road%2C+New+Zealand&amp;destination=Tasman+Valley+Car+Park%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lake+Pukaki+Visitor+Centre%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>导航03</t>
+          <t>导航04</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>lake-loop-route</t>
+          <t>lindis-pass-route</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>湖区午餐小环线</t>
+          <t>完整山口路线</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2735,26 +2735,26 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Lake+Ruataniwha+Reserve%2C+Twizel%2C+New+Zealand%7CHigh+Country+Salmon%2C+2602+Twizel-Omarama+Highway%2C+Twizel%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand%7CLindis+Pass+Lookout%2C+New+Zealand%7CLuggate%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>导航04</t>
+          <t>导航05</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>pukaki-visitor-route</t>
+          <t>nav05-a-route</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>可选Pukaki南岸</t>
+          <t>前半程到Lindis Pass</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2764,26 +2764,26 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lake+Pukaki+Visitor+Centre%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lindis+Pass+Lookout%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
-          <t>导航04</t>
+          <t>导航05</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>lindis-pass-route</t>
+          <t>nav05-b-route</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>完整山口路线</t>
+          <t>后半程到已订住宿</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2793,7 +2793,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand%7CLindis+Pass+Lookout%2C+New+Zealand%7CLuggate%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Lindis+Pass+Lookout%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Luggate%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -2807,12 +2807,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>nav05-a-route</t>
+          <t>mount-iron-route</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>前半程到Lindis Pass</t>
+          <t>去Mount Iron</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2822,26 +2822,26 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Twizel+Holiday+Park%2C+122+Mackenzie+Drive%2C+Twizel%2C+New+Zealand&amp;destination=Lindis+Pass+Lookout%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Omarama%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>导航05</t>
+          <t>导航06</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>nav05-b-route</t>
+          <t>wanaka-lakefront-route</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>后半程到已订住宿</t>
+          <t>去湖滨</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2851,26 +2851,26 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Lindis+Pass+Lookout%2C+New+Zealand&amp;destination=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Luggate%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;destination=Wanaka+Lakefront%2C+Ardmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
-          <t>导航05</t>
+          <t>导航06</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>mount-iron-route</t>
+          <t>kika-route</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>去Mount Iron</t>
+          <t>去Kika晚餐</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Kika%2C+2+Dunmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -2894,12 +2894,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>wanaka-lakefront-route</t>
+          <t>waterfall-creek-route</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>去湖滨</t>
+          <t>平缓备选Waterfall Creek</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Mount+Iron+Track+Car+Park%2C+Wanaka%2C+New+Zealand&amp;destination=Wanaka+Lakefront%2C+Ardmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Waterfall+Creek+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -2923,12 +2923,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>kika-route</t>
+          <t>nav07-leg1-route</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>去Kika晚餐</t>
+          <t>备选：经Cromwell到Frankton</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2938,26 +2938,26 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Kika%2C+2+Dunmore+Street%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cromwell+Heritage+Precinct%2C+Cromwell%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
-          <t>导航06</t>
+          <t>导航07</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>waterfall-creek-route</t>
+          <t>nav07-leg2-route</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>平缓备选Waterfall Creek</t>
+          <t>第二段Frankton到Te Anau</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2967,26 +2967,26 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Waterfall+Creek+Car+Park%2C+Wanaka%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Frankton%2C+Queenstown%2C+New+Zealand&amp;destination=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Kingston%2C+Otago%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CMossburn%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
-          <t>导航06</t>
+          <t>导航07</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>nav07-leg1-route</t>
+          <t>crown-range-route</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>备选：经Cromwell到Frankton</t>
+          <t>第一段经Crown Range、Arrowtown到Frankton</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2996,7 +2996,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cromwell+Heritage+Precinct%2C+Cromwell%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cardrona+Hotel%2C+Cardrona%2C+New+Zealand%7CCrown+Range+Summit%2C+New+Zealand%7CArrowtown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -3010,12 +3010,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>nav07-leg2-route</t>
+          <t>arrowtown-map</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>第二段Frankton到Te Anau</t>
+          <t>Arrowtown</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3025,26 +3025,26 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Frankton%2C+Queenstown%2C+New+Zealand&amp;destination=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Kingston%2C+Otago%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CMossburn%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Arrowtown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
-          <t>导航07</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>crown-range-route</t>
+          <t>diamond-lake-map</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>第一段经Crown Range、Arrowtown到Frankton</t>
+          <t>Diamond Lake 停车场</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3054,55 +3054,55 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=1+Outlet+Road%2C+Wanaka%2C+New+Zealand&amp;destination=Frankton%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Cardrona+Hotel%2C+Cardrona%2C+New+Zealand%7CCrown+Range+Summit%2C+New+Zealand%7CArrowtown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Diamond+Lake+Track+Car+Park%2C+Wanaka-Mount+Aspiring+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
-          <t>导航07</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>arrowtown-map</t>
+          <t>diamond-lake-official</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Arrowtown</t>
+          <t>Lake Wānaka Lookout Track</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Arrowtown%2C+New+Zealand</t>
+          <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/otago/places/diamond-lake-and-hospital-flat/things-to-do/lake-wanaka-lookout-track</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>diamond-lake-map</t>
+          <t>frankton-map</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Diamond Lake 停车场</t>
+          <t>Frankton / Remarkables Park</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Diamond+Lake+Track+Car+Park%2C+Wanaka-Mount+Aspiring+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Remarkables+Park%2C+Frankton%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -3126,70 +3126,70 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>diamond-lake-official</t>
+          <t>kelvin-trail-map</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Lake Wānaka Lookout Track</t>
+          <t>Kelvin Heights 雕塑环线起点</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://www.doc.govt.nz/parks-and-recreation/places-to-go/otago/places/diamond-lake-and-hospital-flat/things-to-do/lake-wanaka-lookout-track</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Peninsula+Road+and+Grove+Lane%2C+Kelvin+Heights%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>kelvin-trail-official</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Frankton / Remarkables Park</t>
+          <t>Kelvin Heights Peninsula Trail</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Remarkables+Park%2C+Frankton%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.queenstownnz.co.nz/listing/kelvin-heights-peninsula-trail/9101/</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Queenstown NZ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>kelvin-trail-map</t>
+          <t>moke-lake-map</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Kelvin Heights 雕塑环线起点</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Peninsula+Road+and+Grove+Lane%2C+Kelvin+Heights%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Moke+Lake%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
@@ -3213,12 +3213,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>kelvin-trail-official</t>
+          <t>moke-lake-official</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Kelvin Heights Peninsula Trail</t>
+          <t>Moke Lake Loop Track</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3228,26 +3228,26 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://www.queenstownnz.co.nz/listing/kelvin-heights-peninsula-trail/9101/</t>
+          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/otago/places/queenstown-area/things-to-do/moke-lake-loop-track</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Queenstown NZ</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>moke-lake-map</t>
+          <t>barangaroo-map</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Barangaroo Reserve</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Moke+Lake%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Barangaroo+Reserve%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -3271,70 +3271,70 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>moke-lake-official</t>
+          <t>mrs-macquarie-map</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Moke Lake Loop Track</t>
+          <t>Mrs Macquarie's Chair</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/otago/places/queenstown-area/things-to-do/moke-lake-loop-track</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Mrs+Macquarie%27s+Chair%2C+Sydney+NSW%2C+Australia</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>DOC</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>barangaroo-map</t>
+          <t>manly-ferry-official</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Barangaroo Reserve</t>
+          <t>悉尼渡轮（F1 Manly线）</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Barangaroo+Reserve%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://transportnsw.info/travel-info/ways-to-get-around/ferry</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Transport for NSW</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>mrs-macquarie-map</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Mrs Macquarie's Chair</t>
+          <t>Earnslaw Park</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Mrs+Macquarie%27s+Chair%2C+Sydney+NSW%2C+Australia</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3358,70 +3358,70 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>manly-ferry-official</t>
+          <t>waitomo-map</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>悉尼渡轮（F1 Manly线）</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://transportnsw.info/travel-info/ways-to-get-around/ferry</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Transport for NSW</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>glowworm-official</t>
+          <t>viaduct-map</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Te Anau Glowworm Caves（RealNZ）</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://www.realnz.com/en/experiences/glowworm-caves/te-anau-glowworm-caves/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
-          <t>RealNZ</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>wynyard-map</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Earnslaw Park</t>
+          <t>Silo Park / Wynyard Quarter</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
@@ -3445,12 +3445,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>mt-eden-map</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3460,7 +3460,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Maungawhau+Mount+Eden+Summit%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -3474,22 +3474,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>fergburger-map</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Silo Park / Wynyard Quarter</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -3503,51 +3503,51 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>mt-eden-map</t>
+          <t>fergburger-official</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Mt Eden · Maungawhau</t>
+          <t>Fergburger官网</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Maungawhau+Mount+Eden+Summit%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.fergburger.com/</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>fergburger-map</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -3561,22 +3561,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>fergburger-official</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Fergburger官网</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.fergburger.com/</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -3590,12 +3590,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -3619,41 +3619,41 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>完整路线到Fernhill</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3663,26 +3663,26 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>导航08</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>去程经Bennetts Bluff</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3692,26 +3692,26 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>导航09</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Glenorchy回住宿</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3721,26 +3721,26 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>导航09</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>nav10-route</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>机场方向参考路线</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3750,159 +3750,14 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>导航09</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
-        <is>
-          <t>nav09-back-route</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Glenorchy回住宿</t>
-        </is>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>导航09</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
-        <is>
-          <t>nav10-route</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>机场方向参考路线</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr">
-        <is>
           <t>导航10</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
-        <is>
-          <t>nav11-out-route</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>市区参考起点经Matamata到现场</t>
-        </is>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Britomart%2C+Auckland%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>导航11</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>nav11-matamata-route</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Matamata休息后到现场</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Matamata+i-SITE+Visitor+Information+Centre%2C+Matamata%2C+New+Zealand&amp;destination=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>导航11</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>现场回Auckland市中心参考</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>map</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=The+Shire%27s+Rest%2C+501+Buckland+Road%2C+Hinuera%2C+Matamata+3472%2C+New+Zealand&amp;destination=Britomart%2C+Auckland%2C+New+Zealand&amp;travelmode=driving</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>导航11</t>
         </is>
       </c>
     </row>
@@ -4039,7 +3894,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>南岛还车飞Auckland，Hobbiton中文团，城市日后夜航回国。</t>
+          <t>南岛还车飞Auckland，萤火虫洞＋霍比屯一日团，城市日后夜航回国。</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5055,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>09:00左右出发；17:15到RealNZ报到萤火虫团</t>
+          <t>09:00左右出发；10:00前退房</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -5227,8 +5082,7 @@
         <is>
           <t>住宿｜Private Ensuite in the Heart of Te Anau，3 Thomson Place；15:00后入住。
 驾驶安排｜纯驾驶约3.5–4.5小时，加Arrowtown午餐和停靠留5–6小时；抵达时间随休息调整。
-坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。
-傍晚｜17:45 萤火虫洞团。Arrowtown 控制在 90 分钟内，15:00–16:30 到 Te Anau；改走 Cromwell 多 20–30 分钟也赶得上，最晚 16:30 前到住处。</t>
+坏天气｜起雾、大风或下雨时别翻Crown Range，改走Cromwell（导航里有备选链接），从Frankton起两条路一样。</t>
         </is>
       </c>
     </row>
@@ -5681,7 +5535,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Auckland ↔ Hobbiton</t>
+          <t>Auckland ↔ Waitomo ↔ Hobbiton</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -5697,12 +5551,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Hobbiton中文团，一天往返</t>
+          <t>Waitomo萤火虫洞 + Hobbiton一日团</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>保留已付13:50普通话导览，把往返时间留宽。</t>
+          <t>跟团一天：上午坐船看萤火虫，下午走进霍比屯。</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -5717,24 +5571,24 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Waikato约15–26°C，午后日晒强，偶有阵雨。</t>
+          <t>Waikato约15–26°C，午后日晒强，偶有阵雨；洞里常年凉。</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>防晒、帽子、好走的鞋；车上备一件薄外套。</t>
+          <t>防晒、帽子、好走的鞋；带一件外套进洞。</t>
         </is>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>交通待定：一日租车自驾，或大巴 / 接驳</t>
+          <t>跟团大巴（Klook，已订）· 06:00出发，约17:30回到Auckland</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>13:30前到The Shire’s Rest报到</t>
+          <t>06:00出发；上车地点以确认单为准</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -5744,26 +5598,21 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>shire-rest-map</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>hobbiton-booking</t>
-        </is>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
+          <t>waitomo-hobbiton-booking</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>住宿｜回同一家Auckland住宿，第二晚。
-交通待定｜还没决定租车还是公共交通。现票只含Shire’s Rest至片场巴士，不含Auckland往返。
-方案A 租车｜一日租车自驾，往返纯驾驶约4.5–5小时，须支持晚间还车；按下方导航11执行。
-方案B 大巴 / 接驳｜Auckland没有直达Shire’s Rest的公共交通：可坐长途大巴到Matamata再打车到501 Buckland Road，或订接受自购票的纯接送。选这个方案前确认班次能13:30前送到Shire’s Rest、16:20后能接回Auckland。
-回程｜Hobbiton约16:20结束，随后返程，约19:00–20:00回到Auckland。</t>
+跟团｜Klook Hobbiton + Waitomo 一日团：先去Waitomo萤火虫洞（洞里约1小时，最后坐小船看萤火虫，洞内讲解是英文），再去Hobbiton片场；车上有中文讲解。06:00出发，约17:30回到Auckland。
+以确认单为准｜上车地点（集合点还是酒店接送）、午餐是否包含，出发前一周在Klook确认。
+准备｜前一晚早睡；早餐带上车；洞里凉、不能拍照，带外套；车程单程约2–2.5小时，带水和零食。</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8331,34 +8180,22 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17:15–17:30</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau镇上</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>开几分钟到85 Lakefront Drive报到，就是明天Milford的集合点。</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>报到</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>报到时间以确认单为准。</t>
-        </is>
-      </c>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>realnz-map</t>
-        </is>
-      </c>
+          <t>早点吃晚饭。</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -8367,36 +8204,36 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>17:45–20:00</t>
+          <t>20:40–21:15</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Te Anau萤火虫洞</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>RealNZ萤火虫洞团：坐船过湖，步行进洞，再坐小船看萤火虫，约2小时15分。</t>
+          <t>沿Lakefront Drive散步，湖岸朝西，看21:09的日落落在湖上；离住处几分钟，看完回去早点睡。</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>萤火虫</t>
+          <t>湖上日落</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>洞内8–12°C，带外套；洞里不能拍照。</t>
+          <t>明早09:15去Milford报到。</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>realnz-map,glowworm-official</t>
+          <t>realnz-walk-route</t>
         </is>
       </c>
     </row>
@@ -8407,98 +8244,94 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Te Anau镇上</t>
+          <t>Frankton / Kingston / Te Anau</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>回来直接吃晚饭；不少餐厅厨房21:00前后停止点餐，要提前订，选离湖边近的。</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>晚饭</t>
-        </is>
-      </c>
+          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：17:30在Te Anau镇上</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
       <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>21:00–21:15</t>
+          <t>08:00左右</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>饭后沿Lakefront Drive走走，湖岸朝西，看21:09的日落，然后回住宿早点睡。</t>
+          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>湖上日落</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>明早09:15去Milford报到。</t>
-        </is>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>realnz-walk-route</t>
-        </is>
-      </c>
+          <t>装备检查</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:15左右到，09:30前完成报到</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Frankton / Kingston / Te Anau</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：20:15在Te Anau镇上（要订）</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr"/>
+          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>已订集合</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>realnz-map,realnz-walk-route</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8507,30 +8340,34 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>08:00左右</t>
+          <t>09:50–17:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Milford Sound</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>装备检查</t>
+          <t>峡湾</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>realnz-booking</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8539,32 +8376,28 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>09:15左右到，09:30前完成报到</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>已订集合</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>realnz-map,realnz-walk-route</t>
+          <t>redcliff-official</t>
         </is>
       </c>
     </row>
@@ -8575,32 +8408,32 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>09:50–17:00</t>
+          <t>20:45–21:15</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Milford Sound</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>峡湾</t>
+          <t>饭后散步</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>realnz-booking</t>
+          <t>realnz-walk-route</t>
         </is>
       </c>
     </row>
@@ -8611,94 +8444,94 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>redcliff-official</t>
-        </is>
-      </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>20:45–21:15</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>饭后散步</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
       <c r="H77" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
+          <t>nav08-route</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr"/>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>frankton-map</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8707,28 +8540,36 @@
         </is>
       </c>
       <c r="B79" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>13:30–15:00</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>起点在Peninsula Road和Grove Lane路口。</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
         </is>
       </c>
     </row>
@@ -8739,32 +8580,32 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>12:00–13:00</t>
+          <t>15:30–16:00</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Frankton</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>午餐</t>
+          <t>入住Fernhill</t>
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
       <c r="H80" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>fernhill-map</t>
         </is>
       </c>
     </row>
@@ -8775,36 +8616,36 @@
         </is>
       </c>
       <c r="B81" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>13:30–15:00</t>
+          <t>傍晚 17:00–19:00</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Kelvin Peninsula Sculpture Trail</t>
+          <t>Skyline Gondola · Bob’s Peak</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场一圈约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>湖畔雕塑步道</t>
+          <t>俯瞰皇后镇</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>起点在Peninsula Road和Grove Lane路口。</t>
+          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>kelvin-trail-map,kelvin-trail-official</t>
+          <t>skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
@@ -8815,32 +8656,32 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15:30–16:00</t>
+          <t>19:00–20:30</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>Blue Kanu</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
+          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>入住Fernhill</t>
+          <t>晚餐</t>
         </is>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
         <is>
-          <t>fernhill-map</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
     </row>
@@ -8851,36 +8692,32 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>傍晚 17:00–19:00</t>
+          <t>20:40–21:10</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>Earnslaw Park / 湖边</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
+          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>俯瞰皇后镇</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
-        </is>
-      </c>
+          <t>湖边日落</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
     </row>
@@ -8891,98 +8728,98 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>19:00–20:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Blue Kanu</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>晚餐</t>
-        </is>
-      </c>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr">
-        <is>
-          <t>blue-kanu-official</t>
-        </is>
-      </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>20:40–21:10</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Earnslaw Park / 湖边</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>湖边日落</t>
+          <t>湖边公路</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Frankton / Blue Kanu</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr"/>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>红船屋</t>
+        </is>
+      </c>
       <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>bennetts-bluff-official</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -8991,32 +8828,36 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>湖边公路</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr"/>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
     </row>
@@ -9027,32 +8868,28 @@
         </is>
       </c>
       <c r="B88" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>红船屋</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
     </row>
@@ -9063,36 +8900,36 @@
         </is>
       </c>
       <c r="B89" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>18:00–20:30</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>湿地步道</t>
+          <t>傍晚湖面倒影</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
+          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>moke-lake-map,moke-lake-official</t>
         </is>
       </c>
     </row>
@@ -9103,28 +8940,32 @@
         </is>
       </c>
       <c r="B90" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>21:00左右</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr"/>
+          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>皇后镇招牌汉堡</t>
+        </is>
+      </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
         </is>
       </c>
     </row>
@@ -9135,102 +8976,98 @@
         </is>
       </c>
       <c r="B91" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>18:00–20:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>从Glenorchy路岔进Moke Lake Road，约30分钟到湖边。环湖步道约6km、2–2.5小时；不想走完就在营地一侧湖边看倒影，傍晚无风时最好。</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>傍晚湖面倒影</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>后半圈是傍晚斜光；20:30开回碎石路，21:00日落前回到铺装路。</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>moke-lake-map,moke-lake-official</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>21:00左右</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>回市中心吃Fergburger，这个点排队短一些，也可以打包到湖边吃；之后整理行李，准备次日加油还车。</t>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>皇后镇招牌汉堡</t>
+          <t>南岛收车</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
+          <t>nav10-route</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Glenorchy / Fergburger</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr"/>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>等飞机</t>
+        </is>
+      </c>
       <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>zqn-map</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -9239,34 +9076,30 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+          <t>飞奥克兰。</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>南岛收车</t>
+          <t>航班</t>
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>nav10-route</t>
-        </is>
-      </c>
+      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9275,32 +9108,32 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>等飞机</t>
+          <t>连住两晚</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>zqn-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
     </row>
@@ -9311,30 +9144,34 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
+          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>航班</t>
+          <t>情人节晚餐</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>viaduct-map</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -9343,32 +9180,36 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>19:45–20:45</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>Wynyard Quarter / Silo Park</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>取行李，坐 SkyBus 或打车进城（约 45–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>连住两晚</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr"/>
+          <t>海港日落</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>明早06:00出发，看完日落就回酒店早睡。</t>
+        </is>
+      </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>wynyard-map</t>
         </is>
       </c>
     </row>
@@ -9379,102 +9220,102 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>18:00–19:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>情人节晚餐</t>
-        </is>
-      </c>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr">
-        <is>
-          <t>viaduct-map</t>
-        </is>
-      </c>
+      <c r="H98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>19:45–20:45</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Wynyard Quarter / Silo Park</t>
+          <t>Auckland出发</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>沿海边走到Wynyard Quarter / Silo Park，20:00–20:30朝西看海港大桥方向的日落（约20:19），再经Viaduct走回酒店。</t>
+          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>海港日落</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>想换个角度可以上Sky Tower观景台，要另买票，人也多。</t>
-        </is>
-      </c>
+          <t>早起出发</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
+          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>萤火虫洞</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>洞里凉、不能拍照；讲解是英文。</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>waitomo-map</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9483,32 +9324,32 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>08:30–09:30</t>
+          <t>中午–下午</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Auckland市区出发</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>交通方式待定：租车就08:30–09:00取车、09:30前出城；坐大巴或接驳就按班次出发，保证13:30前到Shire’s Rest。</t>
+          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>交通待定</t>
+          <t>霍比屯</t>
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>nav11-out-route,hobbiton-transfers-official</t>
+          <t>shire-rest-map</t>
         </is>
       </c>
     </row>
@@ -9519,30 +9360,26 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>12:30–13:00</t>
+          <t>约17:30</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>The Shire’s Rest</t>
+          <t>回到Auckland</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>到The Shire’s Rest，吃简餐、上洗手间。</t>
+          <t>回到市区，回酒店歇一会儿。</t>
         </is>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>shire-rest-map</t>
-        </is>
-      </c>
+      <c r="H102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9551,34 +9388,26 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>13:30前</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>The Shire’s Rest Ticketing Office</t>
+          <t>Auckland市中心</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>在The Shire’s Rest Ticketing Office报到。</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>已订报到</t>
-        </is>
-      </c>
+          <t>酒店附近吃晚饭。</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr">
-        <is>
-          <t>hobbiton-booking</t>
-        </is>
-      </c>
+      <c r="H103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9587,30 +9416,38 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>13:50–约16:20</t>
+          <t>19:45–20:40（可选）</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>已订Mandarin Language Tour；片场游览约2.5小时。</t>
+          <t>打车约15分钟到山脚，走15–20分钟上山顶，20:18看整座城的日落，下山打车回酒店。</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>中文导览</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+          <t>城市日落</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>早起累了就跳过；山顶不能开车上去。</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>mt-eden-map</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9619,102 +9456,90 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16:30–17:00左右返程</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Hobbiton → Auckland</t>
+          <t>车上 / 途中 / Auckland</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>回Auckland，按约19:00–20:00抵城安排晚餐；租车的话晚上还车，坐大巴或接驳按回程班次。</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>晚间回城</t>
-        </is>
-      </c>
+          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>nav11-back-route</t>
-        </is>
-      </c>
+      <c r="H105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>19:45–20:40（可选，租车时）</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Mt Eden · Maungawhau</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>租车且19:30前回到奥克兰的话，顺路去Mt Eden：车停山脚，走15–20分钟上山顶，20:18看整座城的日落，下山再吃晚饭、还车。</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>城市日落</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>山顶不能开车上去；坐大巴或接驳就跳过。</t>
-        </is>
-      </c>
-      <c r="H106" t="inlineStr">
-        <is>
-          <t>mt-eden-map</t>
-        </is>
-      </c>
+          <t>退房并寄存行李。</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Shire’s Rest / Auckland</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：现场简餐或自备；晚餐：Auckland，避免绑定太早的餐厅时段</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr"/>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>美术馆</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>art-gallery-map,art-gallery-official</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9723,26 +9548,34 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>退房并寄存行李；如租车留到今天，先完成市区还车。</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
+          <t>Britomart午餐，首选Amano，待预约。</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>完整午餐</t>
+        </is>
+      </c>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>amano-map,amano-official</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9751,34 +9584,26 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>Britomart</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>美术馆</t>
-        </is>
-      </c>
+          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>art-gallery-map,art-gallery-official</t>
-        </is>
-      </c>
+      <c r="H109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9787,32 +9612,32 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>晚上</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>Auckland Airport</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>完整午餐</t>
+          <t>夜航回国</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>amano-map,amano-official</t>
+          <t>akl-intl-map,akl-departure-official</t>
         </is>
       </c>
     </row>
@@ -9823,21 +9648,21 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>市区 / Amano</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
         </is>
       </c>
       <c r="F111" t="inlineStr"/>
@@ -9847,66 +9672,70 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d17</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>05:00–09:10</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>广州白云T2</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>夜航回国</t>
+          <t>转机</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr">
-        <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
+      <c r="H112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d17</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:10–11:10</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>CZ3803 → 杭州萧山T4</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9915,98 +9744,30 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>落地后</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>转机</t>
+          <t>按航班实际到达时间</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
       <c r="H114" t="inlineStr"/>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>d17</t>
-        </is>
-      </c>
-      <c r="B115" t="n">
-        <v>20</v>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>09:10–11:10</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>CZ3803 → 杭州萧山T4</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>飞回杭州，取行李回家。</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>到家</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr">
-        <is>
-          <t>hgh-airport-map</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>d17</t>
-        </is>
-      </c>
-      <c r="B116" t="n">
-        <v>90</v>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>饮食</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>落地后</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>按航班实际到达时间</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10019,7 +9780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10389,43 +10150,6 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>nav10-route,zqn-map,qt-airport-rental-official</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>d15</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>导航11 · （若租车）Auckland ↔ Hobbiton</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>08:30–09:00提车，09:30左右离开市区；去回各预留约3小时交通窗口含短休息，13:30前报到。</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Auckland市区实际取车点 → SH1南行 → 按当日导航经SH2 / SH27到Matamata → 501 Buckland Road / The Shire’s Rest；返程回实际还车点</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>取还车点尚未确定，地图先以Britomart作CBD参考；实际使用时替换成车行地址。优先支持晚间自助还车的网点；若必须次晨还，另计过夜停车和租期，2/16先还车再城市活动。现有票不含Auckland接送；纯接送只有确认接受自购票、13:30前送达且16:20后接回才可替代本页自驾。</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>nav11-out-route,nav11-matamata-route,nav11-back-route,shire-rest-map,hobbiton-faq-official,hobbiton-transfers-official</t>
         </is>
       </c>
     </row>
@@ -10440,7 +10164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11442,131 +11166,6 @@
       <c r="E40" t="inlineStr">
         <is>
           <t>12:30 前办托运，JQ296 13:30 起飞。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>10</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>取车点 → Matamata</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>约2–2.5小时，路况另留量</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>可在Matamata短休息；i-SITE只是途中停靠参考，并非这张票的报到点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>20</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Matamata → The Shire’s Rest</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>约15–25分钟</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>最终目的地501 Buckland Road。乡村道路跟当日导航与标识，不套用旧攻略出口号。</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>30</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>现场停车、午餐、报到</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>约30–60分钟缓冲</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>目标12:30–13:00到；停访客停车区，13:30前到Ticketing Office。</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>40</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>13:50 → 约16:20</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>已订导览约2.5小时</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>乘运营商巴士进出片场，私家车停在Shire’s Rest。</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>nav11</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>50</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>约16:30–17:00 → Auckland</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>约2.5–3小时</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>按19:00–20:00抵城安排；堵车、离场晚时顺延，不在当天衔接国际航班。</t>
         </is>
       </c>
     </row>
@@ -11977,7 +11576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12144,42 +11743,42 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>auckland-hotel</t>
+          <t>tour-0215-pickup</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>尽早</t>
+          <t>出发前一周</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>订奥克兰两晚（2/14–16）</t>
+          <t>确认 2/15 一日团的上车地点</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>同一家连住，选 CBD / Britomart 附近，能在 2/16 退房后寄存行李。</t>
+          <t>06:00 出发：在 Klook 确认单或客服问清是集合点还是酒店接送、午餐包不包含；订好奥克兰酒店后把地址发给他们。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hobbiton-transport</t>
+          <t>auckland-hotel</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -12189,17 +11788,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>定了机票后</t>
+          <t>尽早</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>定 2/15 去 Hobbiton 怎么走</t>
+          <t>订奥克兰两晚（2/14–16）</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>租车自驾（要能晚上还车），或坐大巴 / 接驳（要 13:30 前送到 Shire’s Rest、16:20 后能接回）。</t>
+          <t>同一家连住，选 CBD / Britomart 附近，能在 2/16 退房后寄存行李。</t>
         </is>
       </c>
     </row>
@@ -12423,11 +12022,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>glowworm</t>
+          <t>skyline</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -12437,59 +12036,59 @@
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>尽早</t>
+          <t>可选</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>订 Te Anau 萤火虫洞 2/10 17:45 场</t>
+          <t>买 Skyline 缆车票（2/12）</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>RealNZ 坐船过湖进洞，约 2 小时 15 分，约 20:00 回来，每人约 NZ$154；先在官网确认这天有 17:45 场。同时订 20:15 的晚饭（不少餐厅 21:00 前后停止点餐）。</t>
+          <t>网上或现场都能买。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>skyline</t>
+          <t>milford-terms</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>出发前</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>买 Skyline 缆车票（2/12）</t>
+          <t>查 Milford 订单的天气退改规则</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>网上或现场都能买。</t>
+          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>milford-terms</t>
+          <t>host-notes</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -12499,129 +12098,133 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>出发前</t>
+          <t>入住前</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>查 Milford 订单的天气退改规则</t>
+          <t>拿到三处民宿的入住说明</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
+          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>host-notes</t>
+          <t>pay-fernhill</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>入住前</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>拿到三处民宿的入住说明</t>
+          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
+          <t>Apple Pay 付款。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>pay-hikuwai</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>pay</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-01-26</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>pay-teanau</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -12630,68 +12233,68 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>1/28</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Te Anau 尾款 NZ$386.40</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>cancel-metropolitan</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -12700,33 +12303,33 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/3 14:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>基督城 Metropolitan 免费取消截止</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
+          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cancel-metropolitan</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -12740,28 +12343,28 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2/3 14:00</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>基督城 Metropolitan 免费取消截止</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cancel-hikuwai</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -12770,17 +12373,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2027-02-03</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2/3 16:00</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -12792,15 +12395,15 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cancel-teanau</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -12810,50 +12413,15 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2/5 15:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Te Anau 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>280</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>
@@ -12951,7 +12519,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Hobbiton 那天是长日子</t>
+          <t>2/15 要早起</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -12966,15 +12534,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>奥克兰到 Shire’s Rest 单程约 175 公里，来回 4.5–5 小时，加上 2.5 小时导览，全天 10 小时左右，前一天还刚飞过来。</t>
+          <t>一日团 06:00 出发、约 17:30 回来，单程车程约 2–2.5 小时，前一天还刚从皇后镇飞过来。</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>租车的话两人轮流开，09:00 出发更从容；坐大巴或接驳就盯紧 13:30 报到和 16:20 结束。两种都建议 2/14 早点睡、午饭在 Shire’s Rest 解决、晚饭订 20:00 以后。</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>2/14 看完日落就回酒店早睡；早餐带上车；回来后晚上不排硬行程，Mt Eden 看日落只在有精神时去。</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>waitomo-hobbiton-booking</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">

</xml_diff>

<commit_message>
content: 2/12 Skyline gondola + 3 luge rides booked for 16:30–18:30
- Kelvin Peninsula 13:15–14:45, check-in 15:10–15:50, at Brecon Street by 16:15
- Skyline to-do removed (checklist 25 → 24)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,17 +3532,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3554,77 +3554,77 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>两人 ¥644</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3648,12 +3648,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3663,26 +3663,26 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>完整路线到Fernhill</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3692,26 +3692,26 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>导航08</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Glenorchy回住宿</t>
+          <t>去程经Bennetts Bluff</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -3735,12 +3735,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>机场方向参考路线</t>
+          <t>Glenorchy回住宿</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3750,12 +3750,41 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>机场方向参考路线</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
         <is>
           <t>导航10</t>
         </is>
@@ -5266,7 +5295,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>09:30左右出发；15:30–16:00入住</t>
+          <t>09:30左右出发；16:15前到缆车站（16:30已订）</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -5281,7 +5310,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>no-fixed-ticket</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -8544,7 +8573,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>13:30–15:00</t>
+          <t>13:15–14:45</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8564,7 +8593,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>起点在Peninsula Road和Grove Lane路口。</t>
+          <t>起点在Peninsula Road和Grove Lane路口；14:45前走完，留出入住和去缆车的时间。</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -8584,7 +8613,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15:30–16:00</t>
+          <t>15:10–15:50</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8594,7 +8623,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李；车留在住处，晚上在市区吃饭。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -8620,32 +8649,32 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>傍晚 17:00–19:00</t>
+          <t>16:30–18:30</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>Skyline Gondola + Luge · Bob’s Peak</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
+          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>俯瞰皇后镇</t>
+          <t>缆车＋Luge</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
+          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>skyline-booking,skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
@@ -8670,7 +8699,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
+          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -10060,7 +10089,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，12:00–13:00到Frankton；Kelvin半岛步道后15:30–16:00入住。</t>
+          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，12:00–13:00到Frankton；Kelvin半岛步道后15:10–15:50入住，16:30坐缆车（已订）。</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -11576,7 +11605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11953,7 +11982,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>缆车下来后约 19:00。</t>
+          <t>缆车 18:30 下来，约 19:00。</t>
         </is>
       </c>
     </row>
@@ -12022,42 +12051,42 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>skyline</t>
+          <t>milford-terms</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>出发前</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>买 Skyline 缆车票（2/12）</t>
+          <t>查 Milford 订单的天气退改规则</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>网上或现场都能买。</t>
+          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>milford-terms</t>
+          <t>host-notes</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -12067,129 +12096,133 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>出发前</t>
+          <t>入住前</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>查 Milford 订单的天气退改规则</t>
+          <t>拿到三处民宿的入住说明</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
+          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>host-notes</t>
+          <t>pay-fernhill</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>入住前</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>拿到三处民宿的入住说明</t>
+          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
+          <t>Apple Pay 付款。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>pay-hikuwai</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>pay</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-01-26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>pay-teanau</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -12198,68 +12231,68 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>1/28</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Te Anau 尾款 NZ$386.40</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>cancel-metropolitan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -12268,33 +12301,33 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/3 14:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>基督城 Metropolitan 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
+          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-metropolitan</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -12308,28 +12341,28 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/3 14:00</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>基督城 Metropolitan 免费取消截止</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cancel-hikuwai</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -12338,17 +12371,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2027-02-03</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2/3 16:00</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -12360,15 +12393,15 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cancel-teanau</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -12378,50 +12411,15 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2/5 15:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Te Anau 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>280</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>

</xml_diff>

<commit_message>
content: 2/12 Skyline gondola + 3 luge rides booked for 16:30–18:30 (#11)
- Kelvin Peninsula 13:15–14:45, check-in 15:10–15:50, at Brecon Street by 16:15
- Skyline to-do removed (checklist 25 → 24)

Co-authored-by: SeanSun <s413286943-cmyk@users.noreply.github.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G110"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3532,17 +3532,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3554,77 +3554,77 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>两人 ¥644</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3648,12 +3648,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3663,26 +3663,26 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>完整路线到Fernhill</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3692,26 +3692,26 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>导航08</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Glenorchy回住宿</t>
+          <t>去程经Bennetts Bluff</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -3735,12 +3735,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>机场方向参考路线</t>
+          <t>Glenorchy回住宿</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3750,12 +3750,41 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>机场方向参考路线</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
         <is>
           <t>导航10</t>
         </is>
@@ -5266,7 +5295,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>09:30左右出发；15:30–16:00入住</t>
+          <t>09:30左右出发；16:15前到缆车站（16:30已订）</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -5281,7 +5310,7 @@
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>no-fixed-ticket</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
@@ -8544,7 +8573,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>13:30–15:00</t>
+          <t>13:15–14:45</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8564,7 +8593,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>起点在Peninsula Road和Grove Lane路口。</t>
+          <t>起点在Peninsula Road和Grove Lane路口；14:45前走完，留出入住和去缆车的时间。</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -8584,7 +8613,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>15:30–16:00</t>
+          <t>15:10–15:50</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8594,7 +8623,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李休息。</t>
+          <t>开约20分钟到Fernhill，入住15 Greenstone Place，放下行李；车留在住处，晚上在市区吃饭。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -8620,32 +8649,32 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>傍晚 17:00–19:00</t>
+          <t>16:30–18:30</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Skyline Gondola · Bob’s Peak</t>
+          <t>Skyline Gondola + Luge · Bob’s Peak</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>坐Skyline缆车上Bob’s Peak看湖和Remarkables山脉，按1.5–2小时安排；想玩可加Luge滑道。缆车站在Brecon Street，离Fernhill很近。</t>
+          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>俯瞰皇后镇</t>
+          <t>缆车＋Luge</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>缆车夏季约21:00关门，山上赶不上日落；票网上或现场买，大风时可能停运。</t>
+          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>skyline-map,skyline-official</t>
+          <t>skyline-booking,skyline-map,skyline-official</t>
         </is>
       </c>
     </row>
@@ -8670,7 +8699,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>下山吃晚饭Blue Kanu。缆车停运就先去Queenstown Gardens湖边轻走。</t>
+          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -10060,7 +10089,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，12:00–13:00到Frankton；Kelvin半岛步道后15:30–16:00入住。</t>
+          <t>09:30左右出发、10:00前退房；纯驾驶约2–2.5小时，12:00–13:00到Frankton；Kelvin半岛步道后15:10–15:50入住，16:30坐缆车（已订）。</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -11576,7 +11605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11953,7 +11982,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>缆车下来后约 19:00。</t>
+          <t>缆车 18:30 下来，约 19:00。</t>
         </is>
       </c>
     </row>
@@ -12022,42 +12051,42 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>skyline</t>
+          <t>milford-terms</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>可选</t>
+          <t>出发前</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>买 Skyline 缆车票（2/12）</t>
+          <t>查 Milford 订单的天气退改规则</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>网上或现场都能买。</t>
+          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>milford-terms</t>
+          <t>host-notes</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -12067,129 +12096,133 @@
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>出发前</t>
+          <t>入住前</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>查 Milford 订单的天气退改规则</t>
+          <t>拿到三处民宿的入住说明</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Milford Road 封路时是全额退款还是改期，能改到哪天。</t>
+          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>host-notes</t>
+          <t>pay-fernhill</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>pay</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2027-01-05</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>入住前</t>
+          <t>1/5</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>拿到三处民宿的入住说明</t>
+          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Wānaka、Te Anau、Fernhill：停车位置、门锁或钥匙、晚到怎么办。</t>
+          <t>Apple Pay 付款。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>pay-hikuwai</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>pay</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-01-26</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>1/26</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>pay-teanau</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -12198,68 +12231,68 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-01-28</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>1/28</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Te Anau 尾款 NZ$386.40</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>cancel-metropolitan</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -12268,33 +12301,33 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/3 14:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>基督城 Metropolitan 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
+          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-metropolitan</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -12308,28 +12341,28 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/3 14:00</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>基督城 Metropolitan 免费取消截止</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>之后不能取消，房费 ¥601.43 离店扣款；另有 NZ$200 押金会退。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cancel-hikuwai</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -12338,17 +12371,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2027-02-03</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2/3 16:00</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -12360,15 +12393,15 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cancel-teanau</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -12378,50 +12411,15 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2/5 15:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Te Anau 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>280</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>

</xml_diff>

<commit_message>
content: balances are charged to the card automatically, drop the pay to-dos
- Remove the three pay items (Fernhill 1/5, Wānaka 1/26, Te Anau 1/28)
- Lodging info now says when each balance is charged; checklist 25 → 22
- Update note for the 更新 tab

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -11734,7 +11734,11 @@
           <t>Hikuwai Haven 1</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>尾款 NZ$346.84 1/26 自动扣卡，不用操作</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>16:00后入住；10:00前退房；1 Outlet Road, Wānaka</t>
@@ -11780,7 +11784,11 @@
           <t>Private Ensuite in the Heart of Te Anau</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>尾款 NZ$386.40 1/28 自动扣卡，不用操作</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>15:00后入住；10:00前退房；3 Thomson Place</t>
@@ -11828,7 +11836,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>房东Coral</t>
+          <t>房东Coral；NZ$721.63 1/5 自动扣卡，不用操作</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -11910,7 +11918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12484,46 +12492,46 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -12532,230 +12540,125 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>220</v>
+        <v>260</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
-        <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>cancel-hikuwai</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>260</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2027-02-03</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2/3 16:00</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>cancel-teanau</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>270</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2/5 15:00</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Te Anau 免费取消截止</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>280</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>

</xml_diff>

<commit_message>
content: balances are charged to the card automatically, drop the pay to-dos (#17)
- Remove the three pay items (Fernhill 1/5, Wānaka 1/26, Te Anau 1/28)
- Lodging info now says when each balance is charged; checklist 25 → 22
- Update note for the 更新 tab

Co-authored-by: SeanSun <s413286943-cmyk@users.noreply.github.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -11734,7 +11734,11 @@
           <t>Hikuwai Haven 1</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>尾款 NZ$346.84 1/26 自动扣卡，不用操作</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>16:00后入住；10:00前退房；1 Outlet Road, Wānaka</t>
@@ -11780,7 +11784,11 @@
           <t>Private Ensuite in the Heart of Te Anau</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>尾款 NZ$386.40 1/28 自动扣卡，不用操作</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>15:00后入住；10:00前退房；3 Thomson Place</t>
@@ -11828,7 +11836,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>房东Coral</t>
+          <t>房东Coral；NZ$721.63 1/5 自动扣卡，不用操作</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -11910,7 +11918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12484,46 +12492,46 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pay-fernhill</t>
+          <t>cancel-fernhill</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2027-01-05</t>
+          <t>2027-01-13</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1/5</t>
+          <t>1/13 15:00</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 付款 NZ$721.63</t>
+          <t>皇后镇 Fernhill 免费取消截止</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apple Pay 付款。</t>
+          <t>之后到 2/5 15:00 前取消可退一部分。</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cancel-fernhill</t>
+          <t>cancel-greatsouthern</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -12532,230 +12540,125 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2027-01-13</t>
+          <t>2027-02-01</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1/13 15:00</t>
+          <t>2/1 14:00</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>皇后镇 Fernhill 免费取消截止</t>
+          <t>悉尼 Great Southern 免费取消截止</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>之后到 2/5 15:00 前取消可退一部分。</t>
+          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>pay-hikuwai</t>
+          <t>cancel-hikuwai</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>220</v>
+        <v>260</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2027-01-26</t>
+          <t>2027-02-03</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1/26</t>
+          <t>2/3 16:00</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Wānaka Hikuwai 尾款 NZ$346.84</t>
+          <t>Wānaka Hikuwai 免费取消截止</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$86.71 已付。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>pay-teanau</t>
+          <t>cancel-teanau</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>230</v>
+        <v>270</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pay</t>
+          <t>deadline</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2027-01-28</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1/28</t>
+          <t>2/5 15:00</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Te Anau 尾款 NZ$386.40</t>
+          <t>Te Anau 免费取消截止</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apple Pay 扣款，订金 NZ$96.60 已付。</t>
+          <t>之后取消只退一部分。</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cancel-greatsouthern</t>
+          <t>supplies-0205</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>240</v>
+        <v>280</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>deadline</t>
+          <t>prep</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2027-02-01</t>
+          <t>2027-02-05</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2/1 14:00</t>
+          <t>2/5</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>悉尼 Great Southern 免费取消截止</t>
+          <t>买齐长周末补给</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
-        <is>
-          <t>之后不能取消。三晚共 ¥2,027.36，离店扣款；具体取消条款以订单为准。</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>cancel-hikuwai</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>260</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>2027-02-03</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2/3 16:00</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Wānaka Hikuwai 免费取消截止</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>cancel-teanau</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>270</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>deadline</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2/5 15:00</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Te Anau 免费取消截止</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>之后取消只退一部分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>supplies-0205</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>280</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>prep</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>2027-02-05</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2/5</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>买齐长周末补给</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
         <is>
           <t>2/6 Waitangi Day 不少商店不开，取车后在 Ashburton 或 Geraldine 超市把 2/6 的早餐、路餐和水买好。</t>
         </is>

</xml_diff>

<commit_message>
content: 2/7 High Country Salmon as a relaxed food stop, cook salmon at night
- Lunch: look at the ponds, feed the fish, compare sashimi and a hot dish,
  buy a fillet to take back
- Dinner: pan-fry it at the Twizel unit (or the camp kitchen) before Pukaki
- Update note for the 更新 tab

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -7718,7 +7718,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>12:00–13:30</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7728,15 +7728,19 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>High Country Salmon / Logans吃一顿鲑鱼午餐。</t>
+          <t>轻松的美食点：先看看养殖池、喂喂鱼，再在店里点一份刺身和一份热食，对比生吃和熟吃。喜欢的话买一块适合煎的三文鱼带回 Twizel，晚上自己做。</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>鲑鱼午餐</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
+          <t>三文鱼两种吃法</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>鱼食和菜单以当天为准；买生鱼请店里帮忙冷藏包好，回住处马上放冰箱。</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>logans-official</t>
@@ -7764,7 +7768,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>回住宿休息、洗衣或整理行李。</t>
+          <t>回住宿休息、洗衣或整理行李；三文鱼先放冰箱。</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -7787,17 +7791,25 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Twizel</t>
+          <t>Twizel Holiday Park</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>镇上早点吃晚饭。</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
+          <t>用房间厨房煎中午买的三文鱼（房间没灶台就用营地公共厨房），配点沙拉或面包；没买就去镇上吃。早点吃完，20:15 出发去 Pukaki。</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>自己煎三文鱼</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>twizel-holiday-park-map</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7900,7 +7912,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>早餐：镇上或住宿；午餐：High Country Salmon；晚餐：18:30在Twizel</t>
+          <t>早餐：镇上或住宿；午餐：High Country Salmon 刺身＋热食；晚餐：住处自己煎三文鱼</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -10799,7 +10811,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>目的地2602 Twizel–Omarama Highway；午餐留60–90分钟。</t>
+          <t>目的地2602 Twizel–Omarama Highway；看养殖池、喂鱼加午餐留60–90分钟。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: 2/7 High Country Salmon as a relaxed food stop, cook salmon at night (#18)
- Lunch: look at the ponds, feed the fish, compare sashimi and a hot dish,
  buy a fillet to take back
- Dinner: pan-fry it at the Twizel unit (or the camp kitchen) before Pukaki
- Update note for the 更新 tab

Co-authored-by: SeanSun <s413286943-cmyk@users.noreply.github.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -7718,7 +7718,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>12:00–13:30</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -7728,15 +7728,19 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>High Country Salmon / Logans吃一顿鲑鱼午餐。</t>
+          <t>轻松的美食点：先看看养殖池、喂喂鱼，再在店里点一份刺身和一份热食，对比生吃和熟吃。喜欢的话买一块适合煎的三文鱼带回 Twizel，晚上自己做。</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>鲑鱼午餐</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr"/>
+          <t>三文鱼两种吃法</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>鱼食和菜单以当天为准；买生鱼请店里帮忙冷藏包好，回住处马上放冰箱。</t>
+        </is>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
           <t>logans-official</t>
@@ -7764,7 +7768,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>回住宿休息、洗衣或整理行李。</t>
+          <t>回住宿休息、洗衣或整理行李；三文鱼先放冰箱。</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -7787,17 +7791,25 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Twizel</t>
+          <t>Twizel Holiday Park</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>镇上早点吃晚饭。</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr"/>
+          <t>用房间厨房煎中午买的三文鱼（房间没灶台就用营地公共厨房），配点沙拉或面包；没买就去镇上吃。早点吃完，20:15 出发去 Pukaki。</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>自己煎三文鱼</t>
+        </is>
+      </c>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>twizel-holiday-park-map</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -7900,7 +7912,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>早餐：镇上或住宿；午餐：High Country Salmon；晚餐：18:30在Twizel</t>
+          <t>早餐：镇上或住宿；午餐：High Country Salmon 刺身＋热食；晚餐：住处自己煎三文鱼</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -10799,7 +10811,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>目的地2602 Twizel–Omarama Highway；午餐留60–90分钟。</t>
+          <t>目的地2602 Twizel–Omarama Highway；看养殖池、喂鱼加午餐留60–90分钟。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content: D07–D10 forks and add-ons (stargazing, Clay Cliffs, Diamond Lake, Mount Iron, route, Kawarau)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3445,12 +3445,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>mt-john-official</t>
+          <t>clay-cliffs-official</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Mount John · Astro Café（Dark Sky Project）</t>
+          <t>Omarama Clay Cliffs</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3460,113 +3460,113 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://www.darkskyproject.co.nz/eat/astro-cafe/</t>
+          <t>https://www.waitakinz.com/explore/clay-cliffs</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Dark Sky Project</t>
+          <t>Waitaki NZ</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>margaret-official</t>
+          <t>kawarau-bungy-official</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Margaret（Neil Perry）</t>
+          <t>Kawarau Bridge 蹦极中心</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://themargaretfamily.com/venue/margaret/</t>
+          <t>https://www.bungy.co.nz/queenstown/kawarau-bungy-centre/</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>待预约</t>
+          <t>AJ Hackett</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>margaret-map</t>
+          <t>mt-john-official</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Margaret, 30–36 Bay Street, Double Bay</t>
+          <t>Mount John · Astro Café（Dark Sky Project）</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Margaret%2C+30+Bay+Street%2C+Double+Bay+NSW+2028%2C+Australia</t>
+          <t>https://www.darkskyproject.co.nz/eat/astro-cafe/</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Dark Sky Project</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>margaret-official</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Earnslaw Park</t>
+          <t>Margaret（Neil Perry）</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://themargaretfamily.com/venue/margaret/</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>待预约</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>waitomo-map</t>
+          <t>margaret-map</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Waitomo Glowworm Caves</t>
+          <t>Margaret, 30–36 Bay Street, Double Bay</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Margaret%2C+30+Bay+Street%2C+Double+Bay+NSW+2028%2C+Australia</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -3590,12 +3590,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Earnslaw Park</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -3619,12 +3619,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>waitomo-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Silo Park / Wynyard Quarter</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3648,22 +3648,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>fergburger-map</t>
+          <t>viaduct-map</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -3677,128 +3677,128 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>fergburger-official</t>
+          <t>wynyard-map</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Fergburger官网</t>
+          <t>Silo Park / Wynyard Quarter</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.fergburger.com/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>skyline-booking</t>
+          <t>fergburger-map</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>booking</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>两人 ¥644</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>fergburger-official</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>Fergburger官网</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.fergburger.com/</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>两人 ¥644</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -3822,41 +3822,41 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3866,26 +3866,26 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>rippon-map</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>Rippon酒庄</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3895,26 +3895,26 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Glenorchy回住宿</t>
+          <t>完整路线到Fernhill</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3924,26 +3924,26 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>导航08</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>机场方向参考路线</t>
+          <t>去程经Bennetts Bluff</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3953,12 +3953,70 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>nav09-back-route</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Glenorchy回住宿</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>机场方向参考路线</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
         <is>
           <t>导航10</t>
         </is>
@@ -6038,7 +6096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J127"/>
+  <dimension ref="A1:J133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8412,17 +8470,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>22:00后</t>
+          <t>22:30后</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Twizel观星</t>
+          <t>Twizel观星团</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>回Twizel参加观星；具体集合点、语言和时间以确认单为准。</t>
+          <t>参加 Twizel 当地观星团，有人讲解南半球星空、带望远镜；具体集合点、语言和时间以确认单为准。</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -8432,7 +8490,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>23:00左右才完全天黑，订22:00以后、最好22:30以后的场次。</t>
+          <t>23:00左右才完全天黑，订22:30以后的场次。</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -8440,8 +8498,16 @@
           <t>silver-river-official</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>晚上 A · 观星团</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>早睡；团要先订，另外收费。</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8450,51 +8516,63 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>23:00后</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Twizel</t>
+          <t>住处门口</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>早餐：镇上或住宿；午餐：High Country Salmon 刺身＋热食；晚餐：住处自己煎三文鱼</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr"/>
+          <t>不参加团就自己看：23:00 左右天完全黑，在住处门口抬头就能看到银河，不用开车。</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>自己看银河</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>晚上 B · 自己看</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>讲解和望远镜，也没人帮你认南半球的星座。</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>d8</t>
+          <t>d7</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Twizel → Omarama</t>
+          <t>Twizel</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Twizel出发，Omarama短休息。</t>
+          <t>早餐：镇上或住宿；午餐：High Country Salmon 刺身＋热食；晚餐：住处自己煎三文鱼</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -8510,34 +8588,26 @@
         </is>
       </c>
       <c r="B65" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>上午后段</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Lindis Pass Lookout</t>
+          <t>Twizel → Omarama</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Lindis Pass正规观景停车场停15–20分钟。</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>山口公路</t>
-        </is>
-      </c>
+          <t>Twizel出发，Omarama短休息。</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>lindis-pass-route,doc-lindis-official</t>
-        </is>
-      </c>
+      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr"/>
     </row>
@@ -8548,32 +8618,48 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>午后</t>
+          <t>上午 · 约 1–1.5 小时</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Tarras → Luggate → Wānaka</t>
+          <t>Omarama Clay Cliffs</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>经Tarras、Luggate到Wānaka，湖边午餐或咖啡。</t>
+          <t>Omarama 镇外看风蚀黏土尖塔：Quailburn Road 转 Henburn Road，约 3km 碎石路到私人农场大门，门口投币箱交进场费；停车后走 10–15 分钟到峡谷口，进去转转留 1 小时。</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>午后湖岸</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+          <t>黏土尖塔</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>带现金；过了大门的路坑洼、下雨会烂泥，路况不好就停在大门附近走进去，别硬开。手机信号弱。</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>clay-cliffs-official</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>可加 · Clay Cliffs</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>到 Wānaka 晚约 1 小时。</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8582,32 +8668,32 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16:00后</t>
+          <t>上午后段</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Hikuwai Haven 1</t>
+          <t>Lindis Pass Lookout</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>入住Hikuwai Haven 1，放下行李歇一会儿。</t>
+          <t>Lindis Pass正规观景停车场停15–20分钟。</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>入住两晚</t>
+          <t>山口公路</t>
         </is>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
         <is>
-          <t>hikuwai-map</t>
+          <t>lindis-pass-route,doc-lindis-official</t>
         </is>
       </c>
       <c r="I67" t="inlineStr"/>
@@ -8620,24 +8706,28 @@
         </is>
       </c>
       <c r="B68" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>午后</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Wānaka镇上</t>
+          <t>Tarras → Luggate → Wānaka</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>早点吃晚饭；长周末餐厅人多，早去好排队。</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr"/>
+          <t>经Tarras、Luggate到Wānaka，湖边午餐或咖啡。</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>午后湖岸</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
@@ -8650,36 +8740,32 @@
         </is>
       </c>
       <c r="B69" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>18:45–21:15（天气好再去）</t>
+          <t>16:00后</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Diamond Lake / Lake Wānaka Lookout</t>
+          <t>Hikuwai Haven 1</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>天气好、有精神才去：18:45出发，开约 20 分钟到 Diamond Lake 停车场，先到 Diamond Lake 湖边，再上 Lake Wānaka Lookout 俯瞰整个湖，往返约 2 小时，台阶多。只想轻松走就绕 Diamond Lake 一圈，约 45 分钟。累了就在 Wānaka 湖边散步看日落。</t>
+          <t>入住Hikuwai Haven 1，放下行李歇一会儿。</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>傍晚俯瞰 Wānaka 湖</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>去了的话，明早不再爬 Mount Iron；21:15前回到停车场。</t>
-        </is>
-      </c>
+          <t>入住两晚</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr">
         <is>
-          <t>diamond-lake-map,diamond-lake-official</t>
+          <t>hikuwai-map</t>
         </is>
       </c>
       <c r="I69" t="inlineStr"/>
@@ -8692,21 +8778,21 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>途中 / Wānaka</t>
+          <t>Wānaka镇上</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>早餐：Twizel；午餐：途中或Wānaka；晚餐：Wānaka镇上</t>
+          <t>早点吃晚饭；长周末餐厅人多，早去好排队。</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -8718,76 +8804,80 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>09:00–11:00</t>
+          <t>18:45–21:15</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Mount Iron / 湖边平路</t>
+          <t>Diamond Lake / Lake Wānaka Lookout</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>2/8 没去 Diamond Lake：爬 Mount Iron，按 1.5–2 小时准备，有上下坡。去过了：从镇上沿湖走到 Waterfall Creek，平路 60–90 分钟。</t>
+          <t>天气好、有精神才去：18:45出发，开约 20 分钟到 Diamond Lake 停车场，先到 Diamond Lake 湖边，再上 Lake Wānaka Lookout 俯瞰整个湖，往返约 2 小时，台阶多。只想轻松走就绕 Diamond Lake 一圈，约 45 分钟。不去就在 Wānaka 湖边散步看日落。</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>上午走走</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr"/>
+          <t>傍晚俯瞰 Wānaka 湖</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>20:00–20:30在观景台看斜阳照湖；21:15前回到停车场，趁天没黑开回住处。</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>mount-iron-official,mount-iron-route,wanaka-lakefront-route</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
+          <t>diamond-lake-map,diamond-lake-official</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>可加 · Diamond Lake</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>早点休息；去了的话 2/9 上午走湖边平路，不再爬 Mount Iron。</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>d9</t>
+          <t>d8</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>中午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Wānaka湖边</t>
+          <t>途中 / Wānaka</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>湖边吃午饭、散步，之后咖啡和休息。</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>湖边午餐</t>
-        </is>
-      </c>
+          <t>早餐：Twizel；午餐：途中或Wānaka；晚餐：Wānaka镇上</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>wanaka-lakefront-route</t>
-        </is>
-      </c>
+      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
     </row>
@@ -8798,36 +8888,44 @@
         </is>
       </c>
       <c r="B73" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>09:00–11:00</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>湖边 / Cinema Paradiso</t>
+          <t>Mount Iron</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>沿湖走走；喜欢电影时查看Cinema Paradiso实际片单。</t>
+          <t>爬 Mount Iron，按 1.5–2 小时准备，有上下坡，山顶看 Wānaka 镇和湖。2/8 没去 Diamond Lake 就选这个。</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>可选电影</t>
+          <t>山顶看湖</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr">
         <is>
-          <t>paradiso-official</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
+          <t>mount-iron-official,mount-iron-route</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>上午 A · Mount Iron</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>上午沿湖慢走的时间。</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8836,40 +8934,44 @@
         </is>
       </c>
       <c r="B74" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>下午（可选）</t>
+          <t>09:30–11:00</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Rippon品酒</t>
+          <t>Wānaka 湖边 → Waterfall Creek</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>可选：Rippon湖景酒庄品酒，约45–60分钟，需提前预约场次；驾驶者不饮酒。</t>
+          <t>从镇上沿湖走到 Waterfall Creek，平路 60–90 分钟。2/8 去过 Diamond Lake 就选这个，腿歇一歇。</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>补选项</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>订不到场次就跳过，不影响晚餐。</t>
-        </is>
-      </c>
+          <t>湖边平路</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>rippon-official,rippon-map</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+          <t>wanaka-lakefront-route</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>上午 B · 湖边平路</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Mount Iron 山顶俯瞰 Wānaka 的视角。</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8878,36 +8980,32 @@
         </is>
       </c>
       <c r="B75" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>18:00左右</t>
+          <t>中午</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Kika</t>
+          <t>Wānaka湖边</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Kika分享式晚餐，待预约。</t>
+          <t>湖边吃午饭、散步，之后咖啡和休息。</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>认真吃一顿</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>Kika待预约。</t>
-        </is>
-      </c>
+          <t>湖边午餐</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr">
         <is>
-          <t>kika-official,kika-route</t>
+          <t>wanaka-lakefront-route</t>
         </is>
       </c>
       <c r="I75" t="inlineStr"/>
@@ -8920,38 +9018,26 @@
         </is>
       </c>
       <c r="B76" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>20:15–21:10</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Roys Bay · That Wānaka Tree</t>
+          <t>Wānaka 湖边</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>饭后走约10分钟到Roys Bay湖岸，看That Wānaka Tree后面的日落；之后打车回住宿。</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>湖里那棵树的日落</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>只在岸边看，不攀爬、不下水靠近；拍照的人多。</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>wanaka-tree-map</t>
-        </is>
-      </c>
+          <t>沿湖走走、喝咖啡、休息。</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr"/>
     </row>
@@ -8962,104 +9048,132 @@
         </is>
       </c>
       <c r="B77" t="n">
-        <v>90</v>
+        <v>32</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>下午 · 约 2 小时</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>湖畔 / Kika</t>
+          <t>Cinema Paradiso</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>早餐：出发前；午餐：湖畔简餐；晚餐：Kika</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr"/>
+          <t>看一场电影，片单看当周场次。</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>老电影院</t>
+        </is>
+      </c>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>paradiso-official</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>可加 · 电影</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>下午两小时的湖边时间。</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>下午 · 45–60 分钟</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Wānaka → Cardrona → Crown Range</t>
+          <t>Rippon品酒</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>退房出发，沿Cardrona Valley Road经Cardrona小镇翻Crown Range；山顶观景点短停。</t>
+          <t>Rippon湖景酒庄品酒，需提前预约场次；开车的人不喝。</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>最长转场日</t>
+          <t>湖景酒庄</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>下山一侧连续急弯，低速档慢下。</t>
+          <t>订不到场次就跳过，不影响晚餐。</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>crown-range-route</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
+          <t>rippon-official,rippon-map</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>可加 · Rippon 品酒</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>45–60 分钟的湖边时间；要先订。</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>上午后段至中午</t>
+          <t>18:00左右</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Arrowtown</t>
+          <t>Kika</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Arrowtown老街散步、午餐或咖啡，约60–90分钟；之后到Frankton加油。</t>
+          <t>Kika分享式晚餐，待预约。</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>淘金小镇午餐</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr"/>
+          <t>认真吃一顿</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Kika待预约。</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>arrowtown-map</t>
+          <t>kika-official,kika-route</t>
         </is>
       </c>
       <c r="I79" t="inlineStr"/>
@@ -9068,36 +9182,40 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>中午至下午</t>
+          <t>20:15–21:10</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Kingston → Five Rivers → Mossburn</t>
+          <t>Roys Bay · That Wānaka Tree</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>经Kingston、Five Rivers、Mossburn到Te Anau；Kingston湖边短停，分段休息。</t>
+          <t>饭后走约10分钟到Roys Bay湖岸，看That Wānaka Tree后面的日落；之后打车回住宿。</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>分段休息</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
+          <t>湖里那棵树的日落</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>只在岸边看，不攀爬、不下水靠近；拍照的人多。</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>nav07-leg2-route</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="I80" t="inlineStr"/>
@@ -9106,38 +9224,30 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>d10</t>
+          <t>d9</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15:00–16:30左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>湖畔 / Kika</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>入住，购买翌日路餐、看一眼明早RealNZ的集合点。</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>为Milford准备</t>
-        </is>
-      </c>
+          <t>早餐：出发前；午餐：湖畔简餐；晚餐：Kika</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>te-anau-ensuite-map,realnz-map</t>
-        </is>
-      </c>
+      <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
     </row>
@@ -9148,28 +9258,48 @@
         </is>
       </c>
       <c r="B82" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Te Anau镇上</t>
+          <t>Wānaka → Cardrona → Crown Range</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>早点吃晚饭。</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
+          <t>退房出发，沿Cardrona Valley Road经Cardrona小镇翻Crown Range；山顶观景点短停，下山到 Arrow Junction。</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>最长转场日</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>下山一侧连续急弯，低速档慢下。</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>crown-range-route</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>路线 A · 翻 Crown Range</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>风景上不错过什么，但下山急弯多，开车更累。</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9178,40 +9308,44 @@
         </is>
       </c>
       <c r="B83" t="n">
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>20:40–21:15</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Wānaka → Cromwell → Kawarau 峡谷</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>沿Lakefront Drive散步，湖岸朝西，看21:09的日落落在湖上；离住处几分钟，看完回去早点睡。</t>
+          <t>起雾、大风或下雨就走这条：经 Cromwell 和 Kawarau 峡谷到 Arrow Junction，多约 50 公里、20–30 分钟，照样去 Arrowtown。</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>湖上日落</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>明早09:15去Milford报到。</t>
-        </is>
-      </c>
+          <t>坏天气改道</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
+          <t>nav07-leg1-route</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>路线 B · 经 Cromwell</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Crown Range 山顶观景和 Cardrona 小镇。</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9220,96 +9354,120 @@
         </is>
       </c>
       <c r="B84" t="n">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>上午 · 约 15 分钟</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Frankton / Kingston / Te Anau</t>
+          <t>Kawarau Bridge 蹦极点</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：17:30在Te Anau镇上</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
+          <t>老吊桥上看人蹦极，免费停车、免费看，有咖啡和洗手间。走 A 线从 Arrow Junction 往东多开约 5 分钟；走 B 线会直接路过。</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>看蹦极</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>营业约 9:30–16:00，以当天为准。</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>kawarau-bungy-official</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>可加 · 看蹦极</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>到 Te Anau 晚 20–30 分钟。</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>08:00左右</t>
+          <t>上午后段至中午</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Arrowtown</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+          <t>Arrowtown老街散步、午餐或咖啡，约60–90分钟；之后到Frankton加油。</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>装备检查</t>
+          <t>淘金小镇午餐</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>arrowtown-map</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>09:15左右到，09:30前完成报到</t>
+          <t>中午至下午</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre</t>
+          <t>Kingston → Five Rivers → Mossburn</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
+          <t>经Kingston、Five Rivers、Mossburn到Te Anau；Kingston湖边短停，分段休息。</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>已订集合</t>
+          <t>分段休息</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr">
         <is>
-          <t>realnz-map,realnz-walk-route</t>
+          <t>nav07-leg2-route</t>
         </is>
       </c>
       <c r="I86" t="inlineStr"/>
@@ -9318,36 +9476,36 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>09:50–17:00</t>
+          <t>15:00–16:30左右</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Milford Sound</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
+          <t>入住，购买翌日路餐、看一眼明早RealNZ的集合点。</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>峡湾</t>
+          <t>为Milford准备</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
       <c r="H87" t="inlineStr">
         <is>
-          <t>realnz-booking</t>
+          <t>te-anau-ensuite-map,realnz-map</t>
         </is>
       </c>
       <c r="I87" t="inlineStr"/>
@@ -9356,49 +9514,45 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Te Anau镇上</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+          <t>早点吃晚饭。</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>redcliff-official</t>
-        </is>
-      </c>
+      <c r="H88" t="inlineStr"/>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>20:45–21:15</t>
+          <t>20:40–21:15</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -9408,15 +9562,19 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
+          <t>沿Lakefront Drive散步，湖岸朝西，看21:09的日落落在湖上；离住处几分钟，看完回去早点睡。</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>饭后散步</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr"/>
+          <t>湖上日落</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>明早09:15去Milford报到。</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr">
         <is>
           <t>realnz-walk-route</t>
@@ -9428,7 +9586,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>d11</t>
+          <t>d10</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -9441,12 +9599,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>Frankton / Kingston / Te Anau</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
+          <t>早餐：Wānaka；午餐：Arrowtown；晚餐：17:30在Te Anau镇上</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -9458,7 +9616,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -9466,33 +9624,33 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>08:00左右</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr"/>
+          <t>早餐，带好防水外套、保暖层、防滑鞋、路餐和饮水。</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>装备检查</t>
+        </is>
+      </c>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>nav08-route</t>
-        </is>
-      </c>
+      <c r="H91" t="inlineStr"/>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -9500,28 +9658,28 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>12:00–13:00</t>
+          <t>09:15左右到，09:30前完成报到</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Frankton</t>
+          <t>RealNZ Visitor Centre</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+          <t>RealNZ Visitor Centre前台，85 Lakefront Drive, Te Anau。</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>午餐</t>
+          <t>已订集合</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
       <c r="H92" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>realnz-map,realnz-walk-route</t>
         </is>
       </c>
       <c r="I92" t="inlineStr"/>
@@ -9530,7 +9688,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -9538,32 +9696,28 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>13:15–14:30（晚了就跳过）</t>
+          <t>09:50–17:00</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Kelvin Peninsula Sculpture Trail</t>
+          <t>Milford Sound</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+          <t>已订蒂阿瑙往返大巴＋Milford特色游船，2成人。以运营商安排的沿途停靠为准。</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>湖畔雕塑步道</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>午饭晚了或累了就跳过，直接去Fernhill，优先保证16:30的缆车；起点在Peninsula Road和Grove Lane路口。</t>
-        </is>
-      </c>
+          <t>峡湾</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr">
         <is>
-          <t>kelvin-trail-map,kelvin-trail-official</t>
+          <t>realnz-booking</t>
         </is>
       </c>
       <c r="I93" t="inlineStr"/>
@@ -9572,36 +9726,32 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15:00–15:45</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，15:00入住，放下行李；车留在住处，15:50出发去缆车站。</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>入住Fernhill</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
         <is>
-          <t>fernhill-map</t>
+          <t>redcliff-official</t>
         </is>
       </c>
       <c r="I94" t="inlineStr"/>
@@ -9610,40 +9760,36 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>16:30–18:30</t>
+          <t>20:45–21:15</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Skyline Gondola + Luge · Bob’s Peak</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
+          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>缆车＋Luge</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
-        </is>
-      </c>
+          <t>饭后散步</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>skyline-booking,skyline-map,skyline-official</t>
+          <t>realnz-walk-route</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -9652,38 +9798,30 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>19:00–20:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Blue Kanu</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>晚餐</t>
-        </is>
-      </c>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>blue-kanu-official</t>
-        </is>
-      </c>
+      <c r="H96" t="inlineStr"/>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
     </row>
@@ -9694,32 +9832,28 @@
         </is>
       </c>
       <c r="B97" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>20:40–21:10</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Earnslaw Park / 湖边</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>湖边日落</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
       <c r="H97" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="I97" t="inlineStr"/>
@@ -9732,62 +9866,74 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Frankton / Blue Kanu</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>午餐</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>frankton-map</t>
+        </is>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>13:15–14:30（晚了就跳过）</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>湖边公路</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr"/>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>午饭晚了或累了就跳过，直接去Fernhill，优先保证16:30的缆车；起点在Peninsula Road和Grove Lane路口。</t>
+        </is>
+      </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -9796,36 +9942,36 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>15:00–15:45</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+          <t>开约20分钟到Fernhill，15:00入住，放下行李；车留在住处，15:50出发去缆车站。</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>红船屋</t>
+          <t>入住Fernhill</t>
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
       <c r="H100" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>fernhill-map</t>
         </is>
       </c>
       <c r="I100" t="inlineStr"/>
@@ -9834,40 +9980,40 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>16:30–18:30</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Skyline Gondola + Luge · Bob’s Peak</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>湿地步道</t>
+          <t>缆车＋Luge</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
+          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>skyline-booking,skyline-map,skyline-official</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -9876,32 +10022,36 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>19:00–20:30</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Blue Kanu</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr"/>
+          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>晚餐</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr"/>
       <c r="H102" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -9910,40 +10060,36 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>18:00–19:30（可选）</t>
+          <t>20:40–21:10</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Earnslaw Park / 湖边</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>有精神才去：从Glenorchy路岔进Moke Lake Road，约30分钟到湖边，在营地一侧湖边停30–45分钟看倒影，傍晚无风时最好。还想走再绕湖一圈（约6km、2–2.5小时，20:30前回到车上）。</t>
+          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>傍晚湖面倒影</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>累了或下雨就不去；21:00日落前回到铺装路。</t>
-        </is>
-      </c>
+          <t>湖边日落</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>moke-lake-map,moke-lake-official</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -9952,38 +10098,30 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B104" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>20:00–21:00</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>回市中心吃Fergburger。可以先打电话点单，到店直接付款取餐，不用排外面的长队；隔壁Fergbaker的派也可以带一个。之后整理行李，准备次日加油还车。</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>皇后镇招牌汉堡</t>
-        </is>
-      </c>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
-        </is>
-      </c>
+      <c r="H104" t="inlineStr"/>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
     </row>
@@ -9994,62 +10132,70 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Glenorchy / Fergburger</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr"/>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>湖边公路</t>
+        </is>
+      </c>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>nav09-out-route</t>
+        </is>
+      </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>南岛收车</t>
+          <t>红船屋</t>
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>bennetts-bluff-official</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -10058,36 +10204,40 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>等飞机</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr"/>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>zqn-map</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -10096,70 +10246,74 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>航班</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>nav09-back-route</t>
+        </is>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>18:00–19:30（可选）</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>取行李，打车或 Uber 进城（约 40–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>有精神才去：从Glenorchy路岔进Moke Lake Road，约30分钟到湖边，在营地一侧湖边停30–45分钟看倒影，傍晚无风时最好。还想走再绕湖一圈（约6km、2–2.5小时，20:30前回到车上）。</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>连住两晚</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr"/>
+          <t>傍晚湖面倒影</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>累了或下雨就不去；21:00日落前回到铺装路。</t>
+        </is>
+      </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>moke-lake-map,moke-lake-official</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -10168,36 +10322,36 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>18:00–19:30</t>
+          <t>20:00–21:00</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
+          <t>回市中心吃Fergburger。可以先打电话点单，到店直接付款取餐，不用排外面的长队；隔壁Fergbaker的派也可以带一个。之后整理行李，准备次日加油还车。</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>情人节晚餐</t>
+          <t>皇后镇招牌汉堡</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
       <c r="H110" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
         </is>
       </c>
       <c r="I110" t="inlineStr"/>
@@ -10206,42 +10360,30 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B111" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>19:30–20:30（可选）</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Viaduct Harbour / Wynyard Quarter</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>饭后在Viaduct海边走走就回酒店早睡；有精神再走10分钟到Wynyard Quarter / Silo Park，看20:19的日落。</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>海边散步</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>明早06:00出发，早点睡。</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
-        <is>
-          <t>wynyard-map</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
     </row>
@@ -10252,62 +10394,70 @@
         </is>
       </c>
       <c r="B112" t="n">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr"/>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>南岛收车</t>
+        </is>
+      </c>
       <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Auckland出发</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>早起出发</t>
+          <t>等飞机</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
       <c r="H113" t="inlineStr">
         <is>
-          <t>waitomo-hobbiton-booking</t>
+          <t>zqn-map</t>
         </is>
       </c>
       <c r="I113" t="inlineStr"/>
@@ -10316,78 +10466,70 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B114" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Waitomo Glowworm Caves</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
+          <t>飞奥克兰。</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>萤火虫洞</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>洞里凉、不能拍照；讲解是英文。</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
-        <is>
-          <t>waitomo-map</t>
-        </is>
-      </c>
+          <t>航班</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B115" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>中午–下午</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
+          <t>取行李，打车或 Uber 进城（约 40–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>霍比屯</t>
+          <t>连住两晚</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>shire-rest-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -10396,71 +10538,87 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B116" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>约17:30</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>回到Auckland</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>回到市区，回酒店歇一会儿。</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr"/>
+          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>情人节晚餐</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>viaduct-map</t>
+        </is>
+      </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B117" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:30–20:30（可选）</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Auckland市中心</t>
+          <t>Viaduct Harbour / Wynyard Quarter</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>酒店附近吃晚饭，之后回酒店休息，不再出门。</t>
+          <t>饭后在Viaduct海边走走就回酒店早睡；有精神再走10分钟到Wynyard Quarter / Silo Park，看20:19的日落。</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>休息</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
+          <t>海边散步</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>明早06:00出发，早点睡。</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>wynyard-map</t>
+        </is>
+      </c>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -10473,12 +10631,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>车上 / 途中 / Auckland</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
         </is>
       </c>
       <c r="F118" t="inlineStr"/>
@@ -10490,7 +10648,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -10498,29 +10656,37 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>Auckland出发</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>退房并寄存行李。</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr"/>
+          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>早起出发</t>
+        </is>
+      </c>
       <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>waitomo-hobbiton-booking</t>
+        </is>
+      </c>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -10528,28 +10694,32 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
+          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>美术馆</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr"/>
+          <t>萤火虫洞</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>洞里凉、不能拍照；讲解是英文。</t>
+        </is>
+      </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>art-gallery-map,art-gallery-official</t>
+          <t>waitomo-map</t>
         </is>
       </c>
       <c r="I120" t="inlineStr"/>
@@ -10558,7 +10728,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -10566,28 +10736,28 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>中午–下午</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
+          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>完整午餐</t>
+          <t>霍比屯</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>amano-map,amano-official</t>
+          <t>shire-rest-map</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -10596,7 +10766,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -10604,17 +10774,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>约17:30</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>回到Auckland</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+          <t>回到市区，回酒店歇一会儿。</t>
         </is>
       </c>
       <c r="F122" t="inlineStr"/>
@@ -10626,7 +10796,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -10634,37 +10804,33 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>Auckland市中心</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+          <t>酒店附近吃晚饭，之后回酒店休息，不再出门。</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>夜航回国</t>
+          <t>休息</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr">
-        <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
+      <c r="H123" t="inlineStr"/>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -10677,12 +10843,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>车上 / 途中 / Auckland</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -10694,7 +10860,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -10702,24 +10868,20 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>转机</t>
-        </is>
-      </c>
+          <t>退房并寄存行李。</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
@@ -10728,7 +10890,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -10736,28 +10898,28 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>09:10–11:10</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>CZ3803 → 杭州萧山T4</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>飞回杭州，取行李回家。</t>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>到家</t>
+          <t>美术馆</t>
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
       <c r="H126" t="inlineStr">
         <is>
-          <t>hgh-airport-map</t>
+          <t>art-gallery-map,art-gallery-official</t>
         </is>
       </c>
       <c r="I126" t="inlineStr"/>
@@ -10766,36 +10928,244 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B127" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>落地后</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
+          <t>Britomart午餐，首选Amano，待预约。</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>按航班实际到达时间</t>
+          <t>完整午餐</t>
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>amano-map,amano-official</t>
+        </is>
+      </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>40</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>下午</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Britomart</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>50</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>晚上</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Auckland Airport</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>夜航回国</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>akl-intl-map,akl-departure-official</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>90</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>市区 / Amano</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>10</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>05:00–09:10</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>广州白云T2</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>转机</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>20</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>09:10–11:10</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>CZ3803 → 杭州萧山T4</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>90</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>落地后</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>按航班实际到达时间</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
content: D11–D16 forks, add-ons and rain fallback; one update note for all options
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/nz2027-itinerary.xlsx
+++ b/content/nz2027-itinerary.xlsx
@@ -584,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G119"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3503,12 +3503,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>mt-john-official</t>
+          <t>teanau-bird-sanctuary-official</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Mount John · Astro Café（Dark Sky Project）</t>
+          <t>Punanga Manu o Te Anau 鸟类保护区</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3518,84 +3518,84 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://www.darkskyproject.co.nz/eat/astro-cafe/</t>
+          <t>https://www.fiordland.org.nz/see-and-do/activities/show/punanga-manu-o-te-anau-bird-sanctuary/</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Dark Sky Project</t>
+          <t>Fiordland NZ</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>margaret-official</t>
+          <t>kepler-dock-bay-official</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Margaret（Neil Perry）</t>
+          <t>DOC：游客中心到 Kepler Track 停车场</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://themargaretfamily.com/venue/margaret/</t>
+          <t>https://doc.govt.nz/parks-and-recreation/places-to-go/fiordland/places/fiordland-national-park/things-to-do/tracks/visitor-centre-to-kepler-track-carpark-walk</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>待预约</t>
+          <t>DOC</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>margaret-map</t>
+          <t>bobs-cove-official</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Margaret, 30–36 Bay Street, Double Bay</t>
+          <t>Bob's Cove Track &amp; Nature Walk</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Margaret%2C+30+Bay+Street%2C+Double+Bay+NSW+2028%2C+Australia</t>
+          <t>https://www.queenstownnz.co.nz/listing/bobs-cove-track-%26-nature-walk/9103/</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Queenstown NZ</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>mt-eden-map</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Earnslaw Park</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Maungawhau+Mount+Eden+Summit%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -3619,12 +3619,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>waitomo-map</t>
+          <t>devonport-ferry-map</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Waitomo Glowworm Caves</t>
+          <t>Downtown Ferry Terminal → Devonport</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Downtown+Ferry+Terminal%2C+Auckland%2C+New+Zealand&amp;destination=Devonport+Wharf%2C+Auckland%2C+New+Zealand&amp;travelmode=transit</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -3648,80 +3648,80 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>viaduct-map</t>
+          <t>mt-john-official</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>Mount John · Astro Café（Dark Sky Project）</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
+          <t>https://www.darkskyproject.co.nz/eat/astro-cafe/</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>Dark Sky Project</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>margaret-official</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Silo Park / Wynyard Quarter</t>
+          <t>Margaret（Neil Perry）</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
+          <t>https://themargaretfamily.com/venue/margaret/</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>待预约</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>fergburger-map</t>
+          <t>margaret-map</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Margaret, 30–36 Bay Street, Double Bay</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Margaret%2C+30+Bay+Street%2C+Double+Bay+NSW+2028%2C+Australia</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -3735,70 +3735,70 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>fergburger-official</t>
+          <t>earnslaw-park-map</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Fergburger官网</t>
+          <t>Earnslaw Park</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>restaurant</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>https://www.fergburger.com/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Earnslaw+Park%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>skyline-booking</t>
+          <t>waitomo-map</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>booking</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Waitomo+Glowworm+Caves%2C+Waitomo%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
-          <t>两人 ¥644</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>skyline-map</t>
+          <t>viaduct-map</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Skyline Gondola Queenstown</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Viaduct+Harbour%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E112" t="inlineStr"/>
@@ -3822,51 +3822,51 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>skyline-official</t>
+          <t>wynyard-map</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Skyline Queenstown官网</t>
+          <t>Silo Park / Wynyard Quarter</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>official</t>
+          <t>map</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>https://www.skyline.co.nz/en/queenstown/</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Silo+Park%2C+Wynyard+Quarter%2C+Auckland%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
-          <t>官网</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>wanaka-tree-map</t>
+          <t>fergburger-map</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>That Wānaka Tree</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Fergburger%2C+Shotover+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E114" t="inlineStr"/>
@@ -3880,70 +3880,70 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>rippon-map</t>
+          <t>fergburger-official</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Rippon酒庄</t>
+          <t>Fergburger官网</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>restaurant</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+          <t>https://www.fergburger.com/</t>
         </is>
       </c>
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Google Maps</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>nav08-route</t>
+          <t>skyline-booking</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>完整路线到Fernhill</t>
+          <t>Skyline缆车＋Luge 3圈（已订，2/12 16:30–18:30）</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>booking</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
-          <t>导航08</t>
+          <t>两人 ¥644</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>nav09-out-route</t>
+          <t>skyline-map</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>去程经Bennetts Bluff</t>
+          <t>Skyline Gondola Queenstown</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3953,55 +3953,55 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Skyline+Queenstown%2C+Brecon+Street%2C+Queenstown%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>Google Maps</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>skyline-official</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Glenorchy回住宿</t>
+          <t>Skyline Queenstown官网</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>map</t>
+          <t>official</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.skyline.co.nz/en/queenstown/</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
-          <t>导航09</t>
+          <t>官网</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>wanaka-tree-map</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>机场方向参考路线</t>
+          <t>That Wānaka Tree</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -4011,12 +4011,157 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=That+Wanaka+Tree%2C+Wanaka%2C+New+Zealand</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>rippon-map</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Rippon酒庄</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=Rippon+Vineyard%2C+Wanaka%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Google Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>nav08-route</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>完整路线到Fernhill</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=3+Thomson+Place%2C+Te+Anau%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Mossburn%2C+New+Zealand%7CFive+Rivers%2C+Southland%2C+New+Zealand%7CKingston%2C+Otago%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>导航08</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>nav09-out-route</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>去程经Bennetts Bluff</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;travelmode=driving&amp;waypoints=Bennetts+Bluff+Viewpoint%2C+Queenstown-Glenorchy+Road%2C+New+Zealand</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>nav09-back-route</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Glenorchy回住宿</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=Glenorchy+Wharf%2C+Glenorchy%2C+New+Zealand&amp;destination=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>导航09</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>机场方向参考路线</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/dir/?api=1&amp;origin=15+Greenstone+Place%2C+Fernhill%2C+Queenstown%2C+New+Zealand&amp;destination=Queenstown+Airport%2C+New+Zealand&amp;travelmode=driving</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
         <is>
           <t>导航10</t>
         </is>
@@ -5448,7 +5593,7 @@
       <c r="W12" t="inlineStr">
         <is>
           <t>住宿｜Private Ensuite，第二晚。
-天气｜暴雨、落石时Milford Road（SH94）会临时封路，RealNZ可能取消或改期。前一晚和当天早上看RealNZ通知；若取消，当天改为Te Anau湖边步道和休息，不临时补订其他项目。
+天气｜暴雨、落石时Milford Road（SH94）会临时封路，RealNZ可能取消或改期。前一晚和当天早上看RealNZ通知；若取消，按时间线里的“雨天备选”在 Te Anau 走走，不临时补订其他项目。
 沙蝇｜Milford码头和Te Anau湖边沙蝇多，叮咬会痒好几天；下车前喷驱蚊液，长袖长裤更稳。
 集合｜按约15–20分钟步行窗口留量，09:15到前台；有行李或下雨时打车提前到。订单没有写含午餐。</t>
         </is>
@@ -6096,7 +6241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J133"/>
+  <dimension ref="A1:J137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9730,32 +9875,48 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>18:30左右</t>
+          <t>Milford 取消时</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Te Anau</t>
+          <t>Te Anau 湖边 · 鸟类保护区 · Kepler 湖边段</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>回镇上吃晚餐，可预约The Redcliff。</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
+          <t>沿湖往南走到 Punanga Manu o Te Anau 鸟类保护区（日出到日落开放，免费，欢迎捐款），再到 Kepler Track 停车场，走一段湖边林间步道到 Dock Bay，往返约 1 小时。</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>雨天备选</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>DOC 讲解团每天 10:30，每人约 NZ$10，在 DOC 游客中心买票，以当天为准。</t>
+        </is>
+      </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>redcliff-official</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
+          <t>teanau-bird-sanctuary-official,kepler-dock-bay-official</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>雨天备选</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Milford 峡湾和整条 Milford Road。</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -9764,32 +9925,28 @@
         </is>
       </c>
       <c r="B95" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>20:45–21:15</t>
+          <t>18:30左右</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Te Anau Lakefront</t>
+          <t>Te Anau</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>饭后散步</t>
-        </is>
-      </c>
+          <t>回镇上吃晚餐，可预约The Redcliff。</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr"/>
       <c r="H95" t="inlineStr">
         <is>
-          <t>realnz-walk-route</t>
+          <t>redcliff-official</t>
         </is>
       </c>
       <c r="I95" t="inlineStr"/>
@@ -9802,60 +9959,64 @@
         </is>
       </c>
       <c r="B96" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>20:45–21:15</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>路餐 / The Redcliff</t>
+          <t>Te Anau Lakefront</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr"/>
+          <t>饭后沿湖边走走，看湖上日落，然后回住宿。</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>饭后散步</t>
+        </is>
+      </c>
       <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>realnz-walk-route</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>d12</t>
+          <t>d11</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>09:30左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Te Anau → Kingston</t>
+          <t>路餐 / The Redcliff</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Te Anau退房出发；最迟10:00前退房。</t>
+          <t>早餐：住宿/镇上；午餐：自备路餐，船上饮品小吃可刷卡购买；晚餐：The Redcliff</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr">
-        <is>
-          <t>nav08-route</t>
-        </is>
-      </c>
+      <c r="H97" t="inlineStr"/>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
     </row>
@@ -9866,32 +10027,28 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>12:00–13:00</t>
+          <t>09:30左右</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Frankton</t>
+          <t>Te Anau → Kingston</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>午餐</t>
-        </is>
-      </c>
+          <t>Te Anau退房出发；最迟10:00前退房。</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr">
         <is>
-          <t>frankton-map</t>
+          <t>nav08-route</t>
         </is>
       </c>
       <c r="I98" t="inlineStr"/>
@@ -9904,36 +10061,32 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>13:15–14:30（晚了就跳过）</t>
+          <t>12:00–13:00</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Kelvin Peninsula Sculpture Trail</t>
+          <t>Frankton</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
+          <t>经Kingston到皇后镇附近，在Frankton一带吃午饭，不进市中心。</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>湖畔雕塑步道</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>午饭晚了或累了就跳过，直接去Fernhill，优先保证16:30的缆车；起点在Peninsula Road和Grove Lane路口。</t>
-        </is>
-      </c>
+          <t>午餐</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr">
         <is>
-          <t>kelvin-trail-map,kelvin-trail-official</t>
+          <t>frankton-map</t>
         </is>
       </c>
       <c r="I99" t="inlineStr"/>
@@ -9946,36 +10099,48 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>15:00–15:45</t>
+          <t>13:15–14:30</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>15 Greenstone Place</t>
+          <t>Kelvin Peninsula Sculpture Trail</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>开约20分钟到Fernhill，15:00入住，放下行李；车留在住处，15:50出发去缆车站。</t>
+          <t>Kelvin Heights湖畔雕塑环线，绕高尔夫球场约3.5km、1小时，平路好走，对岸是Walter Peak和皇后镇。</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>入住Fernhill</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr"/>
+          <t>湖畔雕塑步道</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>起点在Peninsula Road和Grove Lane路口；午饭晚了就跳过，直接去 Fernhill。</t>
+        </is>
+      </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>fernhill-map</t>
-        </is>
-      </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
+          <t>kelvin-trail-map,kelvin-trail-official</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>可加 · Kelvin 半岛</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>午饭后歇一会儿的时间；14:30 前要走完，才赶得上 16:30 的缆车。</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -9984,36 +10149,32 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16:30–18:30</t>
+          <t>15:00–15:45</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Skyline Gondola + Luge · Bob’s Peak</t>
+          <t>15 Greenstone Place</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
+          <t>开约20分钟到Fernhill，15:00入住，放下行李；车留在住处，15:50出发去缆车站。</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>缆车＋Luge</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
-        </is>
-      </c>
+          <t>入住Fernhill</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr"/>
       <c r="H101" t="inlineStr">
         <is>
-          <t>skyline-booking,skyline-map,skyline-official</t>
+          <t>fernhill-map</t>
         </is>
       </c>
       <c r="I101" t="inlineStr"/>
@@ -10026,32 +10187,36 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>19:00–20:30</t>
+          <t>16:30–18:30</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Blue Kanu</t>
+          <t>Skyline Gondola + Luge · Bob’s Peak</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
+          <t>已订：Skyline缆车＋Luge滑道3圈，两人。坐缆车上Bob’s Peak看湖和Remarkables山脉，再滑3圈Luge。16:15前到Brecon Street缆车站：从Fernhill打车约5分钟，或步行下坡约20分钟。</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>晚餐</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr"/>
+          <t>缆车＋Luge</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>大风时可能停运，按Skyline通知改期；下山后走约10分钟到Blue Kanu。</t>
+        </is>
+      </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>blue-kanu-official</t>
+          <t>skyline-booking,skyline-map,skyline-official</t>
         </is>
       </c>
       <c r="I102" t="inlineStr"/>
@@ -10064,32 +10229,32 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>20:40–21:10</t>
+          <t>19:00–20:30</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Earnslaw Park / 湖边</t>
+          <t>Blue Kanu</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+          <t>下山走到Blue Kanu吃晚饭。缆车停运就先去Queenstown Gardens湖边轻走。</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>湖边日落</t>
+          <t>晚餐</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
       <c r="H103" t="inlineStr">
         <is>
-          <t>earnslaw-park-map</t>
+          <t>blue-kanu-official</t>
         </is>
       </c>
       <c r="I103" t="inlineStr"/>
@@ -10102,64 +10267,64 @@
         </is>
       </c>
       <c r="B104" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>20:40–21:10</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Frankton / Blue Kanu</t>
+          <t>Earnslaw Park / 湖边</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr"/>
+          <t>饭后走几分钟到Earnslaw Park一带湖边，看Wakatipu湖上的日落；之后打车回Fernhill。</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>湖边日落</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>earnslaw-park-map</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>d13</t>
+          <t>d12</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>09:00左右</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Fernhill → Glenorchy Road</t>
+          <t>Frankton / Blue Kanu</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>湖边公路</t>
-        </is>
-      </c>
+          <t>早餐：Te Anau；午餐：Frankton；晚餐：Blue Kanu</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr">
-        <is>
-          <t>nav09-out-route</t>
-        </is>
-      </c>
+      <c r="H105" t="inlineStr"/>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
     </row>
@@ -10170,32 +10335,32 @@
         </is>
       </c>
       <c r="B106" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>09:00左右</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Bennetts Bluff / Glenorchy码头</t>
+          <t>Fernhill → Glenorchy Road</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
+          <t>Fernhill出发，沿Queenstown–Glenorchy Road向西。</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>红船屋</t>
+          <t>湖边公路</t>
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
       <c r="H106" t="inlineStr">
         <is>
-          <t>bennetts-bluff-official</t>
+          <t>nav09-out-route</t>
         </is>
       </c>
       <c r="I106" t="inlineStr"/>
@@ -10208,36 +10373,32 @@
         </is>
       </c>
       <c r="B107" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>中午前后</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway</t>
+          <t>Bennetts Bluff / Glenorchy码头</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+          <t>Bennetts Bluff正规停车场停靠；到Glenorchy后看码头和红船屋。</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>湿地步道</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>官方路线3.2km，雨后注意积水提示。</t>
-        </is>
-      </c>
+          <t>红船屋</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
       <c r="H107" t="inlineStr">
         <is>
-          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
+          <t>bennetts-bluff-official</t>
         </is>
       </c>
       <c r="I107" t="inlineStr"/>
@@ -10250,28 +10411,36 @@
         </is>
       </c>
       <c r="B108" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>中午前后</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Glenorchy → Queenstown</t>
+          <t>Glenorchy Lagoon Walkway</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
+          <t>Glenorchy Lagoon Walkway，按1–2小时走；随后小镇午餐。</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>湿地步道</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>官方路线3.2km，雨后注意积水提示。</t>
+        </is>
+      </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>nav09-back-route</t>
+          <t>glenorchy-lagoon-official,glenorchy-lagoon-map</t>
         </is>
       </c>
       <c r="I108" t="inlineStr"/>
@@ -10284,36 +10453,28 @@
         </is>
       </c>
       <c r="B109" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>18:00–19:30（可选）</t>
+          <t>下午</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Moke Lake</t>
+          <t>Glenorchy → Queenstown</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>有精神才去：从Glenorchy路岔进Moke Lake Road，约30分钟到湖边，在营地一侧湖边停30–45分钟看倒影，傍晚无风时最好。还想走再绕湖一圈（约6km、2–2.5小时，20:30前回到车上）。</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>傍晚湖面倒影</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>累了或下雨就不去；21:00日落前回到铺装路。</t>
-        </is>
-      </c>
+          <t>沿原路返回，选择一个合适的正规观景点短停。16:00–17:00左右回Queenstown。</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
       <c r="H109" t="inlineStr">
         <is>
-          <t>moke-lake-map,moke-lake-official</t>
+          <t>nav09-back-route</t>
         </is>
       </c>
       <c r="I109" t="inlineStr"/>
@@ -10326,36 +10487,48 @@
         </is>
       </c>
       <c r="B110" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>20:00–21:00</t>
+          <t>下午 · 约 30 分钟–1.5 小时</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Fergburger</t>
+          <t>Bob's Cove</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>回市中心吃Fergburger。可以先打电话点单，到店直接付款取餐，不用排外面的长队；隔壁Fergbaker的派也可以带一个。之后整理行李，准备次日加油还车。</t>
+          <t>回程在 Glenorchy 路边的 Bob's Cove 停车场停下，林间小路走到碧绿色的湖湾，约 20 分钟单程；加走到 Picnic Point 的环线就留 1.5 小时。</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>皇后镇招牌汉堡</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr"/>
+          <t>碧绿湖湾</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>离皇后镇约 14km；夏天停车场很满，不要停路边或倒车上路。</t>
+        </is>
+      </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>fergburger-map,fergburger-official,boundary-street-map</t>
-        </is>
-      </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
+          <t>bobs-cove-official</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>可加 · Bob's Cove</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>回城晚半小时到一小时，傍晚的 Moke Lake 可能就不去了。</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10364,62 +10537,82 @@
         </is>
       </c>
       <c r="B111" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Glenorchy / Fergburger</t>
+          <t>Moke Lake</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
+          <t>有精神才去：从Glenorchy路岔进Moke Lake Road，约30分钟到湖边，在营地一侧湖边停30–45分钟看倒影，傍晚无风时最好。还想走再绕湖一圈（约6km、2–2.5小时，20:30前回到车上）。</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>傍晚湖面倒影</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>累了或下雨就不去；21:00日落前回到铺装路。</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>moke-lake-map,moke-lake-official</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>可加 · Moke Lake</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>早点休息；来回要开约 8km 碎石路。</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>09:15–10:00</t>
+          <t>20:00–21:00</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Fernhill → Frankton → Queenstown Airport</t>
+          <t>Fergburger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
+          <t>回市中心吃Fergburger。可以先打电话点单，到店直接付款取餐，不用排外面的长队；隔壁Fergbaker的派也可以带一个。之后整理行李，准备次日加油还车。</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>南岛收车</t>
+          <t>皇后镇招牌汉堡</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
       <c r="H112" t="inlineStr">
         <is>
-          <t>nav10-route</t>
+          <t>fergburger-map,fergburger-official,boundary-street-map</t>
         </is>
       </c>
       <c r="I112" t="inlineStr"/>
@@ -10428,38 +10621,30 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>d14</t>
+          <t>d13</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>10:00–13:30</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Queenstown Airport</t>
+          <t>Glenorchy / Fergburger</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>等飞机</t>
-        </is>
-      </c>
+          <t>早餐：Queenstown/住宿；午餐：Glenorchy镇上；晚餐：Fergburger</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr">
-        <is>
-          <t>zqn-map</t>
-        </is>
-      </c>
+      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr"/>
     </row>
@@ -10470,30 +10655,34 @@
         </is>
       </c>
       <c r="B114" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>13:30–15:20</t>
+          <t>09:15–10:00</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>JQ296 → Auckland</t>
+          <t>Fernhill → Frankton → Queenstown Airport</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>飞奥克兰。</t>
+          <t>退房出发，Frankton 加油，10:00 机场还车。</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>航班</t>
+          <t>南岛收车</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>nav10-route</t>
+        </is>
+      </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr"/>
     </row>
@@ -10504,32 +10693,32 @@
         </is>
       </c>
       <c r="B115" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>15:20后</t>
+          <t>10:00–13:30</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Auckland Airport → CBD</t>
+          <t>Queenstown Airport</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>取行李，打车或 Uber 进城（约 40–60 分钟），入住 2/14–16 连续两晚。</t>
+          <t>还车后时间宽裕：机场旁 Remarkables Park 吃早午饭，12:30 前回机场办托运。</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>连住两晚</t>
+          <t>等飞机</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
-          <t>akl-intl-map</t>
+          <t>zqn-map</t>
         </is>
       </c>
       <c r="I115" t="inlineStr"/>
@@ -10542,34 +10731,30 @@
         </is>
       </c>
       <c r="B116" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>18:00–19:30</t>
+          <t>13:30–15:20</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Viaduct Harbour</t>
+          <t>JQ296 → Auckland</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
+          <t>飞奥克兰。</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>情人节晚餐</t>
+          <t>航班</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>viaduct-map</t>
-        </is>
-      </c>
+      <c r="H116" t="inlineStr"/>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr"/>
     </row>
@@ -10580,36 +10765,32 @@
         </is>
       </c>
       <c r="B117" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>19:30–20:30（可选）</t>
+          <t>15:20后</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Viaduct Harbour / Wynyard Quarter</t>
+          <t>Auckland Airport → CBD</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>饭后在Viaduct海边走走就回酒店早睡；有精神再走10分钟到Wynyard Quarter / Silo Park，看20:19的日落。</t>
+          <t>取行李，打车或 Uber 进城（约 40–60 分钟），入住 2/14–16 连续两晚。</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>海边散步</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>明早06:00出发，早点睡。</t>
-        </is>
-      </c>
+          <t>连住两晚</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
       <c r="H117" t="inlineStr">
         <is>
-          <t>wynyard-map</t>
+          <t>akl-intl-map</t>
         </is>
       </c>
       <c r="I117" t="inlineStr"/>
@@ -10622,106 +10803,114 @@
         </is>
       </c>
       <c r="B118" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>18:00–19:30</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Queenstown / Auckland</t>
+          <t>Viaduct Harbour</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr"/>
+          <t>情人节晚饭，在Viaduct Harbour一带，要提前订。</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>情人节晚餐</t>
+        </is>
+      </c>
       <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>viaduct-map</t>
+        </is>
+      </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B119" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>19:30–20:30</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Auckland出发</t>
+          <t>Viaduct Harbour / Wynyard Quarter</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
+          <t>饭后在Viaduct海边走走；有精神再走10分钟到Wynyard Quarter / Silo Park，看20:19的日落。</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>早起出发</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr"/>
+          <t>海边日落</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>明早06:00出发，早点睡。</t>
+        </is>
+      </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>waitomo-hobbiton-booking</t>
-        </is>
-      </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
+          <t>wynyard-map</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>可加 · Wynyard 日落</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>早睡一小时，明早 06:00 就要出发。</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>d15</t>
+          <t>d14</t>
         </is>
       </c>
       <c r="B120" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>上午</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Waitomo Glowworm Caves</t>
+          <t>Queenstown / Auckland</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>萤火虫洞</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>洞里凉、不能拍照；讲解是英文。</t>
-        </is>
-      </c>
-      <c r="H120" t="inlineStr">
-        <is>
-          <t>waitomo-map</t>
-        </is>
-      </c>
+          <t>早餐：Fernhill；午餐：皇后镇机场附近；晚餐：Viaduct Harbour情人节晚餐</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
       <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr"/>
     </row>
@@ -10732,32 +10921,32 @@
         </is>
       </c>
       <c r="B121" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>中午–下午</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Hobbiton Movie Set</t>
+          <t>Auckland出发</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
+          <t>按确认单的时间和地点上车，早餐在车上吃。</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>霍比屯</t>
+          <t>早起出发</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
       <c r="H121" t="inlineStr">
         <is>
-          <t>shire-rest-map</t>
+          <t>waitomo-hobbiton-booking</t>
         </is>
       </c>
       <c r="I121" t="inlineStr"/>
@@ -10770,26 +10959,38 @@
         </is>
       </c>
       <c r="B122" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>约17:30</t>
+          <t>上午</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>回到Auckland</t>
+          <t>Waitomo Glowworm Caves</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>回到市区，回酒店歇一会儿。</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr"/>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
+          <t>萤火虫洞导览约1小时：先走溶洞，最后坐小船在黑暗里看满洞顶的萤火虫。</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>萤火虫洞</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>洞里凉、不能拍照；讲解是英文。</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>waitomo-map</t>
+        </is>
+      </c>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
     </row>
@@ -10800,30 +11001,34 @@
         </is>
       </c>
       <c r="B123" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>中午–下午</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Auckland市中心</t>
+          <t>Hobbiton Movie Set</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>酒店附近吃晚饭，之后回酒店休息，不再出门。</t>
+          <t>霍比屯片场导览：44个霍比特人洞、磨坊、双拱桥、派对树，在Green Dragon Inn喝一杯，Bag End门口拍照。</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>休息</t>
+          <t>霍比屯</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>shire-rest-map</t>
+        </is>
+      </c>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
     </row>
@@ -10834,21 +11039,21 @@
         </is>
       </c>
       <c r="B124" t="n">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>约17:30</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>车上 / 途中 / Auckland</t>
+          <t>回到Auckland</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
+          <t>回到市区，回酒店歇一会儿。</t>
         </is>
       </c>
       <c r="F124" t="inlineStr"/>
@@ -10860,28 +11065,32 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B125" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>早餐后</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>酒店</t>
+          <t>Auckland市中心</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>退房并寄存行李。</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr"/>
+          <t>酒店附近吃晚饭，之后回酒店休息，不再出门。</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>休息</t>
+        </is>
+      </c>
       <c r="G125" t="inlineStr"/>
       <c r="H125" t="inlineStr"/>
       <c r="I125" t="inlineStr"/>
@@ -10890,38 +11099,30 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>d16</t>
+          <t>d15</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>10:00–12:00</t>
+          <t>饮食</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery</t>
+          <t>车上 / 途中 / Auckland</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>美术馆</t>
-        </is>
-      </c>
+          <t>早餐：带上车；午餐：途中或Hobbiton（以确认单为准）；晚餐：Auckland市中心</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr">
-        <is>
-          <t>art-gallery-map,art-gallery-official</t>
-        </is>
-      </c>
+      <c r="H126" t="inlineStr"/>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr"/>
     </row>
@@ -10932,34 +11133,26 @@
         </is>
       </c>
       <c r="B127" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>12:30–14:00</t>
+          <t>早餐后</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Britomart · Amano</t>
+          <t>酒店</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Britomart午餐，首选Amano，待预约。</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>完整午餐</t>
-        </is>
-      </c>
+          <t>退房并寄存行李。</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>amano-map,amano-official</t>
-        </is>
-      </c>
+      <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr"/>
     </row>
@@ -10970,28 +11163,44 @@
         </is>
       </c>
       <c r="B128" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>下午</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Britomart</t>
+          <t>Auckland Art Gallery</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>GIAPO甜点或咖啡、短距离购物；按航班倒推结束城市活动。</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr"/>
+          <t>Auckland Art Gallery Toi o Tāmaki，按1.5–2小时安排。</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>美术馆</t>
+        </is>
+      </c>
       <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>art-gallery-map,art-gallery-official</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>上午 A · 美术馆</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Mt Eden 山顶看整座城。</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -11000,36 +11209,48 @@
         </is>
       </c>
       <c r="B129" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>晚上</t>
+          <t>10:00–12:00</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Auckland Airport</t>
+          <t>Mt Eden · Maungawhau</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
+          <t>打车约 15 分钟到山脚，走 15–20 分钟上山顶，看火山口和奥克兰全景，按 1.5 小时安排，再打车回 Britomart 吃午饭。</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>夜航回国</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr"/>
+          <t>火山口全景</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>山顶不能开车上去。</t>
+        </is>
+      </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>akl-intl-map,akl-departure-official</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
+          <t>mt-eden-map</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>上午 B · Mt Eden</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>美术馆。</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -11038,134 +11259,298 @@
         </is>
       </c>
       <c r="B130" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>12:30–14:00</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>市区 / Amano</t>
+          <t>Britomart · Amano</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr"/>
+          <t>Britomart午餐，首选Amano，待预约。</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>完整午餐</t>
+        </is>
+      </c>
       <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>amano-map,amano-official</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>05:00–09:10</t>
+          <t>14:00–17:30</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>广州白云T2</t>
+          <t>Britomart</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>转机</t>
-        </is>
-      </c>
+          <t>GIAPO甜点或咖啡、短距离购物，就在住处附近；17:30 前回酒店取行李。</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>下午 C · Britomart</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>从海上回看奥克兰天际线。</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B132" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>09:10–11:10</t>
+          <t>14:00–17:00</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>CZ3803 → 杭州萧山T4</t>
+          <t>Devonport</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>飞回杭州，取行李回家。</t>
+          <t>从 Downtown 码头坐渡轮约 12–15 分钟到 Devonport，走上 Mt Victoria（Takarunga）回看市中心和海港，镇上喝杯咖啡再坐船回来，约 2–3 小时。</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>到家</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr"/>
+          <t>渡轮和海港天际线</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>渡轮班次约每半小时，周末更少，以当天为准；刷 AT HOP 卡或银行卡感应支付。17:30 前回到酒店。</t>
+        </is>
+      </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>hgh-airport-map</t>
-        </is>
-      </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
+          <t>devonport-ferry-map</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>下午 D · Devonport 渡轮</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>逛街和慢慢吃甜点的时间。</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>d17</t>
+          <t>d16</t>
         </is>
       </c>
       <c r="B133" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>饮食</t>
+          <t>晚上</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>落地后</t>
+          <t>Auckland Airport</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
+          <t>取行李去机场，19:25 前到，办理 CZ306 值机和出境。</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>按航班实际到达时间</t>
+          <t>夜航回国</t>
         </is>
       </c>
       <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>akl-intl-map,akl-departure-official</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>d16</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>90</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>市区 / Amano</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>早餐：市区；午餐：Amano；晚餐：按起飞时刻在市区或机场安排</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>10</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>05:00–09:10</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>广州白云T2</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>入境、按国际转国内流程转机，候机时吃早餐。</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>转机</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>20</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>09:10–11:10</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>CZ3803 → 杭州萧山T4</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>飞回杭州，取行李回家。</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>到家</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>hgh-airport-map</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>d17</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>90</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>饮食</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>落地后</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>早餐：广州机场；午餐：回家简餐；晚餐：在家休息</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>按航班实际到达时间</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>